<commit_message>
Fix duplicate DUID rows in summary.csv
eli_per_duid.feather had duplicate MAPS2PV1 and MBPS2PV1 rows, inflating
the left-join in build_summary to 240 rows / 238 unique DUIDs.

- Dedupe the seeded feather (106 → 104 rows)
- drop_duplicates before the merge as a defensive guard
- Assert DUID uniqueness in tests/validate_outputs.py so any future
  regression fails CI instead of shipping phantom rows
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Update renewable generator dashboard data 2026-07
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -532,12 +532,12 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Actual FY23-24</t>
+          <t>Actual FY24-25</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Actual FY24-25</t>
+          <t>Actual FY25-26</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -644,11 +644,9 @@
         <v>132</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0.0511</v>
-      </c>
-      <c r="K2" s="5" t="n">
         <v>0.1441</v>
       </c>
+      <c r="K2" s="5" t="inlineStr"/>
       <c r="L2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -729,11 +727,9 @@
         <v>66</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.0521</v>
-      </c>
-      <c r="K3" s="5" t="n">
         <v>0.128</v>
       </c>
+      <c r="K3" s="5" t="inlineStr"/>
       <c r="L3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -814,11 +810,9 @@
         <v>132</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="K4" s="5" t="n">
         <v>0.123</v>
       </c>
+      <c r="K4" s="5" t="inlineStr"/>
       <c r="L4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -899,11 +893,9 @@
         <v>22</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="K5" s="5" t="n">
         <v>0.1492</v>
       </c>
+      <c r="K5" s="5" t="inlineStr"/>
       <c r="L5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -1039,11 +1031,9 @@
         <v>132</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.0327</v>
-      </c>
-      <c r="K7" s="5" t="n">
         <v>0.0292</v>
       </c>
+      <c r="K7" s="5" t="inlineStr"/>
       <c r="L7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1108,11 +1098,9 @@
         <v>132</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0862</v>
-      </c>
-      <c r="K8" s="5" t="n">
         <v>0.0799</v>
       </c>
+      <c r="K8" s="5" t="inlineStr"/>
       <c r="L8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -1248,11 +1236,9 @@
         <v>132</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0636</v>
-      </c>
-      <c r="K10" s="5" t="n">
         <v>0.0833</v>
       </c>
+      <c r="K10" s="5" t="inlineStr"/>
       <c r="L10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1317,11 +1303,9 @@
         <v>132</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.0643</v>
-      </c>
-      <c r="K11" s="5" t="n">
         <v>0.0762</v>
       </c>
+      <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="5" t="n">
         <v>0.7032826997896851</v>
       </c>
@@ -1441,11 +1425,9 @@
         <v>66</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="K13" s="5" t="n">
         <v>0.3285</v>
       </c>
+      <c r="K13" s="5" t="inlineStr"/>
       <c r="L13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1591,11 +1573,9 @@
         <v>330</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>0.0328</v>
-      </c>
-      <c r="K15" s="5" t="n">
         <v>0.1353</v>
       </c>
+      <c r="K15" s="5" t="inlineStr"/>
       <c r="L15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -1660,11 +1640,9 @@
         <v>132</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.1268</v>
-      </c>
-      <c r="K16" s="5" t="n">
         <v>0.1778</v>
       </c>
+      <c r="K16" s="5" t="inlineStr"/>
       <c r="L16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -1745,11 +1723,9 @@
         <v>132</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.1304</v>
-      </c>
-      <c r="K17" s="5" t="n">
         <v>0.2781</v>
       </c>
+      <c r="K17" s="5" t="inlineStr"/>
       <c r="L17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1814,11 +1790,9 @@
         <v>66</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.06950000000000001</v>
-      </c>
-      <c r="K18" s="5" t="n">
         <v>0.1147</v>
       </c>
+      <c r="K18" s="5" t="inlineStr"/>
       <c r="L18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1883,11 +1857,9 @@
         <v>132</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.1534</v>
-      </c>
-      <c r="K19" s="5" t="n">
         <v>0.2801</v>
       </c>
+      <c r="K19" s="5" t="inlineStr"/>
       <c r="L19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -1968,11 +1940,9 @@
         <v>220</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.1138</v>
-      </c>
-      <c r="K20" s="5" t="n">
         <v>0.2431</v>
       </c>
+      <c r="K20" s="5" t="inlineStr"/>
       <c r="L20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2053,11 +2023,9 @@
         <v>22</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.1244</v>
-      </c>
-      <c r="K21" s="5" t="n">
         <v>0.2403</v>
       </c>
+      <c r="K21" s="5" t="inlineStr"/>
       <c r="L21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2138,11 +2106,9 @@
         <v>132</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.4514</v>
-      </c>
-      <c r="K22" s="5" t="n">
         <v>0.5511</v>
       </c>
+      <c r="K22" s="5" t="inlineStr"/>
       <c r="L22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2223,11 +2189,9 @@
         <v>132</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="K23" s="5" t="n">
         <v>0.0614</v>
       </c>
+      <c r="K23" s="5" t="inlineStr"/>
       <c r="L23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2308,11 +2272,9 @@
         <v>66</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="K24" s="5" t="n">
         <v>0.5639</v>
       </c>
+      <c r="K24" s="5" t="inlineStr"/>
       <c r="L24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2393,11 +2355,9 @@
         <v>66</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="K25" s="5" t="n">
         <v>0.0089</v>
       </c>
+      <c r="K25" s="5" t="inlineStr"/>
       <c r="L25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -2649,11 +2609,9 @@
         <v>132</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>0.0332</v>
-      </c>
-      <c r="K29" s="5" t="n">
         <v>0.078</v>
       </c>
+      <c r="K29" s="5" t="inlineStr"/>
       <c r="L29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2734,11 +2692,9 @@
         <v>330</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.0851</v>
-      </c>
-      <c r="K30" s="5" t="n">
         <v>0.125</v>
       </c>
+      <c r="K30" s="5" t="inlineStr"/>
       <c r="L30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2819,11 +2775,9 @@
         <v>330</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>0.0885</v>
-      </c>
-      <c r="K31" s="5" t="n">
         <v>0.1153</v>
       </c>
+      <c r="K31" s="5" t="inlineStr"/>
       <c r="L31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2904,11 +2858,9 @@
         <v>132</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0277</v>
-      </c>
-      <c r="K32" s="5" t="n">
         <v>0.0388</v>
       </c>
+      <c r="K32" s="5" t="inlineStr"/>
       <c r="L32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2989,11 +2941,9 @@
         <v>66</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="K33" s="5" t="n">
         <v>0.2694</v>
       </c>
+      <c r="K33" s="5" t="inlineStr"/>
       <c r="L33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -3168,11 +3118,9 @@
         <v>220</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1059</v>
-      </c>
-      <c r="K36" s="5" t="n">
         <v>0.1146</v>
       </c>
+      <c r="K36" s="5" t="inlineStr"/>
       <c r="L36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -3253,11 +3201,9 @@
         <v>132</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>0.1766</v>
-      </c>
-      <c r="K37" s="5" t="n">
         <v>0.2365</v>
       </c>
+      <c r="K37" s="5" t="inlineStr"/>
       <c r="L37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -3565,11 +3511,9 @@
         <v>132</v>
       </c>
       <c r="J41" s="5" t="n">
-        <v>0.1231</v>
-      </c>
-      <c r="K41" s="5" t="n">
         <v>0.1167</v>
       </c>
+      <c r="K41" s="5" t="inlineStr"/>
       <c r="L41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3650,11 +3594,9 @@
         <v>66</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.1585</v>
-      </c>
-      <c r="K42" s="5" t="n">
         <v>0.2501</v>
       </c>
+      <c r="K42" s="5" t="inlineStr"/>
       <c r="L42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3864,10 +3806,10 @@
       <c r="I45" s="2" t="n">
         <v>330</v>
       </c>
-      <c r="J45" s="5" t="inlineStr"/>
-      <c r="K45" s="5" t="n">
+      <c r="J45" s="5" t="n">
         <v>0.0616</v>
       </c>
+      <c r="K45" s="5" t="inlineStr"/>
       <c r="L45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3948,11 +3890,9 @@
         <v>132</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>0.0315</v>
-      </c>
-      <c r="K46" s="5" t="n">
         <v>0.0306</v>
       </c>
+      <c r="K46" s="5" t="inlineStr"/>
       <c r="L46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -4033,11 +3973,9 @@
         <v>132</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>0.1433</v>
-      </c>
-      <c r="K47" s="5" t="n">
         <v>0.1883</v>
       </c>
+      <c r="K47" s="5" t="inlineStr"/>
       <c r="L47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -4102,11 +4040,9 @@
         <v>132</v>
       </c>
       <c r="J48" s="5" t="n">
-        <v>0.06519999999999999</v>
-      </c>
-      <c r="K48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
+      <c r="K48" s="5" t="inlineStr"/>
       <c r="L48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -4252,11 +4188,9 @@
         <v>132</v>
       </c>
       <c r="J50" s="5" t="n">
-        <v>0.2031</v>
-      </c>
-      <c r="K50" s="5" t="n">
         <v>0.1969</v>
       </c>
+      <c r="K50" s="5" t="inlineStr"/>
       <c r="L50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -4315,11 +4249,9 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="5" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="K51" s="5" t="n">
         <v>0.0528</v>
       </c>
+      <c r="K51" s="5" t="inlineStr"/>
       <c r="L51" s="5" t="inlineStr"/>
       <c r="M51" s="5" t="inlineStr"/>
       <c r="N51" s="5" t="n">
@@ -4374,11 +4306,9 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="5" t="n">
-        <v>0.0983</v>
-      </c>
-      <c r="K52" s="5" t="n">
         <v>0.1308</v>
       </c>
+      <c r="K52" s="5" t="inlineStr"/>
       <c r="L52" s="5" t="inlineStr"/>
       <c r="M52" s="5" t="inlineStr"/>
       <c r="N52" s="5" t="n">
@@ -4433,11 +4363,9 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="5" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="K53" s="5" t="n">
         <v>0.0143</v>
       </c>
+      <c r="K53" s="5" t="inlineStr"/>
       <c r="L53" s="5" t="inlineStr"/>
       <c r="M53" s="5" t="inlineStr"/>
       <c r="N53" s="5" t="n">
@@ -4492,11 +4420,9 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="5" t="n">
-        <v>0.0213</v>
-      </c>
-      <c r="K54" s="5" t="n">
         <v>0.0265</v>
       </c>
+      <c r="K54" s="5" t="inlineStr"/>
       <c r="L54" s="5" t="inlineStr"/>
       <c r="M54" s="5" t="inlineStr"/>
       <c r="N54" s="5" t="n">
@@ -4606,11 +4532,9 @@
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="5" t="n">
-        <v>0.0031</v>
-      </c>
-      <c r="K56" s="5" t="n">
         <v>0.0066</v>
       </c>
+      <c r="K56" s="5" t="inlineStr"/>
       <c r="L56" s="5" t="inlineStr"/>
       <c r="M56" s="5" t="inlineStr"/>
       <c r="N56" s="5" t="n">
@@ -4775,11 +4699,9 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="5" t="n">
-        <v>0.0109</v>
-      </c>
-      <c r="K59" s="5" t="n">
         <v>0.0298</v>
       </c>
+      <c r="K59" s="5" t="inlineStr"/>
       <c r="L59" s="5" t="inlineStr"/>
       <c r="M59" s="5" t="inlineStr"/>
       <c r="N59" s="5" t="n">
@@ -4888,10 +4810,10 @@
         <v>145</v>
       </c>
       <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="5" t="inlineStr"/>
-      <c r="K61" s="5" t="n">
+      <c r="J61" s="5" t="n">
         <v>0.0509</v>
       </c>
+      <c r="K61" s="5" t="inlineStr"/>
       <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr"/>
       <c r="N61" s="5" t="n">
@@ -4946,11 +4868,9 @@
       </c>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="5" t="n">
-        <v>0.0024</v>
-      </c>
-      <c r="K62" s="5" t="n">
         <v>0.0168</v>
       </c>
+      <c r="K62" s="5" t="inlineStr"/>
       <c r="L62" s="5" t="inlineStr"/>
       <c r="M62" s="5" t="inlineStr"/>
       <c r="N62" s="5" t="n">
@@ -5005,11 +4925,9 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="5" t="n">
-        <v>0.0155</v>
-      </c>
-      <c r="K63" s="5" t="n">
         <v>0.055</v>
       </c>
+      <c r="K63" s="5" t="inlineStr"/>
       <c r="L63" s="5" t="inlineStr"/>
       <c r="M63" s="5" t="inlineStr"/>
       <c r="N63" s="5" t="n">
@@ -5064,11 +4982,9 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="5" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="K64" s="5" t="n">
         <v>0.0178</v>
       </c>
+      <c r="K64" s="5" t="inlineStr"/>
       <c r="L64" s="5" t="inlineStr"/>
       <c r="M64" s="5" t="inlineStr"/>
       <c r="N64" s="5" t="n">
@@ -5122,10 +5038,10 @@
         <v>396</v>
       </c>
       <c r="I65" s="2" t="inlineStr"/>
-      <c r="J65" s="5" t="inlineStr"/>
-      <c r="K65" s="5" t="n">
+      <c r="J65" s="5" t="n">
         <v>0.0134</v>
       </c>
+      <c r="K65" s="5" t="inlineStr"/>
       <c r="L65" s="5" t="inlineStr"/>
       <c r="M65" s="5" t="inlineStr"/>
       <c r="N65" s="5" t="n">
@@ -5180,11 +5096,9 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="5" t="n">
-        <v>0.0048</v>
-      </c>
-      <c r="K66" s="5" t="n">
         <v>0.0056</v>
       </c>
+      <c r="K66" s="5" t="inlineStr"/>
       <c r="L66" s="5" t="inlineStr"/>
       <c r="M66" s="5" t="inlineStr"/>
       <c r="N66" s="5" t="n">
@@ -5239,11 +5153,9 @@
       </c>
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="5" t="n">
-        <v>0.0354</v>
-      </c>
-      <c r="K67" s="5" t="n">
         <v>0.064</v>
       </c>
+      <c r="K67" s="5" t="inlineStr"/>
       <c r="L67" s="5" t="inlineStr"/>
       <c r="M67" s="5" t="inlineStr"/>
       <c r="N67" s="5" t="n">
@@ -5298,11 +5210,9 @@
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="K68" s="5" t="n">
         <v>0.0002</v>
       </c>
+      <c r="K68" s="5" t="inlineStr"/>
       <c r="L68" s="5" t="inlineStr"/>
       <c r="M68" s="5" t="inlineStr"/>
       <c r="N68" s="5" t="n">
@@ -5357,11 +5267,9 @@
       </c>
       <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="5" t="n">
-        <v>0.0291</v>
-      </c>
-      <c r="K69" s="5" t="n">
         <v>0.0573</v>
       </c>
+      <c r="K69" s="5" t="inlineStr"/>
       <c r="L69" s="5" t="inlineStr"/>
       <c r="M69" s="5" t="inlineStr"/>
       <c r="N69" s="5" t="n">
@@ -5416,11 +5324,9 @@
       </c>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="5" t="n">
-        <v>0.0157</v>
-      </c>
-      <c r="K70" s="5" t="n">
         <v>0.0294</v>
       </c>
+      <c r="K70" s="5" t="inlineStr"/>
       <c r="L70" s="5" t="inlineStr"/>
       <c r="M70" s="5" t="inlineStr"/>
       <c r="N70" s="5" t="n">
@@ -5499,12 +5405,12 @@
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>CURTAILMENT_ACTUAL_FY23-24</t>
+          <t>CURTAILMENT_ACTUAL_FY24-25</t>
         </is>
       </c>
       <c r="F1" s="7" t="inlineStr">
         <is>
-          <t>CURTAILMENT_ACTUAL_FY24-25</t>
+          <t>CURTAILMENT_ACTUAL_FY25-26</t>
         </is>
       </c>
       <c r="G1" s="7" t="inlineStr">
@@ -5606,11 +5512,9 @@
         <v>0.8395</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.0511</v>
-      </c>
-      <c r="F2" s="5" t="n">
         <v>0.1441</v>
       </c>
+      <c r="F2" s="5" t="inlineStr"/>
       <c r="G2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5690,11 +5594,9 @@
         <v>0.9245</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.0521</v>
-      </c>
-      <c r="F3" s="5" t="n">
         <v>0.128</v>
       </c>
+      <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -5774,11 +5676,9 @@
         <v>0.8823</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="F4" s="5" t="n">
         <v>0.123</v>
       </c>
+      <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5858,11 +5758,9 @@
         <v>0.8436</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="F5" s="5" t="n">
         <v>0.1492</v>
       </c>
+      <c r="F5" s="5" t="inlineStr"/>
       <c r="G5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -6002,11 +5900,9 @@
         <v>0.8416</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.0327</v>
-      </c>
-      <c r="F7" s="5" t="n">
         <v>0.0292</v>
       </c>
+      <c r="F7" s="5" t="inlineStr"/>
       <c r="G7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6070,11 +5966,9 @@
         <v>0.8899</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0862</v>
-      </c>
-      <c r="F8" s="5" t="n">
         <v>0.0799</v>
       </c>
+      <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -6214,11 +6108,9 @@
         <v>0.8554</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0636</v>
-      </c>
-      <c r="F10" s="5" t="n">
         <v>0.0833</v>
       </c>
+      <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6282,11 +6174,9 @@
         <v>0.8521</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.0643</v>
-      </c>
-      <c r="F11" s="5" t="n">
         <v>0.0762</v>
       </c>
+      <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="n">
         <v>0.7032826997896851</v>
       </c>
@@ -6410,11 +6300,9 @@
         <v>0.8918</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="F13" s="5" t="n">
         <v>0.3285</v>
       </c>
+      <c r="F13" s="5" t="inlineStr"/>
       <c r="G13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6558,11 +6446,9 @@
         <v>0.9635</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.0328</v>
-      </c>
-      <c r="F15" s="5" t="n">
         <v>0.1353</v>
       </c>
+      <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -6626,11 +6512,9 @@
         <v>0.8463000000000001</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.1268</v>
-      </c>
-      <c r="F16" s="5" t="n">
         <v>0.1778</v>
       </c>
+      <c r="F16" s="5" t="inlineStr"/>
       <c r="G16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -6710,11 +6594,9 @@
         <v>0.8652</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.1304</v>
-      </c>
-      <c r="F17" s="5" t="n">
         <v>0.2781</v>
       </c>
+      <c r="F17" s="5" t="inlineStr"/>
       <c r="G17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6778,11 +6660,9 @@
         <v>0.8962</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.06950000000000001</v>
-      </c>
-      <c r="F18" s="5" t="n">
         <v>0.1147</v>
       </c>
+      <c r="F18" s="5" t="inlineStr"/>
       <c r="G18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6846,11 +6726,9 @@
         <v>0.8865</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.1534</v>
-      </c>
-      <c r="F19" s="5" t="n">
         <v>0.2801</v>
       </c>
+      <c r="F19" s="5" t="inlineStr"/>
       <c r="G19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -6930,11 +6808,9 @@
         <v>0.8206</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.1138</v>
-      </c>
-      <c r="F20" s="5" t="n">
         <v>0.2431</v>
       </c>
+      <c r="F20" s="5" t="inlineStr"/>
       <c r="G20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -7014,11 +6890,9 @@
         <v>0.8268</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.1244</v>
-      </c>
-      <c r="F21" s="5" t="n">
         <v>0.2403</v>
       </c>
+      <c r="F21" s="5" t="inlineStr"/>
       <c r="G21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -7098,11 +6972,9 @@
         <v>0.9482</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.4514</v>
-      </c>
-      <c r="F22" s="5" t="n">
         <v>0.5511</v>
       </c>
+      <c r="F22" s="5" t="inlineStr"/>
       <c r="G22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7182,11 +7054,9 @@
         <v>0.8657</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.0075</v>
-      </c>
-      <c r="F23" s="5" t="n">
         <v>0.0614</v>
       </c>
+      <c r="F23" s="5" t="inlineStr"/>
       <c r="G23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7266,11 +7136,9 @@
         <v>0.9583</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.488</v>
-      </c>
-      <c r="F24" s="5" t="n">
         <v>0.5639</v>
       </c>
+      <c r="F24" s="5" t="inlineStr"/>
       <c r="G24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7350,11 +7218,9 @@
         <v>0.8509</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.012</v>
-      </c>
-      <c r="F25" s="5" t="n">
         <v>0.0089</v>
       </c>
+      <c r="F25" s="5" t="inlineStr"/>
       <c r="G25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -7614,11 +7480,9 @@
         <v>0.9273</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>0.0332</v>
-      </c>
-      <c r="F29" s="5" t="n">
         <v>0.078</v>
       </c>
+      <c r="F29" s="5" t="inlineStr"/>
       <c r="G29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7698,11 +7562,9 @@
         <v>0.8911</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.0851</v>
-      </c>
-      <c r="F30" s="5" t="n">
         <v>0.125</v>
       </c>
+      <c r="F30" s="5" t="inlineStr"/>
       <c r="G30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7782,11 +7644,9 @@
         <v>0.8911</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.0885</v>
-      </c>
-      <c r="F31" s="5" t="n">
         <v>0.1153</v>
       </c>
+      <c r="F31" s="5" t="inlineStr"/>
       <c r="G31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7866,11 +7726,9 @@
         <v>0.9699</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0277</v>
-      </c>
-      <c r="F32" s="5" t="n">
         <v>0.0388</v>
       </c>
+      <c r="F32" s="5" t="inlineStr"/>
       <c r="G32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7950,11 +7808,9 @@
         <v>0.8918</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>0.123</v>
-      </c>
-      <c r="F33" s="5" t="n">
         <v>0.2694</v>
       </c>
+      <c r="F33" s="5" t="inlineStr"/>
       <c r="G33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -8138,11 +7994,9 @@
         <v>0.8218</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.1059</v>
-      </c>
-      <c r="F36" s="5" t="n">
         <v>0.1146</v>
       </c>
+      <c r="F36" s="5" t="inlineStr"/>
       <c r="G36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -8222,11 +8076,9 @@
         <v>0.8865</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>0.1766</v>
-      </c>
-      <c r="F37" s="5" t="n">
         <v>0.2365</v>
       </c>
+      <c r="F37" s="5" t="inlineStr"/>
       <c r="G37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -8530,11 +8382,9 @@
         <v>0.9091</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>0.1231</v>
-      </c>
-      <c r="F41" s="5" t="n">
         <v>0.1167</v>
       </c>
+      <c r="F41" s="5" t="inlineStr"/>
       <c r="G41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8614,11 +8464,9 @@
         <v>0.8824</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.1585</v>
-      </c>
-      <c r="F42" s="5" t="n">
         <v>0.2501</v>
       </c>
+      <c r="F42" s="5" t="inlineStr"/>
       <c r="G42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8825,10 +8673,10 @@
       <c r="D45" s="5" t="n">
         <v>0.9376</v>
       </c>
-      <c r="E45" s="5" t="inlineStr"/>
-      <c r="F45" s="5" t="n">
+      <c r="E45" s="5" t="n">
         <v>0.0616</v>
       </c>
+      <c r="F45" s="5" t="inlineStr"/>
       <c r="G45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8908,11 +8756,9 @@
         <v>0.9273</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>0.0315</v>
-      </c>
-      <c r="F46" s="5" t="n">
         <v>0.0306</v>
       </c>
+      <c r="F46" s="5" t="inlineStr"/>
       <c r="G46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8992,11 +8838,9 @@
         <v>0.8865</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>0.1433</v>
-      </c>
-      <c r="F47" s="5" t="n">
         <v>0.1883</v>
       </c>
+      <c r="F47" s="5" t="inlineStr"/>
       <c r="G47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -9060,11 +8904,9 @@
         <v>0.8265</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>0.06519999999999999</v>
-      </c>
-      <c r="F48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
+      <c r="F48" s="5" t="inlineStr"/>
       <c r="G48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -9208,11 +9050,9 @@
         <v>0.8865</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>0.2031</v>
-      </c>
-      <c r="F50" s="5" t="n">
         <v>0.1969</v>
       </c>
+      <c r="F50" s="5" t="inlineStr"/>
       <c r="G50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -9276,11 +9116,9 @@
         <v>0.9254</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>0.042</v>
-      </c>
-      <c r="F51" s="5" t="n">
         <v>0.0528</v>
       </c>
+      <c r="F51" s="5" t="inlineStr"/>
       <c r="G51" s="5" t="inlineStr"/>
       <c r="H51" s="5" t="inlineStr"/>
       <c r="I51" s="5" t="inlineStr"/>
@@ -9340,11 +9178,9 @@
         <v>0.9391</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>0.0983</v>
-      </c>
-      <c r="F52" s="5" t="n">
         <v>0.1308</v>
       </c>
+      <c r="F52" s="5" t="inlineStr"/>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr"/>
@@ -9404,11 +9240,9 @@
         <v>0.9638</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="F53" s="5" t="n">
         <v>0.0143</v>
       </c>
+      <c r="F53" s="5" t="inlineStr"/>
       <c r="G53" s="5" t="inlineStr"/>
       <c r="H53" s="5" t="inlineStr"/>
       <c r="I53" s="5" t="inlineStr"/>
@@ -9468,11 +9302,9 @@
         <v>0.9545</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>0.0213</v>
-      </c>
-      <c r="F54" s="5" t="n">
         <v>0.0265</v>
       </c>
+      <c r="F54" s="5" t="inlineStr"/>
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="5" t="inlineStr"/>
@@ -9592,11 +9424,9 @@
         <v>0.9643</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>0.0031</v>
-      </c>
-      <c r="F56" s="5" t="n">
         <v>0.0066</v>
       </c>
+      <c r="F56" s="5" t="inlineStr"/>
       <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="5" t="inlineStr"/>
@@ -9776,11 +9606,9 @@
         <v>0.9276</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>0.0109</v>
-      </c>
-      <c r="F59" s="5" t="n">
         <v>0.0298</v>
       </c>
+      <c r="F59" s="5" t="inlineStr"/>
       <c r="G59" s="5" t="inlineStr"/>
       <c r="H59" s="5" t="inlineStr"/>
       <c r="I59" s="5" t="inlineStr"/>
@@ -9899,10 +9727,10 @@
       <c r="D61" s="5" t="n">
         <v>1.0047</v>
       </c>
-      <c r="E61" s="5" t="inlineStr"/>
-      <c r="F61" s="5" t="n">
+      <c r="E61" s="5" t="n">
         <v>0.0509</v>
       </c>
+      <c r="F61" s="5" t="inlineStr"/>
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr"/>
       <c r="I61" s="5" t="inlineStr"/>
@@ -9962,11 +9790,9 @@
         <v>0.9635</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>0.0024</v>
-      </c>
-      <c r="F62" s="5" t="n">
         <v>0.0168</v>
       </c>
+      <c r="F62" s="5" t="inlineStr"/>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr"/>
       <c r="I62" s="5" t="inlineStr"/>
@@ -10026,11 +9852,9 @@
         <v>0.9635</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>0.0155</v>
-      </c>
-      <c r="F63" s="5" t="n">
         <v>0.055</v>
       </c>
+      <c r="F63" s="5" t="inlineStr"/>
       <c r="G63" s="5" t="inlineStr"/>
       <c r="H63" s="5" t="inlineStr"/>
       <c r="I63" s="5" t="inlineStr"/>
@@ -10090,11 +9914,9 @@
         <v>0.9528</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="F64" s="5" t="n">
         <v>0.0178</v>
       </c>
+      <c r="F64" s="5" t="inlineStr"/>
       <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr"/>
       <c r="I64" s="5" t="inlineStr"/>
@@ -10153,10 +9975,10 @@
       <c r="D65" s="5" t="n">
         <v>0.9618</v>
       </c>
-      <c r="E65" s="5" t="inlineStr"/>
-      <c r="F65" s="5" t="n">
+      <c r="E65" s="5" t="n">
         <v>0.0134</v>
       </c>
+      <c r="F65" s="5" t="inlineStr"/>
       <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr"/>
       <c r="I65" s="5" t="inlineStr"/>
@@ -10216,11 +10038,9 @@
         <v>0.8661</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>0.0048</v>
-      </c>
-      <c r="F66" s="5" t="n">
         <v>0.0056</v>
       </c>
+      <c r="F66" s="5" t="inlineStr"/>
       <c r="G66" s="5" t="inlineStr"/>
       <c r="H66" s="5" t="inlineStr"/>
       <c r="I66" s="5" t="inlineStr"/>
@@ -10280,11 +10100,9 @@
         <v>0.896</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>0.0354</v>
-      </c>
-      <c r="F67" s="5" t="n">
         <v>0.064</v>
       </c>
+      <c r="F67" s="5" t="inlineStr"/>
       <c r="G67" s="5" t="inlineStr"/>
       <c r="H67" s="5" t="inlineStr"/>
       <c r="I67" s="5" t="inlineStr"/>
@@ -10344,11 +10162,9 @@
         <v>1.0029</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>0.0001</v>
-      </c>
-      <c r="F68" s="5" t="n">
         <v>0.0002</v>
       </c>
+      <c r="F68" s="5" t="inlineStr"/>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr"/>
       <c r="I68" s="5" t="inlineStr"/>
@@ -10408,11 +10224,9 @@
         <v>0.8265</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>0.0291</v>
-      </c>
-      <c r="F69" s="5" t="n">
         <v>0.0573</v>
       </c>
+      <c r="F69" s="5" t="inlineStr"/>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr"/>
       <c r="I69" s="5" t="inlineStr"/>
@@ -10472,11 +10286,9 @@
         <v>0.9694</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>0.0157</v>
-      </c>
-      <c r="F70" s="5" t="n">
         <v>0.0294</v>
       </c>
+      <c r="F70" s="5" t="inlineStr"/>
       <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr"/>
       <c r="I70" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update renewable generator dashboard data 2026-08
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -646,7 +646,9 @@
       <c r="J2" s="5" t="n">
         <v>0.1441</v>
       </c>
-      <c r="K2" s="5" t="inlineStr"/>
+      <c r="K2" s="5" t="n">
+        <v>0.1695</v>
+      </c>
       <c r="L2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -729,7 +731,9 @@
       <c r="J3" s="5" t="n">
         <v>0.128</v>
       </c>
-      <c r="K3" s="5" t="inlineStr"/>
+      <c r="K3" s="5" t="n">
+        <v>0.078</v>
+      </c>
       <c r="L3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -812,7 +816,9 @@
       <c r="J4" s="5" t="n">
         <v>0.123</v>
       </c>
-      <c r="K4" s="5" t="inlineStr"/>
+      <c r="K4" s="5" t="n">
+        <v>0.1001</v>
+      </c>
       <c r="L4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -895,7 +901,9 @@
       <c r="J5" s="5" t="n">
         <v>0.1492</v>
       </c>
-      <c r="K5" s="5" t="inlineStr"/>
+      <c r="K5" s="5" t="n">
+        <v>0.2117</v>
+      </c>
       <c r="L5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -1033,7 +1041,9 @@
       <c r="J7" s="5" t="n">
         <v>0.0292</v>
       </c>
-      <c r="K7" s="5" t="inlineStr"/>
+      <c r="K7" s="5" t="n">
+        <v>0.0415</v>
+      </c>
       <c r="L7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1100,7 +1110,9 @@
       <c r="J8" s="5" t="n">
         <v>0.0799</v>
       </c>
-      <c r="K8" s="5" t="inlineStr"/>
+      <c r="K8" s="5" t="n">
+        <v>0.1689</v>
+      </c>
       <c r="L8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -1175,7 +1187,9 @@
       </c>
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
-      <c r="K9" s="5" t="inlineStr"/>
+      <c r="K9" s="5" t="n">
+        <v>0.342</v>
+      </c>
       <c r="L9" s="5" t="inlineStr"/>
       <c r="M9" s="5" t="inlineStr"/>
       <c r="N9" s="5" t="n">
@@ -1238,7 +1252,9 @@
       <c r="J10" s="5" t="n">
         <v>0.0833</v>
       </c>
-      <c r="K10" s="5" t="inlineStr"/>
+      <c r="K10" s="5" t="n">
+        <v>0.1175</v>
+      </c>
       <c r="L10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1427,7 +1443,9 @@
       <c r="J13" s="5" t="n">
         <v>0.3285</v>
       </c>
-      <c r="K13" s="5" t="inlineStr"/>
+      <c r="K13" s="5" t="n">
+        <v>0.3999</v>
+      </c>
       <c r="L13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1575,7 +1593,9 @@
       <c r="J15" s="5" t="n">
         <v>0.1353</v>
       </c>
-      <c r="K15" s="5" t="inlineStr"/>
+      <c r="K15" s="5" t="n">
+        <v>0.2162</v>
+      </c>
       <c r="L15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -1642,7 +1662,9 @@
       <c r="J16" s="5" t="n">
         <v>0.1778</v>
       </c>
-      <c r="K16" s="5" t="inlineStr"/>
+      <c r="K16" s="5" t="n">
+        <v>0.2693</v>
+      </c>
       <c r="L16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -1725,7 +1747,9 @@
       <c r="J17" s="5" t="n">
         <v>0.2781</v>
       </c>
-      <c r="K17" s="5" t="inlineStr"/>
+      <c r="K17" s="5" t="n">
+        <v>0.1928</v>
+      </c>
       <c r="L17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -1792,7 +1816,9 @@
       <c r="J18" s="5" t="n">
         <v>0.1147</v>
       </c>
-      <c r="K18" s="5" t="inlineStr"/>
+      <c r="K18" s="5" t="n">
+        <v>0.3103</v>
+      </c>
       <c r="L18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -1859,7 +1885,9 @@
       <c r="J19" s="5" t="n">
         <v>0.2801</v>
       </c>
-      <c r="K19" s="5" t="inlineStr"/>
+      <c r="K19" s="5" t="n">
+        <v>0.2607</v>
+      </c>
       <c r="L19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -1942,7 +1970,9 @@
       <c r="J20" s="5" t="n">
         <v>0.2431</v>
       </c>
-      <c r="K20" s="5" t="inlineStr"/>
+      <c r="K20" s="5" t="n">
+        <v>0.2125</v>
+      </c>
       <c r="L20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2025,7 +2055,9 @@
       <c r="J21" s="5" t="n">
         <v>0.2403</v>
       </c>
-      <c r="K21" s="5" t="inlineStr"/>
+      <c r="K21" s="5" t="n">
+        <v>0.1922</v>
+      </c>
       <c r="L21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -2108,7 +2140,9 @@
       <c r="J22" s="5" t="n">
         <v>0.5511</v>
       </c>
-      <c r="K22" s="5" t="inlineStr"/>
+      <c r="K22" s="5" t="n">
+        <v>0.5341</v>
+      </c>
       <c r="L22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2191,7 +2225,9 @@
       <c r="J23" s="5" t="n">
         <v>0.0614</v>
       </c>
-      <c r="K23" s="5" t="inlineStr"/>
+      <c r="K23" s="5" t="n">
+        <v>0.1487</v>
+      </c>
       <c r="L23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2274,7 +2310,9 @@
       <c r="J24" s="5" t="n">
         <v>0.5639</v>
       </c>
-      <c r="K24" s="5" t="inlineStr"/>
+      <c r="K24" s="5" t="n">
+        <v>0.3973</v>
+      </c>
       <c r="L24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -2357,7 +2395,9 @@
       <c r="J25" s="5" t="n">
         <v>0.0089</v>
       </c>
-      <c r="K25" s="5" t="inlineStr"/>
+      <c r="K25" s="5" t="n">
+        <v>0.0169</v>
+      </c>
       <c r="L25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -2611,7 +2651,9 @@
       <c r="J29" s="5" t="n">
         <v>0.078</v>
       </c>
-      <c r="K29" s="5" t="inlineStr"/>
+      <c r="K29" s="5" t="n">
+        <v>0.2905</v>
+      </c>
       <c r="L29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2694,7 +2736,9 @@
       <c r="J30" s="5" t="n">
         <v>0.125</v>
       </c>
-      <c r="K30" s="5" t="inlineStr"/>
+      <c r="K30" s="5" t="n">
+        <v>0.0318</v>
+      </c>
       <c r="L30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2777,7 +2821,9 @@
       <c r="J31" s="5" t="n">
         <v>0.1153</v>
       </c>
-      <c r="K31" s="5" t="inlineStr"/>
+      <c r="K31" s="5" t="n">
+        <v>0.036</v>
+      </c>
       <c r="L31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -2860,7 +2906,9 @@
       <c r="J32" s="5" t="n">
         <v>0.0388</v>
       </c>
-      <c r="K32" s="5" t="inlineStr"/>
+      <c r="K32" s="5" t="n">
+        <v>0.2983</v>
+      </c>
       <c r="L32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -2943,7 +2991,9 @@
       <c r="J33" s="5" t="n">
         <v>0.2694</v>
       </c>
-      <c r="K33" s="5" t="inlineStr"/>
+      <c r="K33" s="5" t="n">
+        <v>0.2848</v>
+      </c>
       <c r="L33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -3120,7 +3170,9 @@
       <c r="J36" s="5" t="n">
         <v>0.1146</v>
       </c>
-      <c r="K36" s="5" t="inlineStr"/>
+      <c r="K36" s="5" t="n">
+        <v>0.0936</v>
+      </c>
       <c r="L36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -3203,7 +3255,9 @@
       <c r="J37" s="5" t="n">
         <v>0.2365</v>
       </c>
-      <c r="K37" s="5" t="inlineStr"/>
+      <c r="K37" s="5" t="n">
+        <v>0.2465</v>
+      </c>
       <c r="L37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -3349,7 +3403,9 @@
         <v>330</v>
       </c>
       <c r="J39" s="5" t="inlineStr"/>
-      <c r="K39" s="5" t="inlineStr"/>
+      <c r="K39" s="5" t="n">
+        <v>0.08939999999999999</v>
+      </c>
       <c r="L39" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -3430,7 +3486,9 @@
         <v>330</v>
       </c>
       <c r="J40" s="5" t="inlineStr"/>
-      <c r="K40" s="5" t="inlineStr"/>
+      <c r="K40" s="5" t="n">
+        <v>0.0813</v>
+      </c>
       <c r="L40" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -3513,7 +3571,9 @@
       <c r="J41" s="5" t="n">
         <v>0.1167</v>
       </c>
-      <c r="K41" s="5" t="inlineStr"/>
+      <c r="K41" s="5" t="n">
+        <v>0.2803</v>
+      </c>
       <c r="L41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3596,7 +3656,9 @@
       <c r="J42" s="5" t="n">
         <v>0.2501</v>
       </c>
-      <c r="K42" s="5" t="inlineStr"/>
+      <c r="K42" s="5" t="n">
+        <v>0.2261</v>
+      </c>
       <c r="L42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3677,7 +3739,9 @@
         <v>330</v>
       </c>
       <c r="J43" s="5" t="inlineStr"/>
-      <c r="K43" s="5" t="inlineStr"/>
+      <c r="K43" s="5" t="n">
+        <v>0.2674</v>
+      </c>
       <c r="L43" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3742,7 +3806,9 @@
         <v>330</v>
       </c>
       <c r="J44" s="5" t="inlineStr"/>
-      <c r="K44" s="5" t="inlineStr"/>
+      <c r="K44" s="5" t="n">
+        <v>0.2715</v>
+      </c>
       <c r="L44" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -3809,7 +3875,9 @@
       <c r="J45" s="5" t="n">
         <v>0.0616</v>
       </c>
-      <c r="K45" s="5" t="inlineStr"/>
+      <c r="K45" s="5" t="n">
+        <v>0.0283</v>
+      </c>
       <c r="L45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3892,7 +3960,9 @@
       <c r="J46" s="5" t="n">
         <v>0.0306</v>
       </c>
-      <c r="K46" s="5" t="inlineStr"/>
+      <c r="K46" s="5" t="n">
+        <v>0.081</v>
+      </c>
       <c r="L46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -3975,7 +4045,9 @@
       <c r="J47" s="5" t="n">
         <v>0.1883</v>
       </c>
-      <c r="K47" s="5" t="inlineStr"/>
+      <c r="K47" s="5" t="n">
+        <v>0.1353</v>
+      </c>
       <c r="L47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -4042,7 +4114,9 @@
       <c r="J48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
-      <c r="K48" s="5" t="inlineStr"/>
+      <c r="K48" s="5" t="n">
+        <v>0.0301</v>
+      </c>
       <c r="L48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -4123,7 +4197,9 @@
         <v>330</v>
       </c>
       <c r="J49" s="5" t="inlineStr"/>
-      <c r="K49" s="5" t="inlineStr"/>
+      <c r="K49" s="5" t="n">
+        <v>0.0216</v>
+      </c>
       <c r="L49" s="5" t="n">
         <v>0.158699742317549</v>
       </c>
@@ -4190,7 +4266,9 @@
       <c r="J50" s="5" t="n">
         <v>0.1969</v>
       </c>
-      <c r="K50" s="5" t="inlineStr"/>
+      <c r="K50" s="5" t="n">
+        <v>0.1655</v>
+      </c>
       <c r="L50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -4251,7 +4329,9 @@
       <c r="J51" s="5" t="n">
         <v>0.0528</v>
       </c>
-      <c r="K51" s="5" t="inlineStr"/>
+      <c r="K51" s="5" t="n">
+        <v>0.0629</v>
+      </c>
       <c r="L51" s="5" t="inlineStr"/>
       <c r="M51" s="5" t="inlineStr"/>
       <c r="N51" s="5" t="n">
@@ -4308,7 +4388,9 @@
       <c r="J52" s="5" t="n">
         <v>0.1308</v>
       </c>
-      <c r="K52" s="5" t="inlineStr"/>
+      <c r="K52" s="5" t="n">
+        <v>0.1312</v>
+      </c>
       <c r="L52" s="5" t="inlineStr"/>
       <c r="M52" s="5" t="inlineStr"/>
       <c r="N52" s="5" t="n">
@@ -4365,7 +4447,9 @@
       <c r="J53" s="5" t="n">
         <v>0.0143</v>
       </c>
-      <c r="K53" s="5" t="inlineStr"/>
+      <c r="K53" s="5" t="n">
+        <v>0.0042</v>
+      </c>
       <c r="L53" s="5" t="inlineStr"/>
       <c r="M53" s="5" t="inlineStr"/>
       <c r="N53" s="5" t="n">
@@ -4422,7 +4506,9 @@
       <c r="J54" s="5" t="n">
         <v>0.0265</v>
       </c>
-      <c r="K54" s="5" t="inlineStr"/>
+      <c r="K54" s="5" t="n">
+        <v>0.0185</v>
+      </c>
       <c r="L54" s="5" t="inlineStr"/>
       <c r="M54" s="5" t="inlineStr"/>
       <c r="N54" s="5" t="n">
@@ -4534,7 +4620,9 @@
       <c r="J56" s="5" t="n">
         <v>0.0066</v>
       </c>
-      <c r="K56" s="5" t="inlineStr"/>
+      <c r="K56" s="5" t="n">
+        <v>0.0089</v>
+      </c>
       <c r="L56" s="5" t="inlineStr"/>
       <c r="M56" s="5" t="inlineStr"/>
       <c r="N56" s="5" t="n">
@@ -4589,7 +4677,9 @@
       </c>
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="5" t="inlineStr"/>
-      <c r="K57" s="5" t="inlineStr"/>
+      <c r="K57" s="5" t="n">
+        <v>0.0144</v>
+      </c>
       <c r="L57" s="5" t="inlineStr"/>
       <c r="M57" s="5" t="inlineStr"/>
       <c r="N57" s="5" t="n">
@@ -4644,7 +4734,9 @@
       </c>
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr"/>
-      <c r="K58" s="5" t="inlineStr"/>
+      <c r="K58" s="5" t="n">
+        <v>0.0219</v>
+      </c>
       <c r="L58" s="5" t="inlineStr"/>
       <c r="M58" s="5" t="inlineStr"/>
       <c r="N58" s="5" t="n">
@@ -4701,7 +4793,9 @@
       <c r="J59" s="5" t="n">
         <v>0.0298</v>
       </c>
-      <c r="K59" s="5" t="inlineStr"/>
+      <c r="K59" s="5" t="n">
+        <v>0.0184</v>
+      </c>
       <c r="L59" s="5" t="inlineStr"/>
       <c r="M59" s="5" t="inlineStr"/>
       <c r="N59" s="5" t="n">
@@ -4813,7 +4907,9 @@
       <c r="J61" s="5" t="n">
         <v>0.0509</v>
       </c>
-      <c r="K61" s="5" t="inlineStr"/>
+      <c r="K61" s="5" t="n">
+        <v>0.019</v>
+      </c>
       <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr"/>
       <c r="N61" s="5" t="n">
@@ -4870,7 +4966,9 @@
       <c r="J62" s="5" t="n">
         <v>0.0168</v>
       </c>
-      <c r="K62" s="5" t="inlineStr"/>
+      <c r="K62" s="5" t="n">
+        <v>0.0077</v>
+      </c>
       <c r="L62" s="5" t="inlineStr"/>
       <c r="M62" s="5" t="inlineStr"/>
       <c r="N62" s="5" t="n">
@@ -4927,7 +5025,9 @@
       <c r="J63" s="5" t="n">
         <v>0.055</v>
       </c>
-      <c r="K63" s="5" t="inlineStr"/>
+      <c r="K63" s="5" t="n">
+        <v>0.009900000000000001</v>
+      </c>
       <c r="L63" s="5" t="inlineStr"/>
       <c r="M63" s="5" t="inlineStr"/>
       <c r="N63" s="5" t="n">
@@ -4984,7 +5084,9 @@
       <c r="J64" s="5" t="n">
         <v>0.0178</v>
       </c>
-      <c r="K64" s="5" t="inlineStr"/>
+      <c r="K64" s="5" t="n">
+        <v>0.0214</v>
+      </c>
       <c r="L64" s="5" t="inlineStr"/>
       <c r="M64" s="5" t="inlineStr"/>
       <c r="N64" s="5" t="n">
@@ -5041,7 +5143,9 @@
       <c r="J65" s="5" t="n">
         <v>0.0134</v>
       </c>
-      <c r="K65" s="5" t="inlineStr"/>
+      <c r="K65" s="5" t="n">
+        <v>0.0043</v>
+      </c>
       <c r="L65" s="5" t="inlineStr"/>
       <c r="M65" s="5" t="inlineStr"/>
       <c r="N65" s="5" t="n">
@@ -5098,7 +5202,9 @@
       <c r="J66" s="5" t="n">
         <v>0.0056</v>
       </c>
-      <c r="K66" s="5" t="inlineStr"/>
+      <c r="K66" s="5" t="n">
+        <v>0.0102</v>
+      </c>
       <c r="L66" s="5" t="inlineStr"/>
       <c r="M66" s="5" t="inlineStr"/>
       <c r="N66" s="5" t="n">
@@ -5155,7 +5261,9 @@
       <c r="J67" s="5" t="n">
         <v>0.064</v>
       </c>
-      <c r="K67" s="5" t="inlineStr"/>
+      <c r="K67" s="5" t="n">
+        <v>0.07679999999999999</v>
+      </c>
       <c r="L67" s="5" t="inlineStr"/>
       <c r="M67" s="5" t="inlineStr"/>
       <c r="N67" s="5" t="n">
@@ -5212,7 +5320,9 @@
       <c r="J68" s="5" t="n">
         <v>0.0002</v>
       </c>
-      <c r="K68" s="5" t="inlineStr"/>
+      <c r="K68" s="5" t="n">
+        <v>0.0035</v>
+      </c>
       <c r="L68" s="5" t="inlineStr"/>
       <c r="M68" s="5" t="inlineStr"/>
       <c r="N68" s="5" t="n">
@@ -5269,7 +5379,9 @@
       <c r="J69" s="5" t="n">
         <v>0.0573</v>
       </c>
-      <c r="K69" s="5" t="inlineStr"/>
+      <c r="K69" s="5" t="n">
+        <v>0.0549</v>
+      </c>
       <c r="L69" s="5" t="inlineStr"/>
       <c r="M69" s="5" t="inlineStr"/>
       <c r="N69" s="5" t="n">
@@ -5326,7 +5438,9 @@
       <c r="J70" s="5" t="n">
         <v>0.0294</v>
       </c>
-      <c r="K70" s="5" t="inlineStr"/>
+      <c r="K70" s="5" t="n">
+        <v>0.023</v>
+      </c>
       <c r="L70" s="5" t="inlineStr"/>
       <c r="M70" s="5" t="inlineStr"/>
       <c r="N70" s="5" t="n">
@@ -5514,7 +5628,9 @@
       <c r="E2" s="5" t="n">
         <v>0.1441</v>
       </c>
-      <c r="F2" s="5" t="inlineStr"/>
+      <c r="F2" s="5" t="n">
+        <v>0.1695</v>
+      </c>
       <c r="G2" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5596,7 +5712,9 @@
       <c r="E3" s="5" t="n">
         <v>0.128</v>
       </c>
-      <c r="F3" s="5" t="inlineStr"/>
+      <c r="F3" s="5" t="n">
+        <v>0.078</v>
+      </c>
       <c r="G3" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -5678,7 +5796,9 @@
       <c r="E4" s="5" t="n">
         <v>0.123</v>
       </c>
-      <c r="F4" s="5" t="inlineStr"/>
+      <c r="F4" s="5" t="n">
+        <v>0.1001</v>
+      </c>
       <c r="G4" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -5760,7 +5880,9 @@
       <c r="E5" s="5" t="n">
         <v>0.1492</v>
       </c>
-      <c r="F5" s="5" t="inlineStr"/>
+      <c r="F5" s="5" t="n">
+        <v>0.2117</v>
+      </c>
       <c r="G5" s="5" t="n">
         <v>0.399270575823056</v>
       </c>
@@ -5902,7 +6024,9 @@
       <c r="E7" s="5" t="n">
         <v>0.0292</v>
       </c>
-      <c r="F7" s="5" t="inlineStr"/>
+      <c r="F7" s="5" t="n">
+        <v>0.0415</v>
+      </c>
       <c r="G7" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -5968,7 +6092,9 @@
       <c r="E8" s="5" t="n">
         <v>0.0799</v>
       </c>
-      <c r="F8" s="5" t="inlineStr"/>
+      <c r="F8" s="5" t="n">
+        <v>0.1689</v>
+      </c>
       <c r="G8" s="5" t="n">
         <v>0.529503172508041</v>
       </c>
@@ -6048,7 +6174,9 @@
         <v>0.8903</v>
       </c>
       <c r="E9" s="5" t="inlineStr"/>
-      <c r="F9" s="5" t="inlineStr"/>
+      <c r="F9" s="5" t="n">
+        <v>0.342</v>
+      </c>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
       <c r="I9" s="5" t="inlineStr"/>
@@ -6110,7 +6238,9 @@
       <c r="E10" s="5" t="n">
         <v>0.0833</v>
       </c>
-      <c r="F10" s="5" t="inlineStr"/>
+      <c r="F10" s="5" t="n">
+        <v>0.1175</v>
+      </c>
       <c r="G10" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6302,7 +6432,9 @@
       <c r="E13" s="5" t="n">
         <v>0.3285</v>
       </c>
-      <c r="F13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="n">
+        <v>0.3999</v>
+      </c>
       <c r="G13" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6448,7 +6580,9 @@
       <c r="E15" s="5" t="n">
         <v>0.1353</v>
       </c>
-      <c r="F15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="n">
+        <v>0.2162</v>
+      </c>
       <c r="G15" s="5" t="n">
         <v>0.165388664850326</v>
       </c>
@@ -6514,7 +6648,9 @@
       <c r="E16" s="5" t="n">
         <v>0.1778</v>
       </c>
-      <c r="F16" s="5" t="inlineStr"/>
+      <c r="F16" s="5" t="n">
+        <v>0.2693</v>
+      </c>
       <c r="G16" s="5" t="n">
         <v>0.903607825126104</v>
       </c>
@@ -6596,7 +6732,9 @@
       <c r="E17" s="5" t="n">
         <v>0.2781</v>
       </c>
-      <c r="F17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="n">
+        <v>0.1928</v>
+      </c>
       <c r="G17" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -6662,7 +6800,9 @@
       <c r="E18" s="5" t="n">
         <v>0.1147</v>
       </c>
-      <c r="F18" s="5" t="inlineStr"/>
+      <c r="F18" s="5" t="n">
+        <v>0.3103</v>
+      </c>
       <c r="G18" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -6728,7 +6868,9 @@
       <c r="E19" s="5" t="n">
         <v>0.2801</v>
       </c>
-      <c r="F19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="n">
+        <v>0.2607</v>
+      </c>
       <c r="G19" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -6810,7 +6952,9 @@
       <c r="E20" s="5" t="n">
         <v>0.2431</v>
       </c>
-      <c r="F20" s="5" t="inlineStr"/>
+      <c r="F20" s="5" t="n">
+        <v>0.2125</v>
+      </c>
       <c r="G20" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -6892,7 +7036,9 @@
       <c r="E21" s="5" t="n">
         <v>0.2403</v>
       </c>
-      <c r="F21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="n">
+        <v>0.1922</v>
+      </c>
       <c r="G21" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -6974,7 +7120,9 @@
       <c r="E22" s="5" t="n">
         <v>0.5511</v>
       </c>
-      <c r="F22" s="5" t="inlineStr"/>
+      <c r="F22" s="5" t="n">
+        <v>0.5341</v>
+      </c>
       <c r="G22" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7056,7 +7204,9 @@
       <c r="E23" s="5" t="n">
         <v>0.0614</v>
       </c>
-      <c r="F23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="n">
+        <v>0.1487</v>
+      </c>
       <c r="G23" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7138,7 +7288,9 @@
       <c r="E24" s="5" t="n">
         <v>0.5639</v>
       </c>
-      <c r="F24" s="5" t="inlineStr"/>
+      <c r="F24" s="5" t="n">
+        <v>0.3973</v>
+      </c>
       <c r="G24" s="5" t="n">
         <v>0.919931770355409</v>
       </c>
@@ -7220,7 +7372,9 @@
       <c r="E25" s="5" t="n">
         <v>0.0089</v>
       </c>
-      <c r="F25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="n">
+        <v>0.0169</v>
+      </c>
       <c r="G25" s="5" t="n">
         <v>0.188257195450457</v>
       </c>
@@ -7482,7 +7636,9 @@
       <c r="E29" s="5" t="n">
         <v>0.078</v>
       </c>
-      <c r="F29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="n">
+        <v>0.2905</v>
+      </c>
       <c r="G29" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7564,7 +7720,9 @@
       <c r="E30" s="5" t="n">
         <v>0.125</v>
       </c>
-      <c r="F30" s="5" t="inlineStr"/>
+      <c r="F30" s="5" t="n">
+        <v>0.0318</v>
+      </c>
       <c r="G30" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7646,7 +7804,9 @@
       <c r="E31" s="5" t="n">
         <v>0.1153</v>
       </c>
-      <c r="F31" s="5" t="inlineStr"/>
+      <c r="F31" s="5" t="n">
+        <v>0.036</v>
+      </c>
       <c r="G31" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -7728,7 +7888,9 @@
       <c r="E32" s="5" t="n">
         <v>0.0388</v>
       </c>
-      <c r="F32" s="5" t="inlineStr"/>
+      <c r="F32" s="5" t="n">
+        <v>0.2983</v>
+      </c>
       <c r="G32" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -7810,7 +7972,9 @@
       <c r="E33" s="5" t="n">
         <v>0.2694</v>
       </c>
-      <c r="F33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="n">
+        <v>0.2848</v>
+      </c>
       <c r="G33" s="5" t="n">
         <v>0.87127903942823</v>
       </c>
@@ -7996,7 +8160,9 @@
       <c r="E36" s="5" t="n">
         <v>0.1146</v>
       </c>
-      <c r="F36" s="5" t="inlineStr"/>
+      <c r="F36" s="5" t="n">
+        <v>0.0936</v>
+      </c>
       <c r="G36" s="5" t="n">
         <v>0.505349468159863</v>
       </c>
@@ -8078,7 +8244,9 @@
       <c r="E37" s="5" t="n">
         <v>0.2365</v>
       </c>
-      <c r="F37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="n">
+        <v>0.2465</v>
+      </c>
       <c r="G37" s="5" t="n">
         <v>0.1571570475144</v>
       </c>
@@ -8222,7 +8390,9 @@
         <v>0.9427</v>
       </c>
       <c r="E39" s="5" t="inlineStr"/>
-      <c r="F39" s="5" t="inlineStr"/>
+      <c r="F39" s="5" t="n">
+        <v>0.08939999999999999</v>
+      </c>
       <c r="G39" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -8302,7 +8472,9 @@
         <v>0.9427</v>
       </c>
       <c r="E40" s="5" t="inlineStr"/>
-      <c r="F40" s="5" t="inlineStr"/>
+      <c r="F40" s="5" t="n">
+        <v>0.0813</v>
+      </c>
       <c r="G40" s="5" t="n">
         <v>0.636442356808484</v>
       </c>
@@ -8384,7 +8556,9 @@
       <c r="E41" s="5" t="n">
         <v>0.1167</v>
       </c>
-      <c r="F41" s="5" t="inlineStr"/>
+      <c r="F41" s="5" t="n">
+        <v>0.2803</v>
+      </c>
       <c r="G41" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8466,7 +8640,9 @@
       <c r="E42" s="5" t="n">
         <v>0.2501</v>
       </c>
-      <c r="F42" s="5" t="inlineStr"/>
+      <c r="F42" s="5" t="n">
+        <v>0.2261</v>
+      </c>
       <c r="G42" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8546,7 +8722,9 @@
         <v>0.8908</v>
       </c>
       <c r="E43" s="5" t="inlineStr"/>
-      <c r="F43" s="5" t="inlineStr"/>
+      <c r="F43" s="5" t="n">
+        <v>0.2674</v>
+      </c>
       <c r="G43" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8610,7 +8788,9 @@
         <v>0.8894</v>
       </c>
       <c r="E44" s="5" t="inlineStr"/>
-      <c r="F44" s="5" t="inlineStr"/>
+      <c r="F44" s="5" t="n">
+        <v>0.2715</v>
+      </c>
       <c r="G44" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -8676,7 +8856,9 @@
       <c r="E45" s="5" t="n">
         <v>0.0616</v>
       </c>
-      <c r="F45" s="5" t="inlineStr"/>
+      <c r="F45" s="5" t="n">
+        <v>0.0283</v>
+      </c>
       <c r="G45" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8758,7 +8940,9 @@
       <c r="E46" s="5" t="n">
         <v>0.0306</v>
       </c>
-      <c r="F46" s="5" t="inlineStr"/>
+      <c r="F46" s="5" t="n">
+        <v>0.081</v>
+      </c>
       <c r="G46" s="5" t="n">
         <v>0.15663609258386</v>
       </c>
@@ -8840,7 +9024,9 @@
       <c r="E47" s="5" t="n">
         <v>0.1883</v>
       </c>
-      <c r="F47" s="5" t="inlineStr"/>
+      <c r="F47" s="5" t="n">
+        <v>0.1353</v>
+      </c>
       <c r="G47" s="5" t="n">
         <v>0.64186785726147</v>
       </c>
@@ -8906,7 +9092,9 @@
       <c r="E48" s="5" t="n">
         <v>0.06469999999999999</v>
       </c>
-      <c r="F48" s="5" t="inlineStr"/>
+      <c r="F48" s="5" t="n">
+        <v>0.0301</v>
+      </c>
       <c r="G48" s="5" t="n">
         <v>0.231026075027885</v>
       </c>
@@ -8986,7 +9174,9 @@
         <v>0.955</v>
       </c>
       <c r="E49" s="5" t="inlineStr"/>
-      <c r="F49" s="5" t="inlineStr"/>
+      <c r="F49" s="5" t="n">
+        <v>0.0216</v>
+      </c>
       <c r="G49" s="5" t="n">
         <v>0.158699742317549</v>
       </c>
@@ -9052,7 +9242,9 @@
       <c r="E50" s="5" t="n">
         <v>0.1969</v>
       </c>
-      <c r="F50" s="5" t="inlineStr"/>
+      <c r="F50" s="5" t="n">
+        <v>0.1655</v>
+      </c>
       <c r="G50" s="5" t="n">
         <v>0.5859908275658871</v>
       </c>
@@ -9118,7 +9310,9 @@
       <c r="E51" s="5" t="n">
         <v>0.0528</v>
       </c>
-      <c r="F51" s="5" t="inlineStr"/>
+      <c r="F51" s="5" t="n">
+        <v>0.0629</v>
+      </c>
       <c r="G51" s="5" t="inlineStr"/>
       <c r="H51" s="5" t="inlineStr"/>
       <c r="I51" s="5" t="inlineStr"/>
@@ -9180,7 +9374,9 @@
       <c r="E52" s="5" t="n">
         <v>0.1308</v>
       </c>
-      <c r="F52" s="5" t="inlineStr"/>
+      <c r="F52" s="5" t="n">
+        <v>0.1312</v>
+      </c>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr"/>
@@ -9242,7 +9438,9 @@
       <c r="E53" s="5" t="n">
         <v>0.0143</v>
       </c>
-      <c r="F53" s="5" t="inlineStr"/>
+      <c r="F53" s="5" t="n">
+        <v>0.0042</v>
+      </c>
       <c r="G53" s="5" t="inlineStr"/>
       <c r="H53" s="5" t="inlineStr"/>
       <c r="I53" s="5" t="inlineStr"/>
@@ -9304,7 +9502,9 @@
       <c r="E54" s="5" t="n">
         <v>0.0265</v>
       </c>
-      <c r="F54" s="5" t="inlineStr"/>
+      <c r="F54" s="5" t="n">
+        <v>0.0185</v>
+      </c>
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="5" t="inlineStr"/>
@@ -9426,7 +9626,9 @@
       <c r="E56" s="5" t="n">
         <v>0.0066</v>
       </c>
-      <c r="F56" s="5" t="inlineStr"/>
+      <c r="F56" s="5" t="n">
+        <v>0.0089</v>
+      </c>
       <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="5" t="inlineStr"/>
@@ -9486,7 +9688,9 @@
         <v>0.9644</v>
       </c>
       <c r="E57" s="5" t="inlineStr"/>
-      <c r="F57" s="5" t="inlineStr"/>
+      <c r="F57" s="5" t="n">
+        <v>0.0144</v>
+      </c>
       <c r="G57" s="5" t="inlineStr"/>
       <c r="H57" s="5" t="inlineStr"/>
       <c r="I57" s="5" t="inlineStr"/>
@@ -9546,7 +9750,9 @@
         <v>0.9641999999999999</v>
       </c>
       <c r="E58" s="5" t="inlineStr"/>
-      <c r="F58" s="5" t="inlineStr"/>
+      <c r="F58" s="5" t="n">
+        <v>0.0219</v>
+      </c>
       <c r="G58" s="5" t="inlineStr"/>
       <c r="H58" s="5" t="inlineStr"/>
       <c r="I58" s="5" t="inlineStr"/>
@@ -9608,7 +9814,9 @@
       <c r="E59" s="5" t="n">
         <v>0.0298</v>
       </c>
-      <c r="F59" s="5" t="inlineStr"/>
+      <c r="F59" s="5" t="n">
+        <v>0.0184</v>
+      </c>
       <c r="G59" s="5" t="inlineStr"/>
       <c r="H59" s="5" t="inlineStr"/>
       <c r="I59" s="5" t="inlineStr"/>
@@ -9730,7 +9938,9 @@
       <c r="E61" s="5" t="n">
         <v>0.0509</v>
       </c>
-      <c r="F61" s="5" t="inlineStr"/>
+      <c r="F61" s="5" t="n">
+        <v>0.019</v>
+      </c>
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr"/>
       <c r="I61" s="5" t="inlineStr"/>
@@ -9792,7 +10002,9 @@
       <c r="E62" s="5" t="n">
         <v>0.0168</v>
       </c>
-      <c r="F62" s="5" t="inlineStr"/>
+      <c r="F62" s="5" t="n">
+        <v>0.0077</v>
+      </c>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr"/>
       <c r="I62" s="5" t="inlineStr"/>
@@ -9854,7 +10066,9 @@
       <c r="E63" s="5" t="n">
         <v>0.055</v>
       </c>
-      <c r="F63" s="5" t="inlineStr"/>
+      <c r="F63" s="5" t="n">
+        <v>0.009900000000000001</v>
+      </c>
       <c r="G63" s="5" t="inlineStr"/>
       <c r="H63" s="5" t="inlineStr"/>
       <c r="I63" s="5" t="inlineStr"/>
@@ -9916,7 +10130,9 @@
       <c r="E64" s="5" t="n">
         <v>0.0178</v>
       </c>
-      <c r="F64" s="5" t="inlineStr"/>
+      <c r="F64" s="5" t="n">
+        <v>0.0214</v>
+      </c>
       <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr"/>
       <c r="I64" s="5" t="inlineStr"/>
@@ -9978,7 +10194,9 @@
       <c r="E65" s="5" t="n">
         <v>0.0134</v>
       </c>
-      <c r="F65" s="5" t="inlineStr"/>
+      <c r="F65" s="5" t="n">
+        <v>0.0043</v>
+      </c>
       <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr"/>
       <c r="I65" s="5" t="inlineStr"/>
@@ -10040,7 +10258,9 @@
       <c r="E66" s="5" t="n">
         <v>0.0056</v>
       </c>
-      <c r="F66" s="5" t="inlineStr"/>
+      <c r="F66" s="5" t="n">
+        <v>0.0102</v>
+      </c>
       <c r="G66" s="5" t="inlineStr"/>
       <c r="H66" s="5" t="inlineStr"/>
       <c r="I66" s="5" t="inlineStr"/>
@@ -10102,7 +10322,9 @@
       <c r="E67" s="5" t="n">
         <v>0.064</v>
       </c>
-      <c r="F67" s="5" t="inlineStr"/>
+      <c r="F67" s="5" t="n">
+        <v>0.07679999999999999</v>
+      </c>
       <c r="G67" s="5" t="inlineStr"/>
       <c r="H67" s="5" t="inlineStr"/>
       <c r="I67" s="5" t="inlineStr"/>
@@ -10164,7 +10386,9 @@
       <c r="E68" s="5" t="n">
         <v>0.0002</v>
       </c>
-      <c r="F68" s="5" t="inlineStr"/>
+      <c r="F68" s="5" t="n">
+        <v>0.0035</v>
+      </c>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr"/>
       <c r="I68" s="5" t="inlineStr"/>
@@ -10226,7 +10450,9 @@
       <c r="E69" s="5" t="n">
         <v>0.0573</v>
       </c>
-      <c r="F69" s="5" t="inlineStr"/>
+      <c r="F69" s="5" t="n">
+        <v>0.0549</v>
+      </c>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr"/>
       <c r="I69" s="5" t="inlineStr"/>
@@ -10288,7 +10514,9 @@
       <c r="E70" s="5" t="n">
         <v>0.0294</v>
       </c>
-      <c r="F70" s="5" t="inlineStr"/>
+      <c r="F70" s="5" t="n">
+        <v>0.023</v>
+      </c>
       <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr"/>
       <c r="I70" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update renewable generator dashboard data 2026-10
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -644,10 +644,10 @@
         <v>132</v>
       </c>
       <c r="J2" s="5" t="n">
-        <v>0.1441</v>
+        <v>0.1499</v>
       </c>
       <c r="K2" s="5" t="n">
-        <v>0.1695</v>
+        <v>0.2043</v>
       </c>
       <c r="L2" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -729,10 +729,10 @@
         <v>66</v>
       </c>
       <c r="J3" s="5" t="n">
-        <v>0.128</v>
+        <v>0.1357</v>
       </c>
       <c r="K3" s="5" t="n">
-        <v>0.078</v>
+        <v>0.0837</v>
       </c>
       <c r="L3" s="5" t="n">
         <v>0.636442356808484</v>
@@ -814,10 +814,10 @@
         <v>132</v>
       </c>
       <c r="J4" s="5" t="n">
-        <v>0.123</v>
+        <v>0.1299</v>
       </c>
       <c r="K4" s="5" t="n">
-        <v>0.1001</v>
+        <v>0.1043</v>
       </c>
       <c r="L4" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -899,10 +899,10 @@
         <v>22</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.1492</v>
+        <v>0.1569</v>
       </c>
       <c r="K5" s="5" t="n">
-        <v>0.2117</v>
+        <v>0.2455</v>
       </c>
       <c r="L5" s="5" t="n">
         <v>0.399270575823056</v>
@@ -1039,10 +1039,10 @@
         <v>132</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.0292</v>
+        <v>0.0296</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>0.0415</v>
+        <v>0.0419</v>
       </c>
       <c r="L7" s="5" t="n">
         <v>0.64186785726147</v>
@@ -1108,10 +1108,10 @@
         <v>132</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.0799</v>
+        <v>0.0827</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>0.1689</v>
+        <v>0.2172</v>
       </c>
       <c r="L8" s="5" t="n">
         <v>0.529503172508041</v>
@@ -1188,7 +1188,7 @@
       <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr"/>
       <c r="K9" s="5" t="n">
-        <v>0.342</v>
+        <v>0.4061</v>
       </c>
       <c r="L9" s="5" t="inlineStr"/>
       <c r="M9" s="5" t="inlineStr"/>
@@ -1250,10 +1250,10 @@
         <v>132</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.0833</v>
+        <v>0.0882</v>
       </c>
       <c r="K10" s="5" t="n">
-        <v>0.1175</v>
+        <v>0.126</v>
       </c>
       <c r="L10" s="5" t="n">
         <v>0.64186785726147</v>
@@ -1319,7 +1319,7 @@
         <v>132</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.0762</v>
+        <v>0.0806</v>
       </c>
       <c r="K11" s="5" t="inlineStr"/>
       <c r="L11" s="5" t="n">
@@ -1441,10 +1441,10 @@
         <v>66</v>
       </c>
       <c r="J13" s="5" t="n">
-        <v>0.3285</v>
+        <v>0.3634</v>
       </c>
       <c r="K13" s="5" t="n">
-        <v>0.3999</v>
+        <v>0.469</v>
       </c>
       <c r="L13" s="5" t="n">
         <v>0.87127903942823</v>
@@ -1591,10 +1591,10 @@
         <v>330</v>
       </c>
       <c r="J15" s="5" t="n">
-        <v>0.1353</v>
+        <v>0.1456</v>
       </c>
       <c r="K15" s="5" t="n">
-        <v>0.2162</v>
+        <v>0.2826</v>
       </c>
       <c r="L15" s="5" t="n">
         <v>0.165388664850326</v>
@@ -1660,10 +1660,10 @@
         <v>132</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>0.1778</v>
+        <v>0.1888</v>
       </c>
       <c r="K16" s="5" t="n">
-        <v>0.2693</v>
+        <v>0.3026</v>
       </c>
       <c r="L16" s="5" t="n">
         <v>0.903607825126104</v>
@@ -1745,10 +1745,10 @@
         <v>132</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>0.2781</v>
+        <v>0.3083</v>
       </c>
       <c r="K17" s="5" t="n">
-        <v>0.1928</v>
+        <v>0.2523</v>
       </c>
       <c r="L17" s="5" t="n">
         <v>0.64186785726147</v>
@@ -1814,10 +1814,10 @@
         <v>66</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>0.1147</v>
+        <v>0.119</v>
       </c>
       <c r="K18" s="5" t="n">
-        <v>0.3103</v>
+        <v>0.3509</v>
       </c>
       <c r="L18" s="5" t="n">
         <v>0.87127903942823</v>
@@ -1883,10 +1883,10 @@
         <v>132</v>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0.2801</v>
+        <v>0.297</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>0.2607</v>
+        <v>0.302</v>
       </c>
       <c r="L19" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -1968,10 +1968,10 @@
         <v>220</v>
       </c>
       <c r="J20" s="5" t="n">
-        <v>0.2431</v>
+        <v>0.2549</v>
       </c>
       <c r="K20" s="5" t="n">
-        <v>0.2125</v>
+        <v>0.2348</v>
       </c>
       <c r="L20" s="5" t="n">
         <v>0.505349468159863</v>
@@ -2053,10 +2053,10 @@
         <v>22</v>
       </c>
       <c r="J21" s="5" t="n">
-        <v>0.2403</v>
+        <v>0.254</v>
       </c>
       <c r="K21" s="5" t="n">
-        <v>0.1922</v>
+        <v>0.2107</v>
       </c>
       <c r="L21" s="5" t="n">
         <v>0.505349468159863</v>
@@ -2138,10 +2138,10 @@
         <v>132</v>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0.5511</v>
+        <v>0.6709000000000001</v>
       </c>
       <c r="K22" s="5" t="n">
-        <v>0.5341</v>
+        <v>0.673</v>
       </c>
       <c r="L22" s="5" t="n">
         <v>0.919931770355409</v>
@@ -2223,10 +2223,10 @@
         <v>132</v>
       </c>
       <c r="J23" s="5" t="n">
-        <v>0.0614</v>
+        <v>0.0711</v>
       </c>
       <c r="K23" s="5" t="n">
-        <v>0.1487</v>
+        <v>0.1724</v>
       </c>
       <c r="L23" s="5" t="n">
         <v>0.231026075027885</v>
@@ -2308,10 +2308,10 @@
         <v>66</v>
       </c>
       <c r="J24" s="5" t="n">
-        <v>0.5639</v>
+        <v>0.6756</v>
       </c>
       <c r="K24" s="5" t="n">
-        <v>0.3973</v>
+        <v>0.4942</v>
       </c>
       <c r="L24" s="5" t="n">
         <v>0.919931770355409</v>
@@ -2393,7 +2393,7 @@
         <v>66</v>
       </c>
       <c r="J25" s="5" t="n">
-        <v>0.0089</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="K25" s="5" t="n">
         <v>0.0169</v>
@@ -2649,10 +2649,10 @@
         <v>132</v>
       </c>
       <c r="J29" s="5" t="n">
-        <v>0.078</v>
+        <v>0.0799</v>
       </c>
       <c r="K29" s="5" t="n">
-        <v>0.2905</v>
+        <v>0.3181</v>
       </c>
       <c r="L29" s="5" t="n">
         <v>0.15663609258386</v>
@@ -2734,10 +2734,10 @@
         <v>330</v>
       </c>
       <c r="J30" s="5" t="n">
-        <v>0.125</v>
+        <v>0.14</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>0.0318</v>
+        <v>0.0323</v>
       </c>
       <c r="L30" s="5" t="n">
         <v>0.231026075027885</v>
@@ -2819,10 +2819,10 @@
         <v>330</v>
       </c>
       <c r="J31" s="5" t="n">
-        <v>0.1153</v>
+        <v>0.1269</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>0.036</v>
+        <v>0.0365</v>
       </c>
       <c r="L31" s="5" t="n">
         <v>0.231026075027885</v>
@@ -2904,10 +2904,10 @@
         <v>132</v>
       </c>
       <c r="J32" s="5" t="n">
-        <v>0.0388</v>
+        <v>0.0393</v>
       </c>
       <c r="K32" s="5" t="n">
-        <v>0.2983</v>
+        <v>0.3484</v>
       </c>
       <c r="L32" s="5" t="n">
         <v>0.15663609258386</v>
@@ -2989,10 +2989,10 @@
         <v>66</v>
       </c>
       <c r="J33" s="5" t="n">
-        <v>0.2694</v>
+        <v>0.304</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>0.2848</v>
+        <v>0.326</v>
       </c>
       <c r="L33" s="5" t="n">
         <v>0.87127903942823</v>
@@ -3168,10 +3168,10 @@
         <v>220</v>
       </c>
       <c r="J36" s="5" t="n">
-        <v>0.1146</v>
+        <v>0.1174</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>0.0936</v>
+        <v>0.0941</v>
       </c>
       <c r="L36" s="5" t="n">
         <v>0.505349468159863</v>
@@ -3253,10 +3253,10 @@
         <v>132</v>
       </c>
       <c r="J37" s="5" t="n">
-        <v>0.2365</v>
+        <v>0.2596</v>
       </c>
       <c r="K37" s="5" t="n">
-        <v>0.2465</v>
+        <v>0.2874</v>
       </c>
       <c r="L37" s="5" t="n">
         <v>0.1571570475144</v>
@@ -3404,7 +3404,7 @@
       </c>
       <c r="J39" s="5" t="inlineStr"/>
       <c r="K39" s="5" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.099</v>
       </c>
       <c r="L39" s="5" t="n">
         <v>0.636442356808484</v>
@@ -3487,7 +3487,7 @@
       </c>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="5" t="n">
-        <v>0.0813</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="L40" s="5" t="n">
         <v>0.636442356808484</v>
@@ -3569,10 +3569,10 @@
         <v>132</v>
       </c>
       <c r="J41" s="5" t="n">
-        <v>0.1167</v>
+        <v>0.1216</v>
       </c>
       <c r="K41" s="5" t="n">
-        <v>0.2803</v>
+        <v>0.3194</v>
       </c>
       <c r="L41" s="5" t="n">
         <v>0.15663609258386</v>
@@ -3654,10 +3654,10 @@
         <v>66</v>
       </c>
       <c r="J42" s="5" t="n">
-        <v>0.2501</v>
+        <v>0.2655</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>0.2261</v>
+        <v>0.2642</v>
       </c>
       <c r="L42" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -3740,7 +3740,7 @@
       </c>
       <c r="J43" s="5" t="inlineStr"/>
       <c r="K43" s="5" t="n">
-        <v>0.2674</v>
+        <v>0.3035</v>
       </c>
       <c r="L43" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -3807,7 +3807,7 @@
       </c>
       <c r="J44" s="5" t="inlineStr"/>
       <c r="K44" s="5" t="n">
-        <v>0.2715</v>
+        <v>0.3103</v>
       </c>
       <c r="L44" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -3873,10 +3873,10 @@
         <v>330</v>
       </c>
       <c r="J45" s="5" t="n">
-        <v>0.0616</v>
+        <v>0.06569999999999999</v>
       </c>
       <c r="K45" s="5" t="n">
-        <v>0.0283</v>
+        <v>0.0285</v>
       </c>
       <c r="L45" s="5" t="n">
         <v>0.15663609258386</v>
@@ -3958,10 +3958,10 @@
         <v>132</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>0.0306</v>
+        <v>0.0317</v>
       </c>
       <c r="K46" s="5" t="n">
-        <v>0.081</v>
+        <v>0.0929</v>
       </c>
       <c r="L46" s="5" t="n">
         <v>0.15663609258386</v>
@@ -4043,10 +4043,10 @@
         <v>132</v>
       </c>
       <c r="J47" s="5" t="n">
-        <v>0.1883</v>
+        <v>0.1993</v>
       </c>
       <c r="K47" s="5" t="n">
-        <v>0.1353</v>
+        <v>0.1422</v>
       </c>
       <c r="L47" s="5" t="n">
         <v>0.64186785726147</v>
@@ -4112,10 +4112,10 @@
         <v>132</v>
       </c>
       <c r="J48" s="5" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.0653</v>
       </c>
       <c r="K48" s="5" t="n">
-        <v>0.0301</v>
+        <v>0.0303</v>
       </c>
       <c r="L48" s="5" t="n">
         <v>0.231026075027885</v>
@@ -4198,7 +4198,7 @@
       </c>
       <c r="J49" s="5" t="inlineStr"/>
       <c r="K49" s="5" t="n">
-        <v>0.0216</v>
+        <v>0.0219</v>
       </c>
       <c r="L49" s="5" t="n">
         <v>0.158699742317549</v>
@@ -4264,10 +4264,10 @@
         <v>132</v>
       </c>
       <c r="J50" s="5" t="n">
-        <v>0.1969</v>
+        <v>0.2072</v>
       </c>
       <c r="K50" s="5" t="n">
-        <v>0.1655</v>
+        <v>0.1731</v>
       </c>
       <c r="L50" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -4327,10 +4327,10 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="5" t="n">
-        <v>0.0528</v>
+        <v>0.0554</v>
       </c>
       <c r="K51" s="5" t="n">
-        <v>0.0629</v>
+        <v>0.0665</v>
       </c>
       <c r="L51" s="5" t="inlineStr"/>
       <c r="M51" s="5" t="inlineStr"/>
@@ -4386,10 +4386,10 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="5" t="n">
-        <v>0.1308</v>
+        <v>0.1371</v>
       </c>
       <c r="K52" s="5" t="n">
-        <v>0.1312</v>
+        <v>0.1505</v>
       </c>
       <c r="L52" s="5" t="inlineStr"/>
       <c r="M52" s="5" t="inlineStr"/>
@@ -4445,10 +4445,10 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="5" t="n">
-        <v>0.0143</v>
+        <v>0.0145</v>
       </c>
       <c r="K53" s="5" t="n">
-        <v>0.0042</v>
+        <v>0.0037</v>
       </c>
       <c r="L53" s="5" t="inlineStr"/>
       <c r="M53" s="5" t="inlineStr"/>
@@ -4504,10 +4504,10 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="5" t="n">
-        <v>0.0265</v>
+        <v>0.0266</v>
       </c>
       <c r="K54" s="5" t="n">
-        <v>0.0185</v>
+        <v>0.0182</v>
       </c>
       <c r="L54" s="5" t="inlineStr"/>
       <c r="M54" s="5" t="inlineStr"/>
@@ -4618,10 +4618,10 @@
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="5" t="n">
-        <v>0.0066</v>
+        <v>0.0067</v>
       </c>
       <c r="K56" s="5" t="n">
-        <v>0.0089</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="L56" s="5" t="inlineStr"/>
       <c r="M56" s="5" t="inlineStr"/>
@@ -4678,7 +4678,7 @@
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="5" t="inlineStr"/>
       <c r="K57" s="5" t="n">
-        <v>0.0144</v>
+        <v>0.0146</v>
       </c>
       <c r="L57" s="5" t="inlineStr"/>
       <c r="M57" s="5" t="inlineStr"/>
@@ -4735,7 +4735,7 @@
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr"/>
       <c r="K58" s="5" t="n">
-        <v>0.0219</v>
+        <v>0.0221</v>
       </c>
       <c r="L58" s="5" t="inlineStr"/>
       <c r="M58" s="5" t="inlineStr"/>
@@ -4791,10 +4791,10 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="5" t="n">
-        <v>0.0298</v>
+        <v>0.0311</v>
       </c>
       <c r="K59" s="5" t="n">
-        <v>0.0184</v>
+        <v>0.0188</v>
       </c>
       <c r="L59" s="5" t="inlineStr"/>
       <c r="M59" s="5" t="inlineStr"/>
@@ -4905,10 +4905,10 @@
       </c>
       <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="5" t="n">
-        <v>0.0509</v>
+        <v>0.052</v>
       </c>
       <c r="K61" s="5" t="n">
-        <v>0.019</v>
+        <v>0.0195</v>
       </c>
       <c r="L61" s="5" t="inlineStr"/>
       <c r="M61" s="5" t="inlineStr"/>
@@ -4964,10 +4964,10 @@
       </c>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="5" t="n">
-        <v>0.0168</v>
+        <v>0.0171</v>
       </c>
       <c r="K62" s="5" t="n">
-        <v>0.0077</v>
+        <v>0.0076</v>
       </c>
       <c r="L62" s="5" t="inlineStr"/>
       <c r="M62" s="5" t="inlineStr"/>
@@ -5023,10 +5023,10 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="5" t="n">
-        <v>0.055</v>
+        <v>0.0574</v>
       </c>
       <c r="K63" s="5" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="L63" s="5" t="inlineStr"/>
       <c r="M63" s="5" t="inlineStr"/>
@@ -5082,10 +5082,10 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="5" t="n">
-        <v>0.0178</v>
+        <v>0.018</v>
       </c>
       <c r="K64" s="5" t="n">
-        <v>0.0214</v>
+        <v>0.0217</v>
       </c>
       <c r="L64" s="5" t="inlineStr"/>
       <c r="M64" s="5" t="inlineStr"/>
@@ -5141,10 +5141,10 @@
       </c>
       <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="5" t="n">
-        <v>0.0134</v>
+        <v>0.0136</v>
       </c>
       <c r="K65" s="5" t="n">
-        <v>0.0043</v>
+        <v>0.004</v>
       </c>
       <c r="L65" s="5" t="inlineStr"/>
       <c r="M65" s="5" t="inlineStr"/>
@@ -5200,10 +5200,10 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="5" t="n">
-        <v>0.0056</v>
+        <v>0.0057</v>
       </c>
       <c r="K66" s="5" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="L66" s="5" t="inlineStr"/>
       <c r="M66" s="5" t="inlineStr"/>
@@ -5259,10 +5259,10 @@
       </c>
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="5" t="n">
-        <v>0.064</v>
+        <v>0.0655</v>
       </c>
       <c r="K67" s="5" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.0804</v>
       </c>
       <c r="L67" s="5" t="inlineStr"/>
       <c r="M67" s="5" t="inlineStr"/>
@@ -5321,7 +5321,7 @@
         <v>0.0002</v>
       </c>
       <c r="K68" s="5" t="n">
-        <v>0.0035</v>
+        <v>0.0034</v>
       </c>
       <c r="L68" s="5" t="inlineStr"/>
       <c r="M68" s="5" t="inlineStr"/>
@@ -5377,10 +5377,10 @@
       </c>
       <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="5" t="n">
-        <v>0.0573</v>
+        <v>0.0579</v>
       </c>
       <c r="K69" s="5" t="n">
-        <v>0.0549</v>
+        <v>0.0601</v>
       </c>
       <c r="L69" s="5" t="inlineStr"/>
       <c r="M69" s="5" t="inlineStr"/>
@@ -5436,10 +5436,10 @@
       </c>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="5" t="n">
-        <v>0.0294</v>
+        <v>0.0304</v>
       </c>
       <c r="K70" s="5" t="n">
-        <v>0.023</v>
+        <v>0.0235</v>
       </c>
       <c r="L70" s="5" t="inlineStr"/>
       <c r="M70" s="5" t="inlineStr"/>
@@ -5626,10 +5626,10 @@
         <v>0.8395</v>
       </c>
       <c r="E2" s="5" t="n">
-        <v>0.1441</v>
+        <v>0.1499</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.1695</v>
+        <v>0.2043</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -5710,10 +5710,10 @@
         <v>0.9245</v>
       </c>
       <c r="E3" s="5" t="n">
-        <v>0.128</v>
+        <v>0.1357</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.078</v>
+        <v>0.0837</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>0.636442356808484</v>
@@ -5794,10 +5794,10 @@
         <v>0.8823</v>
       </c>
       <c r="E4" s="5" t="n">
-        <v>0.123</v>
+        <v>0.1299</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.1001</v>
+        <v>0.1043</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -5878,10 +5878,10 @@
         <v>0.8436</v>
       </c>
       <c r="E5" s="5" t="n">
-        <v>0.1492</v>
+        <v>0.1569</v>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0.2117</v>
+        <v>0.2455</v>
       </c>
       <c r="G5" s="5" t="n">
         <v>0.399270575823056</v>
@@ -6022,10 +6022,10 @@
         <v>0.8416</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.0292</v>
+        <v>0.0296</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>0.0415</v>
+        <v>0.0419</v>
       </c>
       <c r="G7" s="5" t="n">
         <v>0.64186785726147</v>
@@ -6090,10 +6090,10 @@
         <v>0.8899</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0799</v>
+        <v>0.0827</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.1689</v>
+        <v>0.2172</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0.529503172508041</v>
@@ -6175,7 +6175,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="n">
-        <v>0.342</v>
+        <v>0.4061</v>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
@@ -6236,10 +6236,10 @@
         <v>0.8554</v>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0.0833</v>
+        <v>0.0882</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0.1175</v>
+        <v>0.126</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>0.64186785726147</v>
@@ -6304,7 +6304,7 @@
         <v>0.8521</v>
       </c>
       <c r="E11" s="5" t="n">
-        <v>0.0762</v>
+        <v>0.0806</v>
       </c>
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="n">
@@ -6430,10 +6430,10 @@
         <v>0.8918</v>
       </c>
       <c r="E13" s="5" t="n">
-        <v>0.3285</v>
+        <v>0.3634</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.3999</v>
+        <v>0.469</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0.87127903942823</v>
@@ -6578,10 +6578,10 @@
         <v>0.9635</v>
       </c>
       <c r="E15" s="5" t="n">
-        <v>0.1353</v>
+        <v>0.1456</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.2162</v>
+        <v>0.2826</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>0.165388664850326</v>
@@ -6646,10 +6646,10 @@
         <v>0.8463000000000001</v>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0.1778</v>
+        <v>0.1888</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.2693</v>
+        <v>0.3026</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>0.903607825126104</v>
@@ -6730,10 +6730,10 @@
         <v>0.8652</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>0.2781</v>
+        <v>0.3083</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.1928</v>
+        <v>0.2523</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>0.64186785726147</v>
@@ -6798,10 +6798,10 @@
         <v>0.8962</v>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.1147</v>
+        <v>0.119</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.3103</v>
+        <v>0.3509</v>
       </c>
       <c r="G18" s="5" t="n">
         <v>0.87127903942823</v>
@@ -6866,10 +6866,10 @@
         <v>0.8865</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0.2801</v>
+        <v>0.297</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.2607</v>
+        <v>0.302</v>
       </c>
       <c r="G19" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -6950,10 +6950,10 @@
         <v>0.8206</v>
       </c>
       <c r="E20" s="5" t="n">
-        <v>0.2431</v>
+        <v>0.2549</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.2125</v>
+        <v>0.2348</v>
       </c>
       <c r="G20" s="5" t="n">
         <v>0.505349468159863</v>
@@ -7034,10 +7034,10 @@
         <v>0.8268</v>
       </c>
       <c r="E21" s="5" t="n">
-        <v>0.2403</v>
+        <v>0.254</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.1922</v>
+        <v>0.2107</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>0.505349468159863</v>
@@ -7118,10 +7118,10 @@
         <v>0.9482</v>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.5511</v>
+        <v>0.6709000000000001</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.5341</v>
+        <v>0.673</v>
       </c>
       <c r="G22" s="5" t="n">
         <v>0.919931770355409</v>
@@ -7202,10 +7202,10 @@
         <v>0.8657</v>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.0614</v>
+        <v>0.0711</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.1487</v>
+        <v>0.1724</v>
       </c>
       <c r="G23" s="5" t="n">
         <v>0.231026075027885</v>
@@ -7286,10 +7286,10 @@
         <v>0.9583</v>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.5639</v>
+        <v>0.6756</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.3973</v>
+        <v>0.4942</v>
       </c>
       <c r="G24" s="5" t="n">
         <v>0.919931770355409</v>
@@ -7370,7 +7370,7 @@
         <v>0.8509</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.0089</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="F25" s="5" t="n">
         <v>0.0169</v>
@@ -7634,10 +7634,10 @@
         <v>0.9273</v>
       </c>
       <c r="E29" s="5" t="n">
-        <v>0.078</v>
+        <v>0.0799</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.2905</v>
+        <v>0.3181</v>
       </c>
       <c r="G29" s="5" t="n">
         <v>0.15663609258386</v>
@@ -7718,10 +7718,10 @@
         <v>0.8911</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.125</v>
+        <v>0.14</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.0318</v>
+        <v>0.0323</v>
       </c>
       <c r="G30" s="5" t="n">
         <v>0.231026075027885</v>
@@ -7802,10 +7802,10 @@
         <v>0.8911</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.1153</v>
+        <v>0.1269</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.036</v>
+        <v>0.0365</v>
       </c>
       <c r="G31" s="5" t="n">
         <v>0.231026075027885</v>
@@ -7886,10 +7886,10 @@
         <v>0.9699</v>
       </c>
       <c r="E32" s="5" t="n">
-        <v>0.0388</v>
+        <v>0.0393</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.2983</v>
+        <v>0.3484</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>0.15663609258386</v>
@@ -7970,10 +7970,10 @@
         <v>0.8918</v>
       </c>
       <c r="E33" s="5" t="n">
-        <v>0.2694</v>
+        <v>0.304</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.2848</v>
+        <v>0.326</v>
       </c>
       <c r="G33" s="5" t="n">
         <v>0.87127903942823</v>
@@ -8158,10 +8158,10 @@
         <v>0.8218</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.1146</v>
+        <v>0.1174</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.0936</v>
+        <v>0.0941</v>
       </c>
       <c r="G36" s="5" t="n">
         <v>0.505349468159863</v>
@@ -8242,10 +8242,10 @@
         <v>0.8865</v>
       </c>
       <c r="E37" s="5" t="n">
-        <v>0.2365</v>
+        <v>0.2596</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.2465</v>
+        <v>0.2874</v>
       </c>
       <c r="G37" s="5" t="n">
         <v>0.1571570475144</v>
@@ -8391,7 +8391,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr"/>
       <c r="F39" s="5" t="n">
-        <v>0.08939999999999999</v>
+        <v>0.099</v>
       </c>
       <c r="G39" s="5" t="n">
         <v>0.636442356808484</v>
@@ -8473,7 +8473,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr"/>
       <c r="F40" s="5" t="n">
-        <v>0.0813</v>
+        <v>0.09030000000000001</v>
       </c>
       <c r="G40" s="5" t="n">
         <v>0.636442356808484</v>
@@ -8554,10 +8554,10 @@
         <v>0.9091</v>
       </c>
       <c r="E41" s="5" t="n">
-        <v>0.1167</v>
+        <v>0.1216</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.2803</v>
+        <v>0.3194</v>
       </c>
       <c r="G41" s="5" t="n">
         <v>0.15663609258386</v>
@@ -8638,10 +8638,10 @@
         <v>0.8824</v>
       </c>
       <c r="E42" s="5" t="n">
-        <v>0.2501</v>
+        <v>0.2655</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.2261</v>
+        <v>0.2642</v>
       </c>
       <c r="G42" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -8723,7 +8723,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr"/>
       <c r="F43" s="5" t="n">
-        <v>0.2674</v>
+        <v>0.3035</v>
       </c>
       <c r="G43" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -8789,7 +8789,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr"/>
       <c r="F44" s="5" t="n">
-        <v>0.2715</v>
+        <v>0.3103</v>
       </c>
       <c r="G44" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -8854,10 +8854,10 @@
         <v>0.9376</v>
       </c>
       <c r="E45" s="5" t="n">
-        <v>0.0616</v>
+        <v>0.06569999999999999</v>
       </c>
       <c r="F45" s="5" t="n">
-        <v>0.0283</v>
+        <v>0.0285</v>
       </c>
       <c r="G45" s="5" t="n">
         <v>0.15663609258386</v>
@@ -8938,10 +8938,10 @@
         <v>0.9273</v>
       </c>
       <c r="E46" s="5" t="n">
-        <v>0.0306</v>
+        <v>0.0317</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.081</v>
+        <v>0.0929</v>
       </c>
       <c r="G46" s="5" t="n">
         <v>0.15663609258386</v>
@@ -9022,10 +9022,10 @@
         <v>0.8865</v>
       </c>
       <c r="E47" s="5" t="n">
-        <v>0.1883</v>
+        <v>0.1993</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.1353</v>
+        <v>0.1422</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>0.64186785726147</v>
@@ -9090,10 +9090,10 @@
         <v>0.8265</v>
       </c>
       <c r="E48" s="5" t="n">
-        <v>0.06469999999999999</v>
+        <v>0.0653</v>
       </c>
       <c r="F48" s="5" t="n">
-        <v>0.0301</v>
+        <v>0.0303</v>
       </c>
       <c r="G48" s="5" t="n">
         <v>0.231026075027885</v>
@@ -9175,7 +9175,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr"/>
       <c r="F49" s="5" t="n">
-        <v>0.0216</v>
+        <v>0.0219</v>
       </c>
       <c r="G49" s="5" t="n">
         <v>0.158699742317549</v>
@@ -9240,10 +9240,10 @@
         <v>0.8865</v>
       </c>
       <c r="E50" s="5" t="n">
-        <v>0.1969</v>
+        <v>0.2072</v>
       </c>
       <c r="F50" s="5" t="n">
-        <v>0.1655</v>
+        <v>0.1731</v>
       </c>
       <c r="G50" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -9308,10 +9308,10 @@
         <v>0.9254</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>0.0528</v>
+        <v>0.0554</v>
       </c>
       <c r="F51" s="5" t="n">
-        <v>0.0629</v>
+        <v>0.0665</v>
       </c>
       <c r="G51" s="5" t="inlineStr"/>
       <c r="H51" s="5" t="inlineStr"/>
@@ -9372,10 +9372,10 @@
         <v>0.9391</v>
       </c>
       <c r="E52" s="5" t="n">
-        <v>0.1308</v>
+        <v>0.1371</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.1312</v>
+        <v>0.1505</v>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr"/>
@@ -9436,10 +9436,10 @@
         <v>0.9638</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>0.0143</v>
+        <v>0.0145</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0.0042</v>
+        <v>0.0037</v>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
       <c r="H53" s="5" t="inlineStr"/>
@@ -9500,10 +9500,10 @@
         <v>0.9545</v>
       </c>
       <c r="E54" s="5" t="n">
-        <v>0.0265</v>
+        <v>0.0266</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>0.0185</v>
+        <v>0.0182</v>
       </c>
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr"/>
@@ -9624,10 +9624,10 @@
         <v>0.9643</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>0.0066</v>
+        <v>0.0067</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>0.0089</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr"/>
@@ -9689,7 +9689,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr"/>
       <c r="F57" s="5" t="n">
-        <v>0.0144</v>
+        <v>0.0146</v>
       </c>
       <c r="G57" s="5" t="inlineStr"/>
       <c r="H57" s="5" t="inlineStr"/>
@@ -9751,7 +9751,7 @@
       </c>
       <c r="E58" s="5" t="inlineStr"/>
       <c r="F58" s="5" t="n">
-        <v>0.0219</v>
+        <v>0.0221</v>
       </c>
       <c r="G58" s="5" t="inlineStr"/>
       <c r="H58" s="5" t="inlineStr"/>
@@ -9812,10 +9812,10 @@
         <v>0.9276</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>0.0298</v>
+        <v>0.0311</v>
       </c>
       <c r="F59" s="5" t="n">
-        <v>0.0184</v>
+        <v>0.0188</v>
       </c>
       <c r="G59" s="5" t="inlineStr"/>
       <c r="H59" s="5" t="inlineStr"/>
@@ -9936,10 +9936,10 @@
         <v>1.0047</v>
       </c>
       <c r="E61" s="5" t="n">
-        <v>0.0509</v>
+        <v>0.052</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>0.019</v>
+        <v>0.0195</v>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr"/>
@@ -10000,10 +10000,10 @@
         <v>0.9635</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>0.0168</v>
+        <v>0.0171</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0.0077</v>
+        <v>0.0076</v>
       </c>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr"/>
@@ -10064,10 +10064,10 @@
         <v>0.9635</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>0.055</v>
+        <v>0.0574</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.01</v>
       </c>
       <c r="G63" s="5" t="inlineStr"/>
       <c r="H63" s="5" t="inlineStr"/>
@@ -10128,10 +10128,10 @@
         <v>0.9528</v>
       </c>
       <c r="E64" s="5" t="n">
-        <v>0.0178</v>
+        <v>0.018</v>
       </c>
       <c r="F64" s="5" t="n">
-        <v>0.0214</v>
+        <v>0.0217</v>
       </c>
       <c r="G64" s="5" t="inlineStr"/>
       <c r="H64" s="5" t="inlineStr"/>
@@ -10192,10 +10192,10 @@
         <v>0.9618</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>0.0134</v>
+        <v>0.0136</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>0.0043</v>
+        <v>0.004</v>
       </c>
       <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr"/>
@@ -10256,10 +10256,10 @@
         <v>0.8661</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>0.0056</v>
+        <v>0.0057</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>0.0102</v>
+        <v>0.0103</v>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
       <c r="H66" s="5" t="inlineStr"/>
@@ -10320,10 +10320,10 @@
         <v>0.896</v>
       </c>
       <c r="E67" s="5" t="n">
-        <v>0.064</v>
+        <v>0.0655</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>0.07679999999999999</v>
+        <v>0.0804</v>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
       <c r="H67" s="5" t="inlineStr"/>
@@ -10387,7 +10387,7 @@
         <v>0.0002</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>0.0035</v>
+        <v>0.0034</v>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr"/>
@@ -10448,10 +10448,10 @@
         <v>0.8265</v>
       </c>
       <c r="E69" s="5" t="n">
-        <v>0.0573</v>
+        <v>0.0579</v>
       </c>
       <c r="F69" s="5" t="n">
-        <v>0.0549</v>
+        <v>0.0601</v>
       </c>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr"/>
@@ -10512,10 +10512,10 @@
         <v>0.9694</v>
       </c>
       <c r="E70" s="5" t="n">
-        <v>0.0294</v>
+        <v>0.0304</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>0.023</v>
+        <v>0.0235</v>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
Update renewable generator dashboard data 2026-10-06 (REZ from the ELI appendices, wind ELI by name, refreshed actuals)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -549,12 +549,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>ELI Near Term</t>
+          <t>ELI Near Term (2026-28)</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>ELI Med Term</t>
+          <t>ELI Med Term (2030-35)</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
@@ -646,7 +646,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -664,7 +664,7 @@
         <v>0.1499</v>
       </c>
       <c r="L2" s="5" t="n">
-        <v>0.2043</v>
+        <v>0.2036</v>
       </c>
       <c r="M2" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -741,7 +741,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -759,7 +759,7 @@
         <v>0.1357</v>
       </c>
       <c r="L3" s="5" t="n">
-        <v>0.0837</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="M3" s="5" t="n">
         <v>0.636442356808484</v>
@@ -836,7 +836,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -854,7 +854,7 @@
         <v>0.1299</v>
       </c>
       <c r="L4" s="5" t="n">
-        <v>0.1043</v>
+        <v>0.1044</v>
       </c>
       <c r="M4" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -931,7 +931,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -1075,7 +1075,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1090,7 +1090,7 @@
         <v>132</v>
       </c>
       <c r="K7" s="5" t="n">
-        <v>0.0296</v>
+        <v>0.0293</v>
       </c>
       <c r="L7" s="5" t="n">
         <v>0.0419</v>
@@ -1149,12 +1149,12 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>South west NSW</t>
+          <t>South West New South Wales</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -1169,10 +1169,10 @@
         <v>132</v>
       </c>
       <c r="K8" s="5" t="n">
-        <v>0.0827</v>
+        <v>0.0819</v>
       </c>
       <c r="L8" s="5" t="n">
-        <v>0.2172</v>
+        <v>0.2164</v>
       </c>
       <c r="M8" s="5" t="n">
         <v>0.529503172508041</v>
@@ -1201,7 +1201,7 @@
         <v>0.01</v>
       </c>
       <c r="U8" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="V8" s="6" t="n">
         <v>0.16</v>
@@ -1247,7 +1247,7 @@
       <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="5" t="inlineStr"/>
       <c r="L9" s="5" t="n">
-        <v>0.4061</v>
+        <v>0.4055</v>
       </c>
       <c r="M9" s="5" t="inlineStr"/>
       <c r="N9" s="5" t="inlineStr"/>
@@ -1300,7 +1300,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1379,7 +1379,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1505,7 +1505,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1523,7 +1523,7 @@
         <v>0.3634</v>
       </c>
       <c r="L13" s="5" t="n">
-        <v>0.469</v>
+        <v>0.4689</v>
       </c>
       <c r="M13" s="5" t="n">
         <v>0.87127903942823</v>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1693,7 +1693,7 @@
         <v>0.1456</v>
       </c>
       <c r="L15" s="5" t="n">
-        <v>0.2826</v>
+        <v>0.2819</v>
       </c>
       <c r="M15" s="5" t="n">
         <v>0.165388664850326</v>
@@ -1749,12 +1749,12 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>Northwest NSW</t>
+          <t>Northwest New South Wales</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
@@ -1772,7 +1772,7 @@
         <v>0.1888</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>0.3026</v>
+        <v>0.3015</v>
       </c>
       <c r="M16" s="5" t="n">
         <v>0.903607825126104</v>
@@ -1849,7 +1849,7 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
@@ -1867,7 +1867,7 @@
         <v>0.3083</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>0.2523</v>
+        <v>0.251</v>
       </c>
       <c r="M17" s="5" t="n">
         <v>0.64186785726147</v>
@@ -1928,7 +1928,7 @@
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1946,7 +1946,7 @@
         <v>0.119</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>0.3509</v>
+        <v>0.351</v>
       </c>
       <c r="M18" s="5" t="n">
         <v>0.87127903942823</v>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
@@ -2025,7 +2025,7 @@
         <v>0.297</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>0.302</v>
+        <v>0.301</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -2097,12 +2097,12 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>South west NSW</t>
+          <t>South West New South Wales</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -2120,7 +2120,7 @@
         <v>0.2549</v>
       </c>
       <c r="L20" s="5" t="n">
-        <v>0.2348</v>
+        <v>0.234</v>
       </c>
       <c r="M20" s="5" t="n">
         <v>0.505349468159863</v>
@@ -2149,7 +2149,7 @@
         <v>0.01</v>
       </c>
       <c r="U20" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="V20" s="6" t="n">
         <v>0.16</v>
@@ -2192,12 +2192,12 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>South west NSW</t>
+          <t>South West New South Wales</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
@@ -2215,7 +2215,7 @@
         <v>0.254</v>
       </c>
       <c r="L21" s="5" t="n">
-        <v>0.2107</v>
+        <v>0.2101</v>
       </c>
       <c r="M21" s="5" t="n">
         <v>0.505349468159863</v>
@@ -2244,7 +2244,7 @@
         <v>0.01</v>
       </c>
       <c r="U21" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="V21" s="6" t="n">
         <v>0.16</v>
@@ -2292,7 +2292,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2310,7 +2310,7 @@
         <v>0.6709000000000001</v>
       </c>
       <c r="L22" s="5" t="n">
-        <v>0.673</v>
+        <v>0.6725</v>
       </c>
       <c r="M22" s="5" t="n">
         <v>0.919931770355409</v>
@@ -2387,7 +2387,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2405,7 +2405,7 @@
         <v>0.0711</v>
       </c>
       <c r="L23" s="5" t="n">
-        <v>0.1724</v>
+        <v>0.1716</v>
       </c>
       <c r="M23" s="5" t="n">
         <v>0.231026075027885</v>
@@ -2482,7 +2482,7 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
@@ -2500,7 +2500,7 @@
         <v>0.6756</v>
       </c>
       <c r="L24" s="5" t="n">
-        <v>0.4942</v>
+        <v>0.4936</v>
       </c>
       <c r="M24" s="5" t="n">
         <v>0.919931770355409</v>
@@ -2572,12 +2572,12 @@
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>Northwest NSW</t>
+          <t>Northwest New South Wales</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2592,10 +2592,10 @@
         <v>66</v>
       </c>
       <c r="K25" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0018</v>
       </c>
       <c r="L25" s="5" t="n">
-        <v>0.0169</v>
+        <v>0.017</v>
       </c>
       <c r="M25" s="5" t="n">
         <v>0.188257195450457</v>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2863,7 +2863,7 @@
         <v>0.0799</v>
       </c>
       <c r="L29" s="5" t="n">
-        <v>0.3181</v>
+        <v>0.3177</v>
       </c>
       <c r="M29" s="5" t="n">
         <v>0.15663609258386</v>
@@ -2940,7 +2940,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2955,10 +2955,10 @@
         <v>330</v>
       </c>
       <c r="K30" s="5" t="n">
-        <v>0.14</v>
+        <v>0.1397</v>
       </c>
       <c r="L30" s="5" t="n">
-        <v>0.0323</v>
+        <v>0.0322</v>
       </c>
       <c r="M30" s="5" t="n">
         <v>0.231026075027885</v>
@@ -3035,7 +3035,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -3050,10 +3050,10 @@
         <v>330</v>
       </c>
       <c r="K31" s="5" t="n">
-        <v>0.1269</v>
+        <v>0.1267</v>
       </c>
       <c r="L31" s="5" t="n">
-        <v>0.0365</v>
+        <v>0.0364</v>
       </c>
       <c r="M31" s="5" t="n">
         <v>0.231026075027885</v>
@@ -3130,7 +3130,7 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -3148,7 +3148,7 @@
         <v>0.0393</v>
       </c>
       <c r="L32" s="5" t="n">
-        <v>0.3484</v>
+        <v>0.3485</v>
       </c>
       <c r="M32" s="5" t="n">
         <v>0.15663609258386</v>
@@ -3225,7 +3225,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
@@ -3243,7 +3243,7 @@
         <v>0.304</v>
       </c>
       <c r="L33" s="5" t="n">
-        <v>0.326</v>
+        <v>0.3263</v>
       </c>
       <c r="M33" s="5" t="n">
         <v>0.87127903942823</v>
@@ -3397,12 +3397,12 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>South west NSW</t>
+          <t>South West New South Wales</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3417,10 +3417,10 @@
         <v>220</v>
       </c>
       <c r="K36" s="5" t="n">
-        <v>0.1174</v>
+        <v>0.1173</v>
       </c>
       <c r="L36" s="5" t="n">
-        <v>0.0941</v>
+        <v>0.09420000000000001</v>
       </c>
       <c r="M36" s="5" t="n">
         <v>0.505349468159863</v>
@@ -3449,7 +3449,7 @@
         <v>0.01</v>
       </c>
       <c r="U36" s="6" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="V36" s="6" t="n">
         <v>0.16</v>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
@@ -3515,7 +3515,7 @@
         <v>0.2596</v>
       </c>
       <c r="L37" s="5" t="n">
-        <v>0.2874</v>
+        <v>0.2869</v>
       </c>
       <c r="M37" s="5" t="n">
         <v>0.1571570475144</v>
@@ -3667,7 +3667,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3683,7 +3683,7 @@
       </c>
       <c r="K39" s="5" t="inlineStr"/>
       <c r="L39" s="5" t="n">
-        <v>0.099</v>
+        <v>0.0987</v>
       </c>
       <c r="M39" s="5" t="n">
         <v>0.636442356808484</v>
@@ -3760,7 +3760,7 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="K40" s="5" t="inlineStr"/>
       <c r="L40" s="5" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.08989999999999999</v>
       </c>
       <c r="M40" s="5" t="n">
         <v>0.636442356808484</v>
@@ -3853,7 +3853,7 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
@@ -3871,7 +3871,7 @@
         <v>0.1216</v>
       </c>
       <c r="L41" s="5" t="n">
-        <v>0.3194</v>
+        <v>0.318</v>
       </c>
       <c r="M41" s="5" t="n">
         <v>0.15663609258386</v>
@@ -3948,7 +3948,7 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
@@ -3966,7 +3966,7 @@
         <v>0.2655</v>
       </c>
       <c r="L42" s="5" t="n">
-        <v>0.2642</v>
+        <v>0.2635</v>
       </c>
       <c r="M42" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -4043,7 +4043,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -4059,7 +4059,7 @@
       </c>
       <c r="K43" s="5" t="inlineStr"/>
       <c r="L43" s="5" t="n">
-        <v>0.3035</v>
+        <v>0.3037</v>
       </c>
       <c r="M43" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -4120,7 +4120,7 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -4136,7 +4136,7 @@
       </c>
       <c r="K44" s="5" t="inlineStr"/>
       <c r="L44" s="5" t="n">
-        <v>0.3103</v>
+        <v>0.3105</v>
       </c>
       <c r="M44" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -4197,7 +4197,7 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
@@ -4292,7 +4292,7 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -4310,7 +4310,7 @@
         <v>0.0317</v>
       </c>
       <c r="L46" s="5" t="n">
-        <v>0.0929</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="M46" s="5" t="n">
         <v>0.15663609258386</v>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
@@ -4405,7 +4405,7 @@
         <v>0.1993</v>
       </c>
       <c r="L47" s="5" t="n">
-        <v>0.1422</v>
+        <v>0.1423</v>
       </c>
       <c r="M47" s="5" t="n">
         <v>0.64186785726147</v>
@@ -4466,7 +4466,7 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr">
@@ -4561,7 +4561,7 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr">
@@ -4577,7 +4577,7 @@
       </c>
       <c r="K49" s="5" t="inlineStr"/>
       <c r="L49" s="5" t="n">
-        <v>0.0219</v>
+        <v>0.0122</v>
       </c>
       <c r="M49" s="5" t="n">
         <v>0.158699742317549</v>
@@ -4638,7 +4638,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>seed</t>
+          <t>eli</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4701,9 +4701,21 @@
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr"/>
-      <c r="E51" s="2" t="inlineStr"/>
-      <c r="F51" s="3" t="inlineStr"/>
-      <c r="G51" s="2" t="inlineStr"/>
+      <c r="E51" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -4714,7 +4726,7 @@
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="5" t="n">
-        <v>0.0554</v>
+        <v>0.0555</v>
       </c>
       <c r="L51" s="5" t="n">
         <v>0.0665</v>
@@ -4754,9 +4766,21 @@
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr"/>
-      <c r="E52" s="2" t="inlineStr"/>
-      <c r="F52" s="3" t="inlineStr"/>
-      <c r="G52" s="2" t="inlineStr"/>
+      <c r="E52" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H52" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -4770,7 +4794,7 @@
         <v>0.1371</v>
       </c>
       <c r="L52" s="5" t="n">
-        <v>0.1505</v>
+        <v>0.1498</v>
       </c>
       <c r="M52" s="5" t="inlineStr"/>
       <c r="N52" s="5" t="inlineStr"/>
@@ -4807,9 +4831,21 @@
         </is>
       </c>
       <c r="D53" s="3" t="inlineStr"/>
-      <c r="E53" s="2" t="inlineStr"/>
-      <c r="F53" s="3" t="inlineStr"/>
-      <c r="G53" s="2" t="inlineStr"/>
+      <c r="E53" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>Cooma-Monaro</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -4820,10 +4856,10 @@
       </c>
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="5" t="n">
-        <v>0.0145</v>
+        <v>0.0144</v>
       </c>
       <c r="L53" s="5" t="n">
-        <v>0.0037</v>
+        <v>0.0021</v>
       </c>
       <c r="M53" s="5" t="inlineStr"/>
       <c r="N53" s="5" t="inlineStr"/>
@@ -4834,14 +4870,30 @@
       <c r="Q53" s="5" t="n">
         <v>0.9638</v>
       </c>
-      <c r="R53" s="6" t="inlineStr"/>
-      <c r="S53" s="6" t="inlineStr"/>
-      <c r="T53" s="6" t="inlineStr"/>
-      <c r="U53" s="6" t="inlineStr"/>
-      <c r="V53" s="6" t="inlineStr"/>
-      <c r="W53" s="6" t="inlineStr"/>
-      <c r="X53" s="6" t="inlineStr"/>
-      <c r="Y53" s="6" t="inlineStr"/>
+      <c r="R53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S53" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="T53" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="U53" s="6" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="V53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W53" s="6" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="X53" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="Y53" s="6" t="n">
+        <v>0.05666666666666667</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4860,9 +4912,21 @@
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr"/>
-      <c r="E54" s="2" t="inlineStr"/>
-      <c r="F54" s="3" t="inlineStr"/>
-      <c r="G54" s="2" t="inlineStr"/>
+      <c r="E54" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>Central West Orana</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -4876,7 +4940,7 @@
         <v>0.0266</v>
       </c>
       <c r="L54" s="5" t="n">
-        <v>0.0182</v>
+        <v>0.0178</v>
       </c>
       <c r="M54" s="5" t="inlineStr"/>
       <c r="N54" s="5" t="inlineStr"/>
@@ -4887,14 +4951,30 @@
       <c r="Q54" s="5" t="n">
         <v>0.9545</v>
       </c>
-      <c r="R54" s="6" t="inlineStr"/>
-      <c r="S54" s="6" t="inlineStr"/>
-      <c r="T54" s="6" t="inlineStr"/>
-      <c r="U54" s="6" t="inlineStr"/>
-      <c r="V54" s="6" t="inlineStr"/>
-      <c r="W54" s="6" t="inlineStr"/>
-      <c r="X54" s="6" t="inlineStr"/>
-      <c r="Y54" s="6" t="inlineStr"/>
+      <c r="R54" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S54" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="T54" s="6" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="U54" s="6" t="n">
+        <v>0.1433333333333333</v>
+      </c>
+      <c r="V54" s="6" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="W54" s="6" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="X54" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Y54" s="6" t="n">
+        <v>0.2066666666666667</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -4962,9 +5042,21 @@
         </is>
       </c>
       <c r="D56" s="3" t="inlineStr"/>
-      <c r="E56" s="2" t="inlineStr"/>
-      <c r="F56" s="3" t="inlineStr"/>
-      <c r="G56" s="2" t="inlineStr"/>
+      <c r="E56" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -4975,10 +5067,10 @@
       </c>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="5" t="n">
-        <v>0.0067</v>
+        <v>0.0047</v>
       </c>
       <c r="L56" s="5" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0061</v>
       </c>
       <c r="M56" s="5" t="inlineStr"/>
       <c r="N56" s="5" t="inlineStr"/>
@@ -5015,9 +5107,21 @@
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr"/>
-      <c r="E57" s="2" t="inlineStr"/>
-      <c r="F57" s="3" t="inlineStr"/>
-      <c r="G57" s="2" t="inlineStr"/>
+      <c r="E57" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5066,9 +5170,21 @@
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr"/>
-      <c r="E58" s="2" t="inlineStr"/>
-      <c r="F58" s="3" t="inlineStr"/>
-      <c r="G58" s="2" t="inlineStr"/>
+      <c r="E58" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5117,9 +5233,21 @@
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr"/>
-      <c r="E59" s="2" t="inlineStr"/>
-      <c r="F59" s="3" t="inlineStr"/>
-      <c r="G59" s="2" t="inlineStr"/>
+      <c r="E59" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5130,7 +5258,7 @@
       </c>
       <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="5" t="n">
-        <v>0.0311</v>
+        <v>0.0312</v>
       </c>
       <c r="L59" s="5" t="n">
         <v>0.0188</v>
@@ -5219,9 +5347,21 @@
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr"/>
-      <c r="E61" s="2" t="inlineStr"/>
-      <c r="F61" s="3" t="inlineStr"/>
-      <c r="G61" s="2" t="inlineStr"/>
+      <c r="E61" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>Central West Orana</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5235,7 +5375,7 @@
         <v>0.052</v>
       </c>
       <c r="L61" s="5" t="n">
-        <v>0.0195</v>
+        <v>0.0177</v>
       </c>
       <c r="M61" s="5" t="inlineStr"/>
       <c r="N61" s="5" t="inlineStr"/>
@@ -5246,14 +5386,30 @@
       <c r="Q61" s="5" t="n">
         <v>1.0047</v>
       </c>
-      <c r="R61" s="6" t="inlineStr"/>
-      <c r="S61" s="6" t="inlineStr"/>
-      <c r="T61" s="6" t="inlineStr"/>
-      <c r="U61" s="6" t="inlineStr"/>
-      <c r="V61" s="6" t="inlineStr"/>
-      <c r="W61" s="6" t="inlineStr"/>
-      <c r="X61" s="6" t="inlineStr"/>
-      <c r="Y61" s="6" t="inlineStr"/>
+      <c r="R61" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="S61" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="T61" s="6" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="U61" s="6" t="n">
+        <v>0.1433333333333333</v>
+      </c>
+      <c r="V61" s="6" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="W61" s="6" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="X61" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="Y61" s="6" t="n">
+        <v>0.2066666666666667</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -5272,9 +5428,21 @@
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr"/>
-      <c r="E62" s="2" t="inlineStr"/>
-      <c r="F62" s="3" t="inlineStr"/>
-      <c r="G62" s="2" t="inlineStr"/>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5285,10 +5453,10 @@
       </c>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="5" t="n">
-        <v>0.0171</v>
+        <v>0.0155</v>
       </c>
       <c r="L62" s="5" t="n">
-        <v>0.0076</v>
+        <v>0.0031</v>
       </c>
       <c r="M62" s="5" t="inlineStr"/>
       <c r="N62" s="5" t="inlineStr"/>
@@ -5325,9 +5493,21 @@
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr"/>
-      <c r="E63" s="2" t="inlineStr"/>
-      <c r="F63" s="3" t="inlineStr"/>
-      <c r="G63" s="2" t="inlineStr"/>
+      <c r="E63" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F63" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5338,10 +5518,10 @@
       </c>
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="5" t="n">
-        <v>0.0574</v>
+        <v>0.0565</v>
       </c>
       <c r="L63" s="5" t="n">
-        <v>0.01</v>
+        <v>0.0047</v>
       </c>
       <c r="M63" s="5" t="inlineStr"/>
       <c r="N63" s="5" t="inlineStr"/>
@@ -5378,9 +5558,21 @@
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr"/>
-      <c r="E64" s="2" t="inlineStr"/>
-      <c r="F64" s="3" t="inlineStr"/>
-      <c r="G64" s="2" t="inlineStr"/>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5431,9 +5623,21 @@
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr"/>
-      <c r="E65" s="2" t="inlineStr"/>
-      <c r="F65" s="3" t="inlineStr"/>
-      <c r="G65" s="2" t="inlineStr"/>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F65" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5444,10 +5648,10 @@
       </c>
       <c r="J65" s="2" t="inlineStr"/>
       <c r="K65" s="5" t="n">
-        <v>0.0136</v>
+        <v>0.0135</v>
       </c>
       <c r="L65" s="5" t="n">
-        <v>0.004</v>
+        <v>0.0014</v>
       </c>
       <c r="M65" s="5" t="inlineStr"/>
       <c r="N65" s="5" t="inlineStr"/>
@@ -5484,9 +5688,21 @@
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr"/>
-      <c r="E66" s="2" t="inlineStr"/>
-      <c r="F66" s="3" t="inlineStr"/>
-      <c r="G66" s="2" t="inlineStr"/>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H66" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5497,10 +5713,10 @@
       </c>
       <c r="J66" s="2" t="inlineStr"/>
       <c r="K66" s="5" t="n">
-        <v>0.0057</v>
+        <v>0.0056</v>
       </c>
       <c r="L66" s="5" t="n">
-        <v>0.0103</v>
+        <v>0.0102</v>
       </c>
       <c r="M66" s="5" t="inlineStr"/>
       <c r="N66" s="5" t="inlineStr"/>
@@ -5511,14 +5727,30 @@
       <c r="Q66" s="5" t="n">
         <v>0.8661</v>
       </c>
-      <c r="R66" s="6" t="inlineStr"/>
-      <c r="S66" s="6" t="inlineStr"/>
-      <c r="T66" s="6" t="inlineStr"/>
-      <c r="U66" s="6" t="inlineStr"/>
-      <c r="V66" s="6" t="inlineStr"/>
-      <c r="W66" s="6" t="inlineStr"/>
-      <c r="X66" s="6" t="inlineStr"/>
-      <c r="Y66" s="6" t="inlineStr"/>
+      <c r="R66" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S66" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T66" s="6" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="U66" s="6" t="n">
+        <v>0.1633333333333333</v>
+      </c>
+      <c r="V66" s="6" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="W66" s="6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="X66" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="Y66" s="6" t="n">
+        <v>0.2533333333333334</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5537,9 +5769,21 @@
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr"/>
-      <c r="E67" s="2" t="inlineStr"/>
-      <c r="F67" s="3" t="inlineStr"/>
-      <c r="G67" s="2" t="inlineStr"/>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F67" s="3" t="inlineStr">
+        <is>
+          <t>Broken Hill</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H67" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5553,7 +5797,7 @@
         <v>0.0655</v>
       </c>
       <c r="L67" s="5" t="n">
-        <v>0.0804</v>
+        <v>0.0803</v>
       </c>
       <c r="M67" s="5" t="inlineStr"/>
       <c r="N67" s="5" t="inlineStr"/>
@@ -5564,14 +5808,30 @@
       <c r="Q67" s="5" t="n">
         <v>0.896</v>
       </c>
-      <c r="R67" s="6" t="inlineStr"/>
-      <c r="S67" s="6" t="inlineStr"/>
-      <c r="T67" s="6" t="inlineStr"/>
-      <c r="U67" s="6" t="inlineStr"/>
-      <c r="V67" s="6" t="inlineStr"/>
-      <c r="W67" s="6" t="inlineStr"/>
-      <c r="X67" s="6" t="inlineStr"/>
-      <c r="Y67" s="6" t="inlineStr"/>
+      <c r="R67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S67" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="T67" s="6" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="U67" s="6" t="n">
+        <v>0.01666666666666667</v>
+      </c>
+      <c r="V67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="W67" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="X67" s="6" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="Y67" s="6" t="n">
+        <v>0.06999999999999999</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -5590,9 +5850,21 @@
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr"/>
-      <c r="E68" s="2" t="inlineStr"/>
-      <c r="F68" s="3" t="inlineStr"/>
-      <c r="G68" s="2" t="inlineStr"/>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H68" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5603,10 +5875,10 @@
       </c>
       <c r="J68" s="2" t="inlineStr"/>
       <c r="K68" s="5" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="L68" s="5" t="n">
-        <v>0.0034</v>
+        <v>0</v>
       </c>
       <c r="M68" s="5" t="inlineStr"/>
       <c r="N68" s="5" t="inlineStr"/>
@@ -5643,9 +5915,21 @@
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr"/>
-      <c r="E69" s="2" t="inlineStr"/>
-      <c r="F69" s="3" t="inlineStr"/>
-      <c r="G69" s="2" t="inlineStr"/>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="F69" s="3" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H69" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5659,7 +5943,7 @@
         <v>0.0579</v>
       </c>
       <c r="L69" s="5" t="n">
-        <v>0.0601</v>
+        <v>0.06</v>
       </c>
       <c r="M69" s="5" t="inlineStr"/>
       <c r="N69" s="5" t="inlineStr"/>
@@ -5670,14 +5954,30 @@
       <c r="Q69" s="5" t="n">
         <v>0.8265</v>
       </c>
-      <c r="R69" s="6" t="inlineStr"/>
-      <c r="S69" s="6" t="inlineStr"/>
-      <c r="T69" s="6" t="inlineStr"/>
-      <c r="U69" s="6" t="inlineStr"/>
-      <c r="V69" s="6" t="inlineStr"/>
-      <c r="W69" s="6" t="inlineStr"/>
-      <c r="X69" s="6" t="inlineStr"/>
-      <c r="Y69" s="6" t="inlineStr"/>
+      <c r="R69" s="6" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="S69" s="6" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="T69" s="6" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="U69" s="6" t="n">
+        <v>0.1633333333333333</v>
+      </c>
+      <c r="V69" s="6" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="W69" s="6" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="X69" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="Y69" s="6" t="n">
+        <v>0.2533333333333334</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -5696,9 +5996,21 @@
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr"/>
-      <c r="E70" s="2" t="inlineStr"/>
-      <c r="F70" s="3" t="inlineStr"/>
-      <c r="G70" s="2" t="inlineStr"/>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>N</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="inlineStr">
+        <is>
+          <t>Non-REZ</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>eli</t>
+        </is>
+      </c>
       <c r="H70" s="2" t="inlineStr">
         <is>
           <t>NSW</t>
@@ -5712,7 +6024,7 @@
         <v>0.0304</v>
       </c>
       <c r="L70" s="5" t="n">
-        <v>0.0235</v>
+        <v>0.021</v>
       </c>
       <c r="M70" s="5" t="inlineStr"/>
       <c r="N70" s="5" t="inlineStr"/>
@@ -5903,7 +6215,7 @@
         <v>0.1499</v>
       </c>
       <c r="F2" s="5" t="n">
-        <v>0.2043</v>
+        <v>0.2036</v>
       </c>
       <c r="G2" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -5987,7 +6299,7 @@
         <v>0.1357</v>
       </c>
       <c r="F3" s="5" t="n">
-        <v>0.0837</v>
+        <v>0.08359999999999999</v>
       </c>
       <c r="G3" s="5" t="n">
         <v>0.636442356808484</v>
@@ -6071,7 +6383,7 @@
         <v>0.1299</v>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0.1043</v>
+        <v>0.1044</v>
       </c>
       <c r="G4" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -6272,7 +6584,7 @@
         <v>0.8416</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>0.0296</v>
+        <v>0.0293</v>
       </c>
       <c r="F7" s="5" t="n">
         <v>0.0419</v>
@@ -6284,42 +6596,18 @@
         <v>0.0107432723897736</v>
       </c>
       <c r="I7" s="5" t="inlineStr"/>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J7" s="5" t="inlineStr"/>
       <c r="K7" s="5" t="inlineStr"/>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L7" s="5" t="inlineStr"/>
       <c r="M7" s="5" t="inlineStr"/>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N7" s="5" t="inlineStr"/>
       <c r="O7" s="5" t="inlineStr"/>
       <c r="P7" s="5" t="inlineStr"/>
-      <c r="Q7" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q7" s="5" t="inlineStr"/>
       <c r="R7" s="5" t="inlineStr"/>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S7" s="5" t="inlineStr"/>
       <c r="T7" s="5" t="inlineStr"/>
-      <c r="U7" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U7" s="5" t="inlineStr"/>
       <c r="V7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
@@ -6340,10 +6628,10 @@
         <v>0.8912</v>
       </c>
       <c r="E8" s="5" t="n">
-        <v>0.0827</v>
+        <v>0.0819</v>
       </c>
       <c r="F8" s="5" t="n">
-        <v>0.2172</v>
+        <v>0.2164</v>
       </c>
       <c r="G8" s="5" t="n">
         <v>0.529503172508041</v>
@@ -6376,7 +6664,7 @@
         </is>
       </c>
       <c r="O8" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="P8" s="5" t="n">
         <v>0.16</v>
@@ -6425,7 +6713,7 @@
       </c>
       <c r="E9" s="5" t="inlineStr"/>
       <c r="F9" s="5" t="n">
-        <v>0.4061</v>
+        <v>0.4055</v>
       </c>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
@@ -6474,42 +6762,18 @@
         <v>0.0107432723897736</v>
       </c>
       <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr"/>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L10" s="5" t="inlineStr"/>
       <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N10" s="5" t="inlineStr"/>
       <c r="O10" s="5" t="inlineStr"/>
       <c r="P10" s="5" t="inlineStr"/>
-      <c r="Q10" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q10" s="5" t="inlineStr"/>
       <c r="R10" s="5" t="inlineStr"/>
-      <c r="S10" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S10" s="5" t="inlineStr"/>
       <c r="T10" s="5" t="inlineStr"/>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U10" s="5" t="inlineStr"/>
       <c r="V10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
@@ -6540,42 +6804,18 @@
         <v>0.264676213474225</v>
       </c>
       <c r="I11" s="5" t="inlineStr"/>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J11" s="5" t="inlineStr"/>
       <c r="K11" s="5" t="inlineStr"/>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L11" s="5" t="inlineStr"/>
       <c r="M11" s="5" t="inlineStr"/>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N11" s="5" t="inlineStr"/>
       <c r="O11" s="5" t="inlineStr"/>
       <c r="P11" s="5" t="inlineStr"/>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q11" s="5" t="inlineStr"/>
       <c r="R11" s="5" t="inlineStr"/>
-      <c r="S11" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S11" s="5" t="inlineStr"/>
       <c r="T11" s="5" t="inlineStr"/>
-      <c r="U11" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U11" s="5" t="inlineStr"/>
       <c r="V11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
@@ -6635,7 +6875,7 @@
         <v>0.3634</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>0.469</v>
+        <v>0.4689</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0.87127903942823</v>
@@ -6724,42 +6964,18 @@
         <v>0.0107432723897736</v>
       </c>
       <c r="I14" s="5" t="inlineStr"/>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J14" s="5" t="inlineStr"/>
       <c r="K14" s="5" t="inlineStr"/>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L14" s="5" t="inlineStr"/>
       <c r="M14" s="5" t="inlineStr"/>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N14" s="5" t="inlineStr"/>
       <c r="O14" s="5" t="inlineStr"/>
       <c r="P14" s="5" t="inlineStr"/>
-      <c r="Q14" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q14" s="5" t="inlineStr"/>
       <c r="R14" s="5" t="inlineStr"/>
-      <c r="S14" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S14" s="5" t="inlineStr"/>
       <c r="T14" s="5" t="inlineStr"/>
-      <c r="U14" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U14" s="5" t="inlineStr"/>
       <c r="V14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
@@ -6783,7 +6999,7 @@
         <v>0.1456</v>
       </c>
       <c r="F15" s="5" t="n">
-        <v>0.2826</v>
+        <v>0.2819</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>0.165388664850326</v>
@@ -6792,42 +7008,18 @@
         <v>0.000681438300925263</v>
       </c>
       <c r="I15" s="5" t="inlineStr"/>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J15" s="5" t="inlineStr"/>
       <c r="K15" s="5" t="inlineStr"/>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L15" s="5" t="inlineStr"/>
       <c r="M15" s="5" t="inlineStr"/>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N15" s="5" t="inlineStr"/>
       <c r="O15" s="5" t="inlineStr"/>
       <c r="P15" s="5" t="inlineStr"/>
-      <c r="Q15" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q15" s="5" t="inlineStr"/>
       <c r="R15" s="5" t="inlineStr"/>
-      <c r="S15" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S15" s="5" t="inlineStr"/>
       <c r="T15" s="5" t="inlineStr"/>
-      <c r="U15" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U15" s="5" t="inlineStr"/>
       <c r="V15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
@@ -6851,7 +7043,7 @@
         <v>0.1888</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0.3026</v>
+        <v>0.3015</v>
       </c>
       <c r="G16" s="5" t="n">
         <v>0.903607825126104</v>
@@ -6935,7 +7127,7 @@
         <v>0.3083</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>0.2523</v>
+        <v>0.251</v>
       </c>
       <c r="G17" s="5" t="n">
         <v>0.64186785726147</v>
@@ -6944,42 +7136,18 @@
         <v>0.0107432723897736</v>
       </c>
       <c r="I17" s="5" t="inlineStr"/>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J17" s="5" t="inlineStr"/>
       <c r="K17" s="5" t="inlineStr"/>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L17" s="5" t="inlineStr"/>
       <c r="M17" s="5" t="inlineStr"/>
-      <c r="N17" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N17" s="5" t="inlineStr"/>
       <c r="O17" s="5" t="inlineStr"/>
       <c r="P17" s="5" t="inlineStr"/>
-      <c r="Q17" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q17" s="5" t="inlineStr"/>
       <c r="R17" s="5" t="inlineStr"/>
-      <c r="S17" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S17" s="5" t="inlineStr"/>
       <c r="T17" s="5" t="inlineStr"/>
-      <c r="U17" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U17" s="5" t="inlineStr"/>
       <c r="V17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
@@ -7003,7 +7171,7 @@
         <v>0.119</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>0.3509</v>
+        <v>0.351</v>
       </c>
       <c r="G18" s="5" t="n">
         <v>0.87127903942823</v>
@@ -7012,42 +7180,18 @@
         <v>0.886109380719023</v>
       </c>
       <c r="I18" s="5" t="inlineStr"/>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J18" s="5" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr"/>
-      <c r="L18" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L18" s="5" t="inlineStr"/>
       <c r="M18" s="5" t="inlineStr"/>
-      <c r="N18" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N18" s="5" t="inlineStr"/>
       <c r="O18" s="5" t="inlineStr"/>
       <c r="P18" s="5" t="inlineStr"/>
-      <c r="Q18" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q18" s="5" t="inlineStr"/>
       <c r="R18" s="5" t="inlineStr"/>
-      <c r="S18" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S18" s="5" t="inlineStr"/>
       <c r="T18" s="5" t="inlineStr"/>
-      <c r="U18" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U18" s="5" t="inlineStr"/>
       <c r="V18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
@@ -7071,7 +7215,7 @@
         <v>0.297</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0.302</v>
+        <v>0.301</v>
       </c>
       <c r="G19" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -7155,7 +7299,7 @@
         <v>0.2549</v>
       </c>
       <c r="F20" s="5" t="n">
-        <v>0.2348</v>
+        <v>0.234</v>
       </c>
       <c r="G20" s="5" t="n">
         <v>0.505349468159863</v>
@@ -7188,7 +7332,7 @@
         </is>
       </c>
       <c r="O20" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="P20" s="5" t="n">
         <v>0.16</v>
@@ -7239,7 +7383,7 @@
         <v>0.254</v>
       </c>
       <c r="F21" s="5" t="n">
-        <v>0.2107</v>
+        <v>0.2101</v>
       </c>
       <c r="G21" s="5" t="n">
         <v>0.505349468159863</v>
@@ -7272,7 +7416,7 @@
         </is>
       </c>
       <c r="O21" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="P21" s="5" t="n">
         <v>0.16</v>
@@ -7323,7 +7467,7 @@
         <v>0.6709000000000001</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.673</v>
+        <v>0.6725</v>
       </c>
       <c r="G22" s="5" t="n">
         <v>0.919931770355409</v>
@@ -7407,7 +7551,7 @@
         <v>0.0711</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.1724</v>
+        <v>0.1716</v>
       </c>
       <c r="G23" s="5" t="n">
         <v>0.231026075027885</v>
@@ -7491,7 +7635,7 @@
         <v>0.6756</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.4942</v>
+        <v>0.4936</v>
       </c>
       <c r="G24" s="5" t="n">
         <v>0.919931770355409</v>
@@ -7572,10 +7716,10 @@
         <v>0.8509</v>
       </c>
       <c r="E25" s="5" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.0018</v>
       </c>
       <c r="F25" s="5" t="n">
-        <v>0.0169</v>
+        <v>0.017</v>
       </c>
       <c r="G25" s="5" t="n">
         <v>0.188257195450457</v>
@@ -7736,42 +7880,18 @@
         <v>0.0670248501388058</v>
       </c>
       <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J28" s="5" t="inlineStr"/>
       <c r="K28" s="5" t="inlineStr"/>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L28" s="5" t="inlineStr"/>
       <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N28" s="5" t="inlineStr"/>
       <c r="O28" s="5" t="inlineStr"/>
       <c r="P28" s="5" t="inlineStr"/>
-      <c r="Q28" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q28" s="5" t="inlineStr"/>
       <c r="R28" s="5" t="inlineStr"/>
-      <c r="S28" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S28" s="5" t="inlineStr"/>
       <c r="T28" s="5" t="inlineStr"/>
-      <c r="U28" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U28" s="5" t="inlineStr"/>
       <c r="V28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
@@ -7795,7 +7915,7 @@
         <v>0.0799</v>
       </c>
       <c r="F29" s="5" t="n">
-        <v>0.3181</v>
+        <v>0.3177</v>
       </c>
       <c r="G29" s="5" t="n">
         <v>0.15663609258386</v>
@@ -7876,10 +7996,10 @@
         <v>0.8911</v>
       </c>
       <c r="E30" s="5" t="n">
-        <v>0.14</v>
+        <v>0.1397</v>
       </c>
       <c r="F30" s="5" t="n">
-        <v>0.0323</v>
+        <v>0.0322</v>
       </c>
       <c r="G30" s="5" t="n">
         <v>0.231026075027885</v>
@@ -7960,10 +8080,10 @@
         <v>0.8911</v>
       </c>
       <c r="E31" s="5" t="n">
-        <v>0.1269</v>
+        <v>0.1267</v>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.0365</v>
+        <v>0.0364</v>
       </c>
       <c r="G31" s="5" t="n">
         <v>0.231026075027885</v>
@@ -8047,7 +8167,7 @@
         <v>0.0393</v>
       </c>
       <c r="F32" s="5" t="n">
-        <v>0.3484</v>
+        <v>0.3485</v>
       </c>
       <c r="G32" s="5" t="n">
         <v>0.15663609258386</v>
@@ -8131,7 +8251,7 @@
         <v>0.304</v>
       </c>
       <c r="F33" s="5" t="n">
-        <v>0.326</v>
+        <v>0.3263</v>
       </c>
       <c r="G33" s="5" t="n">
         <v>0.87127903942823</v>
@@ -8140,42 +8260,18 @@
         <v>0.886109380719023</v>
       </c>
       <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J33" s="5" t="inlineStr"/>
       <c r="K33" s="5" t="inlineStr"/>
-      <c r="L33" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L33" s="5" t="inlineStr"/>
       <c r="M33" s="5" t="inlineStr"/>
-      <c r="N33" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N33" s="5" t="inlineStr"/>
       <c r="O33" s="5" t="inlineStr"/>
       <c r="P33" s="5" t="inlineStr"/>
-      <c r="Q33" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q33" s="5" t="inlineStr"/>
       <c r="R33" s="5" t="inlineStr"/>
-      <c r="S33" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S33" s="5" t="inlineStr"/>
       <c r="T33" s="5" t="inlineStr"/>
-      <c r="U33" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U33" s="5" t="inlineStr"/>
       <c r="V33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
@@ -8268,10 +8364,10 @@
         <v>0.8218</v>
       </c>
       <c r="E36" s="5" t="n">
-        <v>0.1174</v>
+        <v>0.1173</v>
       </c>
       <c r="F36" s="5" t="n">
-        <v>0.0941</v>
+        <v>0.09420000000000001</v>
       </c>
       <c r="G36" s="5" t="n">
         <v>0.505349468159863</v>
@@ -8304,7 +8400,7 @@
         </is>
       </c>
       <c r="O36" s="5" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06999999999999999</v>
       </c>
       <c r="P36" s="5" t="n">
         <v>0.16</v>
@@ -8355,7 +8451,7 @@
         <v>0.2596</v>
       </c>
       <c r="F37" s="5" t="n">
-        <v>0.2874</v>
+        <v>0.2869</v>
       </c>
       <c r="G37" s="5" t="n">
         <v>0.1571570475144</v>
@@ -8444,42 +8540,18 @@
         <v>0.000643212863569608</v>
       </c>
       <c r="I38" s="5" t="inlineStr"/>
-      <c r="J38" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J38" s="5" t="inlineStr"/>
       <c r="K38" s="5" t="inlineStr"/>
-      <c r="L38" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L38" s="5" t="inlineStr"/>
       <c r="M38" s="5" t="inlineStr"/>
-      <c r="N38" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N38" s="5" t="inlineStr"/>
       <c r="O38" s="5" t="inlineStr"/>
       <c r="P38" s="5" t="inlineStr"/>
-      <c r="Q38" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q38" s="5" t="inlineStr"/>
       <c r="R38" s="5" t="inlineStr"/>
-      <c r="S38" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S38" s="5" t="inlineStr"/>
       <c r="T38" s="5" t="inlineStr"/>
-      <c r="U38" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U38" s="5" t="inlineStr"/>
       <c r="V38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
@@ -8501,7 +8573,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr"/>
       <c r="F39" s="5" t="n">
-        <v>0.099</v>
+        <v>0.0987</v>
       </c>
       <c r="G39" s="5" t="n">
         <v>0.636442356808484</v>
@@ -8583,7 +8655,7 @@
       </c>
       <c r="E40" s="5" t="inlineStr"/>
       <c r="F40" s="5" t="n">
-        <v>0.09030000000000001</v>
+        <v>0.08989999999999999</v>
       </c>
       <c r="G40" s="5" t="n">
         <v>0.636442356808484</v>
@@ -8667,7 +8739,7 @@
         <v>0.1216</v>
       </c>
       <c r="F41" s="5" t="n">
-        <v>0.3194</v>
+        <v>0.318</v>
       </c>
       <c r="G41" s="5" t="n">
         <v>0.15663609258386</v>
@@ -8751,7 +8823,7 @@
         <v>0.2655</v>
       </c>
       <c r="F42" s="5" t="n">
-        <v>0.2642</v>
+        <v>0.2635</v>
       </c>
       <c r="G42" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -8833,7 +8905,7 @@
       </c>
       <c r="E43" s="5" t="inlineStr"/>
       <c r="F43" s="5" t="n">
-        <v>0.3035</v>
+        <v>0.3037</v>
       </c>
       <c r="G43" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -8842,42 +8914,18 @@
         <v>0.00631707880200049</v>
       </c>
       <c r="I43" s="5" t="inlineStr"/>
-      <c r="J43" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J43" s="5" t="inlineStr"/>
       <c r="K43" s="5" t="inlineStr"/>
-      <c r="L43" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L43" s="5" t="inlineStr"/>
       <c r="M43" s="5" t="inlineStr"/>
-      <c r="N43" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N43" s="5" t="inlineStr"/>
       <c r="O43" s="5" t="inlineStr"/>
       <c r="P43" s="5" t="inlineStr"/>
-      <c r="Q43" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q43" s="5" t="inlineStr"/>
       <c r="R43" s="5" t="inlineStr"/>
-      <c r="S43" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S43" s="5" t="inlineStr"/>
       <c r="T43" s="5" t="inlineStr"/>
-      <c r="U43" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U43" s="5" t="inlineStr"/>
       <c r="V43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
@@ -8899,7 +8947,7 @@
       </c>
       <c r="E44" s="5" t="inlineStr"/>
       <c r="F44" s="5" t="n">
-        <v>0.3103</v>
+        <v>0.3105</v>
       </c>
       <c r="G44" s="5" t="n">
         <v>0.5859908275658871</v>
@@ -8908,42 +8956,18 @@
         <v>0.00631707880200049</v>
       </c>
       <c r="I44" s="5" t="inlineStr"/>
-      <c r="J44" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J44" s="5" t="inlineStr"/>
       <c r="K44" s="5" t="inlineStr"/>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L44" s="5" t="inlineStr"/>
       <c r="M44" s="5" t="inlineStr"/>
-      <c r="N44" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N44" s="5" t="inlineStr"/>
       <c r="O44" s="5" t="inlineStr"/>
       <c r="P44" s="5" t="inlineStr"/>
-      <c r="Q44" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q44" s="5" t="inlineStr"/>
       <c r="R44" s="5" t="inlineStr"/>
-      <c r="S44" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S44" s="5" t="inlineStr"/>
       <c r="T44" s="5" t="inlineStr"/>
-      <c r="U44" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U44" s="5" t="inlineStr"/>
       <c r="V44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
@@ -9051,7 +9075,7 @@
         <v>0.0317</v>
       </c>
       <c r="F46" s="5" t="n">
-        <v>0.0929</v>
+        <v>0.09320000000000001</v>
       </c>
       <c r="G46" s="5" t="n">
         <v>0.15663609258386</v>
@@ -9135,7 +9159,7 @@
         <v>0.1993</v>
       </c>
       <c r="F47" s="5" t="n">
-        <v>0.1422</v>
+        <v>0.1423</v>
       </c>
       <c r="G47" s="5" t="n">
         <v>0.64186785726147</v>
@@ -9144,42 +9168,18 @@
         <v>0.0107432723897736</v>
       </c>
       <c r="I47" s="5" t="inlineStr"/>
-      <c r="J47" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J47" s="5" t="inlineStr"/>
       <c r="K47" s="5" t="inlineStr"/>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L47" s="5" t="inlineStr"/>
       <c r="M47" s="5" t="inlineStr"/>
-      <c r="N47" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N47" s="5" t="inlineStr"/>
       <c r="O47" s="5" t="inlineStr"/>
       <c r="P47" s="5" t="inlineStr"/>
-      <c r="Q47" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q47" s="5" t="inlineStr"/>
       <c r="R47" s="5" t="inlineStr"/>
-      <c r="S47" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S47" s="5" t="inlineStr"/>
       <c r="T47" s="5" t="inlineStr"/>
-      <c r="U47" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U47" s="5" t="inlineStr"/>
       <c r="V47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
@@ -9285,7 +9285,7 @@
       </c>
       <c r="E49" s="5" t="inlineStr"/>
       <c r="F49" s="5" t="n">
-        <v>0.0219</v>
+        <v>0.0122</v>
       </c>
       <c r="G49" s="5" t="n">
         <v>0.158699742317549</v>
@@ -9294,42 +9294,18 @@
         <v>0.000581408571101005</v>
       </c>
       <c r="I49" s="5" t="inlineStr"/>
-      <c r="J49" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J49" s="5" t="inlineStr"/>
       <c r="K49" s="5" t="inlineStr"/>
-      <c r="L49" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L49" s="5" t="inlineStr"/>
       <c r="M49" s="5" t="inlineStr"/>
-      <c r="N49" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N49" s="5" t="inlineStr"/>
       <c r="O49" s="5" t="inlineStr"/>
       <c r="P49" s="5" t="inlineStr"/>
-      <c r="Q49" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q49" s="5" t="inlineStr"/>
       <c r="R49" s="5" t="inlineStr"/>
-      <c r="S49" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S49" s="5" t="inlineStr"/>
       <c r="T49" s="5" t="inlineStr"/>
-      <c r="U49" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U49" s="5" t="inlineStr"/>
       <c r="V49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
@@ -9362,42 +9338,18 @@
         <v>0.00631707880200049</v>
       </c>
       <c r="I50" s="5" t="inlineStr"/>
-      <c r="J50" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="J50" s="5" t="inlineStr"/>
       <c r="K50" s="5" t="inlineStr"/>
-      <c r="L50" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="L50" s="5" t="inlineStr"/>
       <c r="M50" s="5" t="inlineStr"/>
-      <c r="N50" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="N50" s="5" t="inlineStr"/>
       <c r="O50" s="5" t="inlineStr"/>
       <c r="P50" s="5" t="inlineStr"/>
-      <c r="Q50" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
+      <c r="Q50" s="5" t="inlineStr"/>
       <c r="R50" s="5" t="inlineStr"/>
-      <c r="S50" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
+      <c r="S50" s="5" t="inlineStr"/>
       <c r="T50" s="5" t="inlineStr"/>
-      <c r="U50" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
+      <c r="U50" s="5" t="inlineStr"/>
       <c r="V50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
@@ -9418,7 +9370,7 @@
         <v>0.9254</v>
       </c>
       <c r="E51" s="5" t="n">
-        <v>0.0554</v>
+        <v>0.0555</v>
       </c>
       <c r="F51" s="5" t="n">
         <v>0.0665</v>
@@ -9461,7 +9413,7 @@
         <v>0.1371</v>
       </c>
       <c r="F52" s="5" t="n">
-        <v>0.1505</v>
+        <v>0.1498</v>
       </c>
       <c r="G52" s="5" t="inlineStr"/>
       <c r="H52" s="5" t="inlineStr"/>
@@ -9498,27 +9450,67 @@
         <v>0.9638</v>
       </c>
       <c r="E53" s="5" t="n">
-        <v>0.0145</v>
+        <v>0.0144</v>
       </c>
       <c r="F53" s="5" t="n">
-        <v>0.0037</v>
+        <v>0.0021</v>
       </c>
       <c r="G53" s="5" t="inlineStr"/>
       <c r="H53" s="5" t="inlineStr"/>
-      <c r="I53" s="5" t="inlineStr"/>
-      <c r="J53" s="5" t="inlineStr"/>
-      <c r="K53" s="5" t="inlineStr"/>
-      <c r="L53" s="5" t="inlineStr"/>
-      <c r="M53" s="5" t="inlineStr"/>
-      <c r="N53" s="5" t="inlineStr"/>
-      <c r="O53" s="5" t="inlineStr"/>
-      <c r="P53" s="5" t="inlineStr"/>
-      <c r="Q53" s="5" t="inlineStr"/>
-      <c r="R53" s="5" t="inlineStr"/>
-      <c r="S53" s="5" t="inlineStr"/>
-      <c r="T53" s="5" t="inlineStr"/>
-      <c r="U53" s="5" t="inlineStr"/>
-      <c r="V53" s="5" t="inlineStr"/>
+      <c r="I53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="K53" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L53" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="M53" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="N53" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="O53" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="P53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="R53" s="5" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="S53" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="T53" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="U53" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="V53" s="5" t="n">
+        <v>0.05666666666666667</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
@@ -9541,24 +9533,64 @@
         <v>0.0266</v>
       </c>
       <c r="F54" s="5" t="n">
-        <v>0.0182</v>
+        <v>0.0178</v>
       </c>
       <c r="G54" s="5" t="inlineStr"/>
       <c r="H54" s="5" t="inlineStr"/>
-      <c r="I54" s="5" t="inlineStr"/>
-      <c r="J54" s="5" t="inlineStr"/>
-      <c r="K54" s="5" t="inlineStr"/>
-      <c r="L54" s="5" t="inlineStr"/>
-      <c r="M54" s="5" t="inlineStr"/>
-      <c r="N54" s="5" t="inlineStr"/>
-      <c r="O54" s="5" t="inlineStr"/>
-      <c r="P54" s="5" t="inlineStr"/>
-      <c r="Q54" s="5" t="inlineStr"/>
-      <c r="R54" s="5" t="inlineStr"/>
-      <c r="S54" s="5" t="inlineStr"/>
-      <c r="T54" s="5" t="inlineStr"/>
-      <c r="U54" s="5" t="inlineStr"/>
-      <c r="V54" s="5" t="inlineStr"/>
+      <c r="I54" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J54" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="K54" s="5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="L54" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="M54" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="N54" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="O54" s="5" t="n">
+        <v>0.1433333333333333</v>
+      </c>
+      <c r="P54" s="5" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="Q54" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="R54" s="5" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="S54" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="T54" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="U54" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="V54" s="5" t="n">
+        <v>0.2066666666666667</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
@@ -9614,10 +9646,10 @@
         <v>0.9643</v>
       </c>
       <c r="E56" s="5" t="n">
-        <v>0.0067</v>
+        <v>0.0047</v>
       </c>
       <c r="F56" s="5" t="n">
-        <v>0.008800000000000001</v>
+        <v>0.0061</v>
       </c>
       <c r="G56" s="5" t="inlineStr"/>
       <c r="H56" s="5" t="inlineStr"/>
@@ -9730,7 +9762,7 @@
         <v>0.9276</v>
       </c>
       <c r="E59" s="5" t="n">
-        <v>0.0311</v>
+        <v>0.0312</v>
       </c>
       <c r="F59" s="5" t="n">
         <v>0.0188</v>
@@ -9809,24 +9841,64 @@
         <v>0.052</v>
       </c>
       <c r="F61" s="5" t="n">
-        <v>0.0195</v>
+        <v>0.0177</v>
       </c>
       <c r="G61" s="5" t="inlineStr"/>
       <c r="H61" s="5" t="inlineStr"/>
-      <c r="I61" s="5" t="inlineStr"/>
-      <c r="J61" s="5" t="inlineStr"/>
-      <c r="K61" s="5" t="inlineStr"/>
-      <c r="L61" s="5" t="inlineStr"/>
-      <c r="M61" s="5" t="inlineStr"/>
-      <c r="N61" s="5" t="inlineStr"/>
-      <c r="O61" s="5" t="inlineStr"/>
-      <c r="P61" s="5" t="inlineStr"/>
-      <c r="Q61" s="5" t="inlineStr"/>
-      <c r="R61" s="5" t="inlineStr"/>
-      <c r="S61" s="5" t="inlineStr"/>
-      <c r="T61" s="5" t="inlineStr"/>
-      <c r="U61" s="5" t="inlineStr"/>
-      <c r="V61" s="5" t="inlineStr"/>
+      <c r="I61" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="J61" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="K61" s="5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="L61" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="M61" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="N61" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="O61" s="5" t="n">
+        <v>0.1433333333333333</v>
+      </c>
+      <c r="P61" s="5" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="Q61" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="R61" s="5" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="S61" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="T61" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="U61" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="V61" s="5" t="n">
+        <v>0.2066666666666667</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="8" t="inlineStr">
@@ -9846,10 +9918,10 @@
         <v>0.9635</v>
       </c>
       <c r="E62" s="5" t="n">
-        <v>0.0171</v>
+        <v>0.0155</v>
       </c>
       <c r="F62" s="5" t="n">
-        <v>0.0076</v>
+        <v>0.0031</v>
       </c>
       <c r="G62" s="5" t="inlineStr"/>
       <c r="H62" s="5" t="inlineStr"/>
@@ -9886,10 +9958,10 @@
         <v>0.9635</v>
       </c>
       <c r="E63" s="5" t="n">
-        <v>0.0574</v>
+        <v>0.0565</v>
       </c>
       <c r="F63" s="5" t="n">
-        <v>0.01</v>
+        <v>0.0047</v>
       </c>
       <c r="G63" s="5" t="inlineStr"/>
       <c r="H63" s="5" t="inlineStr"/>
@@ -9966,10 +10038,10 @@
         <v>0.9618</v>
       </c>
       <c r="E65" s="5" t="n">
-        <v>0.0136</v>
+        <v>0.0135</v>
       </c>
       <c r="F65" s="5" t="n">
-        <v>0.004</v>
+        <v>0.0014</v>
       </c>
       <c r="G65" s="5" t="inlineStr"/>
       <c r="H65" s="5" t="inlineStr"/>
@@ -10006,27 +10078,67 @@
         <v>0.8661</v>
       </c>
       <c r="E66" s="5" t="n">
-        <v>0.0057</v>
+        <v>0.0056</v>
       </c>
       <c r="F66" s="5" t="n">
-        <v>0.0103</v>
+        <v>0.0102</v>
       </c>
       <c r="G66" s="5" t="inlineStr"/>
       <c r="H66" s="5" t="inlineStr"/>
-      <c r="I66" s="5" t="inlineStr"/>
-      <c r="J66" s="5" t="inlineStr"/>
-      <c r="K66" s="5" t="inlineStr"/>
-      <c r="L66" s="5" t="inlineStr"/>
-      <c r="M66" s="5" t="inlineStr"/>
-      <c r="N66" s="5" t="inlineStr"/>
-      <c r="O66" s="5" t="inlineStr"/>
-      <c r="P66" s="5" t="inlineStr"/>
-      <c r="Q66" s="5" t="inlineStr"/>
-      <c r="R66" s="5" t="inlineStr"/>
-      <c r="S66" s="5" t="inlineStr"/>
-      <c r="T66" s="5" t="inlineStr"/>
-      <c r="U66" s="5" t="inlineStr"/>
-      <c r="V66" s="5" t="inlineStr"/>
+      <c r="I66" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="K66" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L66" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="M66" s="5" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="N66" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="O66" s="5" t="n">
+        <v>0.1633333333333333</v>
+      </c>
+      <c r="P66" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q66" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="R66" s="5" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="S66" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="T66" s="5" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U66" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="V66" s="5" t="n">
+        <v>0.2533333333333334</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
@@ -10049,24 +10161,64 @@
         <v>0.0655</v>
       </c>
       <c r="F67" s="5" t="n">
-        <v>0.0804</v>
+        <v>0.0803</v>
       </c>
       <c r="G67" s="5" t="inlineStr"/>
       <c r="H67" s="5" t="inlineStr"/>
-      <c r="I67" s="5" t="inlineStr"/>
-      <c r="J67" s="5" t="inlineStr"/>
-      <c r="K67" s="5" t="inlineStr"/>
-      <c r="L67" s="5" t="inlineStr"/>
-      <c r="M67" s="5" t="inlineStr"/>
-      <c r="N67" s="5" t="inlineStr"/>
-      <c r="O67" s="5" t="inlineStr"/>
-      <c r="P67" s="5" t="inlineStr"/>
-      <c r="Q67" s="5" t="inlineStr"/>
-      <c r="R67" s="5" t="inlineStr"/>
-      <c r="S67" s="5" t="inlineStr"/>
-      <c r="T67" s="5" t="inlineStr"/>
-      <c r="U67" s="5" t="inlineStr"/>
-      <c r="V67" s="5" t="inlineStr"/>
+      <c r="I67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="K67" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="L67" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="M67" s="5" t="n">
+        <v>0.02</v>
+      </c>
+      <c r="N67" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="O67" s="5" t="n">
+        <v>0.01666666666666667</v>
+      </c>
+      <c r="P67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="R67" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S67" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="T67" s="5" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="U67" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="V67" s="5" t="n">
+        <v>0.06999999999999999</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="8" t="inlineStr">
@@ -10086,10 +10238,10 @@
         <v>1.0029</v>
       </c>
       <c r="E68" s="5" t="n">
-        <v>0.0002</v>
+        <v>0</v>
       </c>
       <c r="F68" s="5" t="n">
-        <v>0.0034</v>
+        <v>0</v>
       </c>
       <c r="G68" s="5" t="inlineStr"/>
       <c r="H68" s="5" t="inlineStr"/>
@@ -10129,24 +10281,64 @@
         <v>0.0579</v>
       </c>
       <c r="F69" s="5" t="n">
-        <v>0.0601</v>
+        <v>0.06</v>
       </c>
       <c r="G69" s="5" t="inlineStr"/>
       <c r="H69" s="5" t="inlineStr"/>
-      <c r="I69" s="5" t="inlineStr"/>
-      <c r="J69" s="5" t="inlineStr"/>
-      <c r="K69" s="5" t="inlineStr"/>
-      <c r="L69" s="5" t="inlineStr"/>
-      <c r="M69" s="5" t="inlineStr"/>
-      <c r="N69" s="5" t="inlineStr"/>
-      <c r="O69" s="5" t="inlineStr"/>
-      <c r="P69" s="5" t="inlineStr"/>
-      <c r="Q69" s="5" t="inlineStr"/>
-      <c r="R69" s="5" t="inlineStr"/>
-      <c r="S69" s="5" t="inlineStr"/>
-      <c r="T69" s="5" t="inlineStr"/>
-      <c r="U69" s="5" t="inlineStr"/>
-      <c r="V69" s="5" t="inlineStr"/>
+      <c r="I69" s="5" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="K69" s="5" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="L69" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="M69" s="5" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="N69" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="O69" s="5" t="n">
+        <v>0.1633333333333333</v>
+      </c>
+      <c r="P69" s="5" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="Q69" s="5" t="inlineStr">
+        <is>
+          <t>25-26</t>
+        </is>
+      </c>
+      <c r="R69" s="5" t="n">
+        <v>0.26</v>
+      </c>
+      <c r="S69" s="5" t="inlineStr">
+        <is>
+          <t>26-27</t>
+        </is>
+      </c>
+      <c r="T69" s="5" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="U69" s="5" t="inlineStr">
+        <is>
+          <t>27-28</t>
+        </is>
+      </c>
+      <c r="V69" s="5" t="n">
+        <v>0.2533333333333334</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="8" t="inlineStr">
@@ -10169,7 +10361,7 @@
         <v>0.0304</v>
       </c>
       <c r="F70" s="5" t="n">
-        <v>0.0235</v>
+        <v>0.021</v>
       </c>
       <c r="G70" s="5" t="inlineStr"/>
       <c r="H70" s="5" t="inlineStr"/>

</xml_diff>

<commit_message>
outputs: regenerate the four state workbooks to match summary.csv (S2-2)
Kept separate so it can be dropped. Not needed for validation, but the lane
publishes outputs/ only when summary.csv changes, and its next run should
reproduce the summary.csv already committed, so without this the workbooks
would keep "per-DUID" in ELI Source (104 rows) and the five old ELI values
until some value next changes. Content changes only: ELI Source per-DUID ->
location (NSW 42, QLD 36, VIC 12, SA 14 cells) and the five NSW ELI cells
(Summary and Heatmap sheets). TAS has no change and is left as is. Built
offline from the committed caches with src.excel_output.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -674,7 +674,7 @@
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P2" s="5" t="n">
@@ -769,7 +769,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P3" s="5" t="n">
@@ -864,7 +864,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P4" s="5" t="n">
@@ -959,7 +959,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P5" s="5" t="n">
@@ -1103,7 +1103,7 @@
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P7" s="5" t="n">
@@ -1182,7 +1182,7 @@
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P8" s="5" t="n">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P10" s="5" t="n">
@@ -1405,7 +1405,7 @@
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P11" s="5" t="n">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P13" s="5" t="n">
@@ -1624,7 +1624,7 @@
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P14" s="5" t="n">
@@ -1703,7 +1703,7 @@
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P15" s="5" t="n">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P16" s="5" t="n">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P17" s="5" t="n">
@@ -1956,7 +1956,7 @@
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P18" s="5" t="n">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P19" s="5" t="n">
@@ -2130,7 +2130,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P20" s="5" t="n">
@@ -2225,7 +2225,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P21" s="5" t="n">
@@ -2320,7 +2320,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P22" s="5" t="n">
@@ -2408,14 +2408,14 @@
         <v>0.1716</v>
       </c>
       <c r="M23" s="5" t="n">
-        <v>0.231026075027885</v>
+        <v>0.229129683776917</v>
       </c>
       <c r="N23" s="5" t="n">
         <v>0.0508351004251619</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P23" s="5" t="n">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P24" s="5" t="n">
@@ -2605,7 +2605,7 @@
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P25" s="5" t="n">
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P28" s="5" t="n">
@@ -2873,7 +2873,7 @@
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P29" s="5" t="n">
@@ -2964,11 +2964,11 @@
         <v>0.231026075027885</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>0.0508351004251619</v>
+        <v>0.0515196699172839</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P30" s="5" t="n">
@@ -3059,11 +3059,11 @@
         <v>0.231026075027885</v>
       </c>
       <c r="N31" s="5" t="n">
-        <v>0.0508351004251619</v>
+        <v>0.0515196699172839</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P31" s="5" t="n">
@@ -3158,7 +3158,7 @@
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P32" s="5" t="n">
@@ -3253,7 +3253,7 @@
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P33" s="5" t="n">
@@ -3430,7 +3430,7 @@
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P36" s="5" t="n">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P37" s="5" t="n">
@@ -3616,7 +3616,7 @@
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P38" s="5" t="n">
@@ -3693,7 +3693,7 @@
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P39" s="5" t="n">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P40" s="5" t="n">
@@ -3881,7 +3881,7 @@
       </c>
       <c r="O41" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P41" s="5" t="n">
@@ -3976,7 +3976,7 @@
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P42" s="5" t="n">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="O43" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P43" s="5" t="n">
@@ -4146,7 +4146,7 @@
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P44" s="5" t="n">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P45" s="5" t="n">
@@ -4320,7 +4320,7 @@
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P46" s="5" t="n">
@@ -4415,7 +4415,7 @@
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P47" s="5" t="n">
@@ -4487,14 +4487,14 @@
         <v>0.0303</v>
       </c>
       <c r="M48" s="5" t="n">
-        <v>0.231026075027885</v>
+        <v>0.229129683776917</v>
       </c>
       <c r="N48" s="5" t="n">
         <v>0.0508351004251619</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P48" s="5" t="n">
@@ -4580,14 +4580,14 @@
         <v>0.0122</v>
       </c>
       <c r="M49" s="5" t="n">
-        <v>0.158699742317549</v>
+        <v>0.158523773309564</v>
       </c>
       <c r="N49" s="5" t="n">
         <v>0.000581408571101005</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P49" s="5" t="n">
@@ -4666,7 +4666,7 @@
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
-          <t>per-DUID</t>
+          <t>location</t>
         </is>
       </c>
       <c r="P50" s="5" t="n">
@@ -7554,7 +7554,7 @@
         <v>0.1716</v>
       </c>
       <c r="G23" s="5" t="n">
-        <v>0.231026075027885</v>
+        <v>0.229129683776917</v>
       </c>
       <c r="H23" s="5" t="n">
         <v>0.0508351004251619</v>
@@ -8005,7 +8005,7 @@
         <v>0.231026075027885</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>0.0508351004251619</v>
+        <v>0.0515196699172839</v>
       </c>
       <c r="I30" s="5" t="n">
         <v>0.1</v>
@@ -8089,7 +8089,7 @@
         <v>0.231026075027885</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>0.0508351004251619</v>
+        <v>0.0515196699172839</v>
       </c>
       <c r="I31" s="5" t="n">
         <v>0.1</v>
@@ -9206,7 +9206,7 @@
         <v>0.0303</v>
       </c>
       <c r="G48" s="5" t="n">
-        <v>0.231026075027885</v>
+        <v>0.229129683776917</v>
       </c>
       <c r="H48" s="5" t="n">
         <v>0.0508351004251619</v>
@@ -9288,7 +9288,7 @@
         <v>0.0122</v>
       </c>
       <c r="G49" s="5" t="n">
-        <v>0.158699742317549</v>
+        <v>0.158523773309564</v>
       </c>
       <c r="H49" s="5" t="n">
         <v>0.000581408571101005</v>

</xml_diff>

<commit_message>
outputs: regenerate summary.csv and workbooks with the 2026 ISP A3 columns
Added to summary.csv (after the existing 38 columns): ISPA3_REZ_ID, ISPA3_REZ_NAME,
ISPA3_MATCH, ISPA3_TRANSMISSION_Y1..Y3, ISPA3_SPILL_Y1..Y3, ISPA3_Y1..Y3_LABEL,
ISPA3_SCENARIO, ISPA3_EDITION. Workbooks: Summary sheet +8 columns (2026 ISP REZ, match,
Step Change transmission curtailment and economic spill per year), Heatmap +6.

Built from the committed caches (python -m src.main on a copy of data/); every existing
column of summary.csv and every existing workbook cell is identical to main's.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/NSW_curtailment.xlsx
+++ b/outputs/NSW_curtailment.xlsx
@@ -456,7 +456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y70"/>
+  <dimension ref="A1:AG70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -484,6 +484,14 @@
     <col width="12" customWidth="1" min="23" max="23"/>
     <col width="12" customWidth="1" min="24" max="24"/>
     <col width="12" customWidth="1" min="25" max="25"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="27" max="27"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="12" customWidth="1" min="30" max="30"/>
+    <col width="12" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="12" customWidth="1" min="33" max="33"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -612,6 +620,46 @@
           <t>Offl Avg</t>
         </is>
       </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP REZ</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP REZ match</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP Step Change Transm Curt 2029-30</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP Step Change Transm Curt 2039-40</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP Step Change Transm Curt 2049-50</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP Step Change Econ Spill 2029-30</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP Step Change Econ Spill 2039-40</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>2026 ISP Step Change Econ Spill 2049-50</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -707,6 +755,34 @@
       <c r="Y2" s="6" t="n">
         <v>0.03333333333333333</v>
       </c>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t>Wagga Wagga</t>
+        </is>
+      </c>
+      <c r="AA2" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD2" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE2" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AF2" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG2" s="6" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -802,6 +878,34 @@
       <c r="Y3" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z3" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA3" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD3" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE3" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF3" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG3" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -897,6 +1001,34 @@
       <c r="Y4" s="6" t="n">
         <v>0.03333333333333333</v>
       </c>
+      <c r="Z4" s="2" t="inlineStr">
+        <is>
+          <t>Wagga Wagga</t>
+        </is>
+      </c>
+      <c r="AA4" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD4" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE4" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AF4" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG4" s="6" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -991,6 +1123,34 @@
       </c>
       <c r="Y5" s="6" t="n">
         <v>0.06999999999999999</v>
+      </c>
+      <c r="Z5" s="2" t="inlineStr">
+        <is>
+          <t>Broken Hill</t>
+        </is>
+      </c>
+      <c r="AA5" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB5" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AC5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD5" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE5" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AF5" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AG5" s="6" t="n">
+        <v>0.46</v>
       </c>
     </row>
     <row r="6">
@@ -1041,6 +1201,14 @@
       <c r="W6" s="6" t="inlineStr"/>
       <c r="X6" s="6" t="inlineStr"/>
       <c r="Y6" s="6" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="6" t="inlineStr"/>
+      <c r="AC6" s="6" t="inlineStr"/>
+      <c r="AD6" s="6" t="inlineStr"/>
+      <c r="AE6" s="6" t="inlineStr"/>
+      <c r="AF6" s="6" t="inlineStr"/>
+      <c r="AG6" s="6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -1120,6 +1288,14 @@
       <c r="W7" s="6" t="inlineStr"/>
       <c r="X7" s="6" t="inlineStr"/>
       <c r="Y7" s="6" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="6" t="inlineStr"/>
+      <c r="AC7" s="6" t="inlineStr"/>
+      <c r="AD7" s="6" t="inlineStr"/>
+      <c r="AE7" s="6" t="inlineStr"/>
+      <c r="AF7" s="6" t="inlineStr"/>
+      <c r="AG7" s="6" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1214,6 +1390,34 @@
       </c>
       <c r="Y8" s="6" t="n">
         <v>0.14</v>
+      </c>
+      <c r="Z8" s="2" t="inlineStr">
+        <is>
+          <t>South West New South Wales</t>
+        </is>
+      </c>
+      <c r="AA8" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB8" s="6" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AC8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD8" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE8" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AF8" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG8" s="6" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="9">
@@ -1266,6 +1470,14 @@
       <c r="W9" s="6" t="inlineStr"/>
       <c r="X9" s="6" t="inlineStr"/>
       <c r="Y9" s="6" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="AA9" s="2" t="inlineStr"/>
+      <c r="AB9" s="6" t="inlineStr"/>
+      <c r="AC9" s="6" t="inlineStr"/>
+      <c r="AD9" s="6" t="inlineStr"/>
+      <c r="AE9" s="6" t="inlineStr"/>
+      <c r="AF9" s="6" t="inlineStr"/>
+      <c r="AG9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1345,6 +1557,14 @@
       <c r="W10" s="6" t="inlineStr"/>
       <c r="X10" s="6" t="inlineStr"/>
       <c r="Y10" s="6" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr"/>
+      <c r="AA10" s="2" t="inlineStr"/>
+      <c r="AB10" s="6" t="inlineStr"/>
+      <c r="AC10" s="6" t="inlineStr"/>
+      <c r="AD10" s="6" t="inlineStr"/>
+      <c r="AE10" s="6" t="inlineStr"/>
+      <c r="AF10" s="6" t="inlineStr"/>
+      <c r="AG10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1422,6 +1642,14 @@
       <c r="W11" s="6" t="inlineStr"/>
       <c r="X11" s="6" t="inlineStr"/>
       <c r="Y11" s="6" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="6" t="inlineStr"/>
+      <c r="AC11" s="6" t="inlineStr"/>
+      <c r="AD11" s="6" t="inlineStr"/>
+      <c r="AE11" s="6" t="inlineStr"/>
+      <c r="AF11" s="6" t="inlineStr"/>
+      <c r="AG11" s="6" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1471,6 +1699,14 @@
       <c r="W12" s="6" t="inlineStr"/>
       <c r="X12" s="6" t="inlineStr"/>
       <c r="Y12" s="6" t="inlineStr"/>
+      <c r="Z12" s="2" t="inlineStr"/>
+      <c r="AA12" s="2" t="inlineStr"/>
+      <c r="AB12" s="6" t="inlineStr"/>
+      <c r="AC12" s="6" t="inlineStr"/>
+      <c r="AD12" s="6" t="inlineStr"/>
+      <c r="AE12" s="6" t="inlineStr"/>
+      <c r="AF12" s="6" t="inlineStr"/>
+      <c r="AG12" s="6" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1565,6 +1801,34 @@
       </c>
       <c r="Y13" s="6" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="Z13" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA13" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD13" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE13" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF13" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG13" s="6" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="14">
@@ -1641,6 +1905,14 @@
       <c r="W14" s="6" t="inlineStr"/>
       <c r="X14" s="6" t="inlineStr"/>
       <c r="Y14" s="6" t="inlineStr"/>
+      <c r="Z14" s="2" t="inlineStr"/>
+      <c r="AA14" s="2" t="inlineStr"/>
+      <c r="AB14" s="6" t="inlineStr"/>
+      <c r="AC14" s="6" t="inlineStr"/>
+      <c r="AD14" s="6" t="inlineStr"/>
+      <c r="AE14" s="6" t="inlineStr"/>
+      <c r="AF14" s="6" t="inlineStr"/>
+      <c r="AG14" s="6" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1720,6 +1992,14 @@
       <c r="W15" s="6" t="inlineStr"/>
       <c r="X15" s="6" t="inlineStr"/>
       <c r="Y15" s="6" t="inlineStr"/>
+      <c r="Z15" s="2" t="inlineStr"/>
+      <c r="AA15" s="2" t="inlineStr"/>
+      <c r="AB15" s="6" t="inlineStr"/>
+      <c r="AC15" s="6" t="inlineStr"/>
+      <c r="AD15" s="6" t="inlineStr"/>
+      <c r="AE15" s="6" t="inlineStr"/>
+      <c r="AF15" s="6" t="inlineStr"/>
+      <c r="AG15" s="6" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1814,6 +2094,34 @@
       </c>
       <c r="Y16" s="6" t="n">
         <v>0.07666666666666667</v>
+      </c>
+      <c r="Z16" s="2" t="inlineStr">
+        <is>
+          <t>North West New South Wales</t>
+        </is>
+      </c>
+      <c r="AA16" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB16" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AC16" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AD16" s="6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AE16" s="6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AF16" s="6" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="AG16" s="6" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="17">
@@ -1894,6 +2202,14 @@
       <c r="W17" s="6" t="inlineStr"/>
       <c r="X17" s="6" t="inlineStr"/>
       <c r="Y17" s="6" t="inlineStr"/>
+      <c r="Z17" s="2" t="inlineStr"/>
+      <c r="AA17" s="2" t="inlineStr"/>
+      <c r="AB17" s="6" t="inlineStr"/>
+      <c r="AC17" s="6" t="inlineStr"/>
+      <c r="AD17" s="6" t="inlineStr"/>
+      <c r="AE17" s="6" t="inlineStr"/>
+      <c r="AF17" s="6" t="inlineStr"/>
+      <c r="AG17" s="6" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1973,6 +2289,14 @@
       <c r="W18" s="6" t="inlineStr"/>
       <c r="X18" s="6" t="inlineStr"/>
       <c r="Y18" s="6" t="inlineStr"/>
+      <c r="Z18" s="2" t="inlineStr"/>
+      <c r="AA18" s="2" t="inlineStr"/>
+      <c r="AB18" s="6" t="inlineStr"/>
+      <c r="AC18" s="6" t="inlineStr"/>
+      <c r="AD18" s="6" t="inlineStr"/>
+      <c r="AE18" s="6" t="inlineStr"/>
+      <c r="AF18" s="6" t="inlineStr"/>
+      <c r="AG18" s="6" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -2068,6 +2392,34 @@
       <c r="Y19" s="6" t="n">
         <v>0.03333333333333333</v>
       </c>
+      <c r="Z19" s="2" t="inlineStr">
+        <is>
+          <t>Wagga Wagga</t>
+        </is>
+      </c>
+      <c r="AA19" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD19" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE19" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AF19" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG19" s="6" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -2163,6 +2515,34 @@
       <c r="Y20" s="6" t="n">
         <v>0.14</v>
       </c>
+      <c r="Z20" s="2" t="inlineStr">
+        <is>
+          <t>South West New South Wales</t>
+        </is>
+      </c>
+      <c r="AA20" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB20" s="6" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AC20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD20" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE20" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AF20" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG20" s="6" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2258,6 +2638,34 @@
       <c r="Y21" s="6" t="n">
         <v>0.14</v>
       </c>
+      <c r="Z21" s="2" t="inlineStr">
+        <is>
+          <t>South West New South Wales</t>
+        </is>
+      </c>
+      <c r="AA21" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB21" s="6" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AC21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD21" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE21" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AF21" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG21" s="6" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2353,6 +2761,34 @@
       <c r="Y22" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z22" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA22" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE22" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF22" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG22" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2448,6 +2884,34 @@
       <c r="Y23" s="6" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="Z23" s="2" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="AA23" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB23" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AC23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD23" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE23" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF23" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG23" s="6" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2543,6 +3007,34 @@
       <c r="Y24" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z24" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA24" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD24" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE24" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF24" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG24" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2637,6 +3129,34 @@
       </c>
       <c r="Y25" s="6" t="n">
         <v>0.07666666666666667</v>
+      </c>
+      <c r="Z25" s="2" t="inlineStr">
+        <is>
+          <t>North West New South Wales</t>
+        </is>
+      </c>
+      <c r="AA25" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB25" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AC25" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AD25" s="6" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="AE25" s="6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AF25" s="6" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="AG25" s="6" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="26">
@@ -2687,6 +3207,14 @@
       <c r="W26" s="6" t="inlineStr"/>
       <c r="X26" s="6" t="inlineStr"/>
       <c r="Y26" s="6" t="inlineStr"/>
+      <c r="Z26" s="2" t="inlineStr"/>
+      <c r="AA26" s="2" t="inlineStr"/>
+      <c r="AB26" s="6" t="inlineStr"/>
+      <c r="AC26" s="6" t="inlineStr"/>
+      <c r="AD26" s="6" t="inlineStr"/>
+      <c r="AE26" s="6" t="inlineStr"/>
+      <c r="AF26" s="6" t="inlineStr"/>
+      <c r="AG26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2736,6 +3264,14 @@
       <c r="W27" s="6" t="inlineStr"/>
       <c r="X27" s="6" t="inlineStr"/>
       <c r="Y27" s="6" t="inlineStr"/>
+      <c r="Z27" s="2" t="inlineStr"/>
+      <c r="AA27" s="2" t="inlineStr"/>
+      <c r="AB27" s="6" t="inlineStr"/>
+      <c r="AC27" s="6" t="inlineStr"/>
+      <c r="AD27" s="6" t="inlineStr"/>
+      <c r="AE27" s="6" t="inlineStr"/>
+      <c r="AF27" s="6" t="inlineStr"/>
+      <c r="AG27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2811,6 +3347,14 @@
       <c r="W28" s="6" t="inlineStr"/>
       <c r="X28" s="6" t="inlineStr"/>
       <c r="Y28" s="6" t="inlineStr"/>
+      <c r="Z28" s="2" t="inlineStr"/>
+      <c r="AA28" s="2" t="inlineStr"/>
+      <c r="AB28" s="6" t="inlineStr"/>
+      <c r="AC28" s="6" t="inlineStr"/>
+      <c r="AD28" s="6" t="inlineStr"/>
+      <c r="AE28" s="6" t="inlineStr"/>
+      <c r="AF28" s="6" t="inlineStr"/>
+      <c r="AG28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2906,6 +3450,34 @@
       <c r="Y29" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z29" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA29" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD29" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE29" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF29" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG29" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -3001,6 +3573,34 @@
       <c r="Y30" s="6" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="Z30" s="2" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="AA30" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB30" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AC30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE30" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF30" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG30" s="6" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -3096,6 +3696,34 @@
       <c r="Y31" s="6" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="Z31" s="2" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="AA31" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB31" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AC31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE31" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF31" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG31" s="6" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -3190,6 +3818,34 @@
       </c>
       <c r="Y32" s="6" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="Z32" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA32" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE32" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF32" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG32" s="6" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="33">
@@ -3270,6 +3926,14 @@
       <c r="W33" s="6" t="inlineStr"/>
       <c r="X33" s="6" t="inlineStr"/>
       <c r="Y33" s="6" t="inlineStr"/>
+      <c r="Z33" s="2" t="inlineStr"/>
+      <c r="AA33" s="2" t="inlineStr"/>
+      <c r="AB33" s="6" t="inlineStr"/>
+      <c r="AC33" s="6" t="inlineStr"/>
+      <c r="AD33" s="6" t="inlineStr"/>
+      <c r="AE33" s="6" t="inlineStr"/>
+      <c r="AF33" s="6" t="inlineStr"/>
+      <c r="AG33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -3319,6 +3983,14 @@
       <c r="W34" s="6" t="inlineStr"/>
       <c r="X34" s="6" t="inlineStr"/>
       <c r="Y34" s="6" t="inlineStr"/>
+      <c r="Z34" s="2" t="inlineStr"/>
+      <c r="AA34" s="2" t="inlineStr"/>
+      <c r="AB34" s="6" t="inlineStr"/>
+      <c r="AC34" s="6" t="inlineStr"/>
+      <c r="AD34" s="6" t="inlineStr"/>
+      <c r="AE34" s="6" t="inlineStr"/>
+      <c r="AF34" s="6" t="inlineStr"/>
+      <c r="AG34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -3368,6 +4040,14 @@
       <c r="W35" s="6" t="inlineStr"/>
       <c r="X35" s="6" t="inlineStr"/>
       <c r="Y35" s="6" t="inlineStr"/>
+      <c r="Z35" s="2" t="inlineStr"/>
+      <c r="AA35" s="2" t="inlineStr"/>
+      <c r="AB35" s="6" t="inlineStr"/>
+      <c r="AC35" s="6" t="inlineStr"/>
+      <c r="AD35" s="6" t="inlineStr"/>
+      <c r="AE35" s="6" t="inlineStr"/>
+      <c r="AF35" s="6" t="inlineStr"/>
+      <c r="AG35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -3463,6 +4143,34 @@
       <c r="Y36" s="6" t="n">
         <v>0.14</v>
       </c>
+      <c r="Z36" s="2" t="inlineStr">
+        <is>
+          <t>South West New South Wales</t>
+        </is>
+      </c>
+      <c r="AA36" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB36" s="6" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="AC36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE36" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AF36" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG36" s="6" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3557,6 +4265,34 @@
       </c>
       <c r="Y37" s="6" t="n">
         <v>0.03333333333333333</v>
+      </c>
+      <c r="Z37" s="2" t="inlineStr">
+        <is>
+          <t>Wagga Wagga</t>
+        </is>
+      </c>
+      <c r="AA37" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE37" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AF37" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG37" s="6" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="38">
@@ -3633,6 +4369,14 @@
       <c r="W38" s="6" t="inlineStr"/>
       <c r="X38" s="6" t="inlineStr"/>
       <c r="Y38" s="6" t="inlineStr"/>
+      <c r="Z38" s="2" t="inlineStr"/>
+      <c r="AA38" s="2" t="inlineStr"/>
+      <c r="AB38" s="6" t="inlineStr"/>
+      <c r="AC38" s="6" t="inlineStr"/>
+      <c r="AD38" s="6" t="inlineStr"/>
+      <c r="AE38" s="6" t="inlineStr"/>
+      <c r="AF38" s="6" t="inlineStr"/>
+      <c r="AG38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3726,6 +4470,34 @@
       <c r="Y39" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z39" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA39" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE39" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF39" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG39" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3819,6 +4591,34 @@
       <c r="Y40" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z40" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA40" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE40" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF40" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG40" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3914,6 +4714,34 @@
       <c r="Y41" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z41" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA41" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE41" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF41" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG41" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -4008,6 +4836,34 @@
       </c>
       <c r="Y42" s="6" t="n">
         <v>0.03333333333333333</v>
+      </c>
+      <c r="Z42" s="2" t="inlineStr">
+        <is>
+          <t>Wagga Wagga</t>
+        </is>
+      </c>
+      <c r="AA42" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE42" s="6" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AF42" s="6" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AG42" s="6" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="43">
@@ -4086,6 +4942,14 @@
       <c r="W43" s="6" t="inlineStr"/>
       <c r="X43" s="6" t="inlineStr"/>
       <c r="Y43" s="6" t="inlineStr"/>
+      <c r="Z43" s="2" t="inlineStr"/>
+      <c r="AA43" s="2" t="inlineStr"/>
+      <c r="AB43" s="6" t="inlineStr"/>
+      <c r="AC43" s="6" t="inlineStr"/>
+      <c r="AD43" s="6" t="inlineStr"/>
+      <c r="AE43" s="6" t="inlineStr"/>
+      <c r="AF43" s="6" t="inlineStr"/>
+      <c r="AG43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -4163,6 +5027,14 @@
       <c r="W44" s="6" t="inlineStr"/>
       <c r="X44" s="6" t="inlineStr"/>
       <c r="Y44" s="6" t="inlineStr"/>
+      <c r="Z44" s="2" t="inlineStr"/>
+      <c r="AA44" s="2" t="inlineStr"/>
+      <c r="AB44" s="6" t="inlineStr"/>
+      <c r="AC44" s="6" t="inlineStr"/>
+      <c r="AD44" s="6" t="inlineStr"/>
+      <c r="AE44" s="6" t="inlineStr"/>
+      <c r="AF44" s="6" t="inlineStr"/>
+      <c r="AG44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -4258,6 +5130,34 @@
       <c r="Y45" s="6" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="Z45" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA45" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE45" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF45" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG45" s="6" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -4352,6 +5252,34 @@
       </c>
       <c r="Y46" s="6" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="Z46" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA46" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE46" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF46" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG46" s="6" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="47">
@@ -4432,6 +5360,14 @@
       <c r="W47" s="6" t="inlineStr"/>
       <c r="X47" s="6" t="inlineStr"/>
       <c r="Y47" s="6" t="inlineStr"/>
+      <c r="Z47" s="2" t="inlineStr"/>
+      <c r="AA47" s="2" t="inlineStr"/>
+      <c r="AB47" s="6" t="inlineStr"/>
+      <c r="AC47" s="6" t="inlineStr"/>
+      <c r="AD47" s="6" t="inlineStr"/>
+      <c r="AE47" s="6" t="inlineStr"/>
+      <c r="AF47" s="6" t="inlineStr"/>
+      <c r="AG47" s="6" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -4526,6 +5462,34 @@
       </c>
       <c r="Y48" s="6" t="n">
         <v>0.2533333333333334</v>
+      </c>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="AA48" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB48" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AC48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE48" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF48" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG48" s="6" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="49">
@@ -4604,6 +5568,14 @@
       <c r="W49" s="6" t="inlineStr"/>
       <c r="X49" s="6" t="inlineStr"/>
       <c r="Y49" s="6" t="inlineStr"/>
+      <c r="Z49" s="2" t="inlineStr"/>
+      <c r="AA49" s="2" t="inlineStr"/>
+      <c r="AB49" s="6" t="inlineStr"/>
+      <c r="AC49" s="6" t="inlineStr"/>
+      <c r="AD49" s="6" t="inlineStr"/>
+      <c r="AE49" s="6" t="inlineStr"/>
+      <c r="AF49" s="6" t="inlineStr"/>
+      <c r="AG49" s="6" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -4683,6 +5655,14 @@
       <c r="W50" s="6" t="inlineStr"/>
       <c r="X50" s="6" t="inlineStr"/>
       <c r="Y50" s="6" t="inlineStr"/>
+      <c r="Z50" s="2" t="inlineStr"/>
+      <c r="AA50" s="2" t="inlineStr"/>
+      <c r="AB50" s="6" t="inlineStr"/>
+      <c r="AC50" s="6" t="inlineStr"/>
+      <c r="AD50" s="6" t="inlineStr"/>
+      <c r="AE50" s="6" t="inlineStr"/>
+      <c r="AF50" s="6" t="inlineStr"/>
+      <c r="AG50" s="6" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -4748,6 +5728,14 @@
       <c r="W51" s="6" t="inlineStr"/>
       <c r="X51" s="6" t="inlineStr"/>
       <c r="Y51" s="6" t="inlineStr"/>
+      <c r="Z51" s="2" t="inlineStr"/>
+      <c r="AA51" s="2" t="inlineStr"/>
+      <c r="AB51" s="6" t="inlineStr"/>
+      <c r="AC51" s="6" t="inlineStr"/>
+      <c r="AD51" s="6" t="inlineStr"/>
+      <c r="AE51" s="6" t="inlineStr"/>
+      <c r="AF51" s="6" t="inlineStr"/>
+      <c r="AG51" s="6" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -4813,6 +5801,14 @@
       <c r="W52" s="6" t="inlineStr"/>
       <c r="X52" s="6" t="inlineStr"/>
       <c r="Y52" s="6" t="inlineStr"/>
+      <c r="Z52" s="2" t="inlineStr"/>
+      <c r="AA52" s="2" t="inlineStr"/>
+      <c r="AB52" s="6" t="inlineStr"/>
+      <c r="AC52" s="6" t="inlineStr"/>
+      <c r="AD52" s="6" t="inlineStr"/>
+      <c r="AE52" s="6" t="inlineStr"/>
+      <c r="AF52" s="6" t="inlineStr"/>
+      <c r="AG52" s="6" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -4894,6 +5890,34 @@
       <c r="Y53" s="6" t="n">
         <v>0.05666666666666667</v>
       </c>
+      <c r="Z53" s="2" t="inlineStr">
+        <is>
+          <t>Cooma-Monaro</t>
+        </is>
+      </c>
+      <c r="AA53" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE53" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AF53" s="6" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AG53" s="6" t="n">
+        <v>0.2</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -4974,6 +5998,34 @@
       </c>
       <c r="Y54" s="6" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="Z54" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA54" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE54" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF54" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG54" s="6" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="55">
@@ -5024,6 +6076,14 @@
       <c r="W55" s="6" t="inlineStr"/>
       <c r="X55" s="6" t="inlineStr"/>
       <c r="Y55" s="6" t="inlineStr"/>
+      <c r="Z55" s="2" t="inlineStr"/>
+      <c r="AA55" s="2" t="inlineStr"/>
+      <c r="AB55" s="6" t="inlineStr"/>
+      <c r="AC55" s="6" t="inlineStr"/>
+      <c r="AD55" s="6" t="inlineStr"/>
+      <c r="AE55" s="6" t="inlineStr"/>
+      <c r="AF55" s="6" t="inlineStr"/>
+      <c r="AG55" s="6" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -5089,6 +6149,14 @@
       <c r="W56" s="6" t="inlineStr"/>
       <c r="X56" s="6" t="inlineStr"/>
       <c r="Y56" s="6" t="inlineStr"/>
+      <c r="Z56" s="2" t="inlineStr"/>
+      <c r="AA56" s="2" t="inlineStr"/>
+      <c r="AB56" s="6" t="inlineStr"/>
+      <c r="AC56" s="6" t="inlineStr"/>
+      <c r="AD56" s="6" t="inlineStr"/>
+      <c r="AE56" s="6" t="inlineStr"/>
+      <c r="AF56" s="6" t="inlineStr"/>
+      <c r="AG56" s="6" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -5152,6 +6220,14 @@
       <c r="W57" s="6" t="inlineStr"/>
       <c r="X57" s="6" t="inlineStr"/>
       <c r="Y57" s="6" t="inlineStr"/>
+      <c r="Z57" s="2" t="inlineStr"/>
+      <c r="AA57" s="2" t="inlineStr"/>
+      <c r="AB57" s="6" t="inlineStr"/>
+      <c r="AC57" s="6" t="inlineStr"/>
+      <c r="AD57" s="6" t="inlineStr"/>
+      <c r="AE57" s="6" t="inlineStr"/>
+      <c r="AF57" s="6" t="inlineStr"/>
+      <c r="AG57" s="6" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -5215,6 +6291,14 @@
       <c r="W58" s="6" t="inlineStr"/>
       <c r="X58" s="6" t="inlineStr"/>
       <c r="Y58" s="6" t="inlineStr"/>
+      <c r="Z58" s="2" t="inlineStr"/>
+      <c r="AA58" s="2" t="inlineStr"/>
+      <c r="AB58" s="6" t="inlineStr"/>
+      <c r="AC58" s="6" t="inlineStr"/>
+      <c r="AD58" s="6" t="inlineStr"/>
+      <c r="AE58" s="6" t="inlineStr"/>
+      <c r="AF58" s="6" t="inlineStr"/>
+      <c r="AG58" s="6" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -5280,6 +6364,14 @@
       <c r="W59" s="6" t="inlineStr"/>
       <c r="X59" s="6" t="inlineStr"/>
       <c r="Y59" s="6" t="inlineStr"/>
+      <c r="Z59" s="2" t="inlineStr"/>
+      <c r="AA59" s="2" t="inlineStr"/>
+      <c r="AB59" s="6" t="inlineStr"/>
+      <c r="AC59" s="6" t="inlineStr"/>
+      <c r="AD59" s="6" t="inlineStr"/>
+      <c r="AE59" s="6" t="inlineStr"/>
+      <c r="AF59" s="6" t="inlineStr"/>
+      <c r="AG59" s="6" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -5329,6 +6421,14 @@
       <c r="W60" s="6" t="inlineStr"/>
       <c r="X60" s="6" t="inlineStr"/>
       <c r="Y60" s="6" t="inlineStr"/>
+      <c r="Z60" s="2" t="inlineStr"/>
+      <c r="AA60" s="2" t="inlineStr"/>
+      <c r="AB60" s="6" t="inlineStr"/>
+      <c r="AC60" s="6" t="inlineStr"/>
+      <c r="AD60" s="6" t="inlineStr"/>
+      <c r="AE60" s="6" t="inlineStr"/>
+      <c r="AF60" s="6" t="inlineStr"/>
+      <c r="AG60" s="6" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -5409,6 +6509,34 @@
       </c>
       <c r="Y61" s="6" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="Z61" s="2" t="inlineStr">
+        <is>
+          <t>Central-West Orana</t>
+        </is>
+      </c>
+      <c r="AA61" s="2" t="inlineStr">
+        <is>
+          <t>renamed</t>
+        </is>
+      </c>
+      <c r="AB61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD61" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE61" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AF61" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AG61" s="6" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="62">
@@ -5475,6 +6603,14 @@
       <c r="W62" s="6" t="inlineStr"/>
       <c r="X62" s="6" t="inlineStr"/>
       <c r="Y62" s="6" t="inlineStr"/>
+      <c r="Z62" s="2" t="inlineStr"/>
+      <c r="AA62" s="2" t="inlineStr"/>
+      <c r="AB62" s="6" t="inlineStr"/>
+      <c r="AC62" s="6" t="inlineStr"/>
+      <c r="AD62" s="6" t="inlineStr"/>
+      <c r="AE62" s="6" t="inlineStr"/>
+      <c r="AF62" s="6" t="inlineStr"/>
+      <c r="AG62" s="6" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -5540,6 +6676,14 @@
       <c r="W63" s="6" t="inlineStr"/>
       <c r="X63" s="6" t="inlineStr"/>
       <c r="Y63" s="6" t="inlineStr"/>
+      <c r="Z63" s="2" t="inlineStr"/>
+      <c r="AA63" s="2" t="inlineStr"/>
+      <c r="AB63" s="6" t="inlineStr"/>
+      <c r="AC63" s="6" t="inlineStr"/>
+      <c r="AD63" s="6" t="inlineStr"/>
+      <c r="AE63" s="6" t="inlineStr"/>
+      <c r="AF63" s="6" t="inlineStr"/>
+      <c r="AG63" s="6" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -5605,6 +6749,14 @@
       <c r="W64" s="6" t="inlineStr"/>
       <c r="X64" s="6" t="inlineStr"/>
       <c r="Y64" s="6" t="inlineStr"/>
+      <c r="Z64" s="2" t="inlineStr"/>
+      <c r="AA64" s="2" t="inlineStr"/>
+      <c r="AB64" s="6" t="inlineStr"/>
+      <c r="AC64" s="6" t="inlineStr"/>
+      <c r="AD64" s="6" t="inlineStr"/>
+      <c r="AE64" s="6" t="inlineStr"/>
+      <c r="AF64" s="6" t="inlineStr"/>
+      <c r="AG64" s="6" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -5670,6 +6822,14 @@
       <c r="W65" s="6" t="inlineStr"/>
       <c r="X65" s="6" t="inlineStr"/>
       <c r="Y65" s="6" t="inlineStr"/>
+      <c r="Z65" s="2" t="inlineStr"/>
+      <c r="AA65" s="2" t="inlineStr"/>
+      <c r="AB65" s="6" t="inlineStr"/>
+      <c r="AC65" s="6" t="inlineStr"/>
+      <c r="AD65" s="6" t="inlineStr"/>
+      <c r="AE65" s="6" t="inlineStr"/>
+      <c r="AF65" s="6" t="inlineStr"/>
+      <c r="AG65" s="6" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -5751,6 +6911,34 @@
       <c r="Y66" s="6" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="Z66" s="2" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="AA66" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB66" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AC66" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD66" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE66" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF66" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG66" s="6" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -5831,6 +7019,34 @@
       </c>
       <c r="Y67" s="6" t="n">
         <v>0.06999999999999999</v>
+      </c>
+      <c r="Z67" s="2" t="inlineStr">
+        <is>
+          <t>Broken Hill</t>
+        </is>
+      </c>
+      <c r="AA67" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB67" s="6" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AC67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD67" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE67" s="6" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AF67" s="6" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AG67" s="6" t="n">
+        <v>0.46</v>
       </c>
     </row>
     <row r="68">
@@ -5897,6 +7113,14 @@
       <c r="W68" s="6" t="inlineStr"/>
       <c r="X68" s="6" t="inlineStr"/>
       <c r="Y68" s="6" t="inlineStr"/>
+      <c r="Z68" s="2" t="inlineStr"/>
+      <c r="AA68" s="2" t="inlineStr"/>
+      <c r="AB68" s="6" t="inlineStr"/>
+      <c r="AC68" s="6" t="inlineStr"/>
+      <c r="AD68" s="6" t="inlineStr"/>
+      <c r="AE68" s="6" t="inlineStr"/>
+      <c r="AF68" s="6" t="inlineStr"/>
+      <c r="AG68" s="6" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -5977,6 +7201,34 @@
       </c>
       <c r="Y69" s="6" t="n">
         <v>0.2533333333333334</v>
+      </c>
+      <c r="Z69" s="2" t="inlineStr">
+        <is>
+          <t>New England</t>
+        </is>
+      </c>
+      <c r="AA69" s="2" t="inlineStr">
+        <is>
+          <t>exact</t>
+        </is>
+      </c>
+      <c r="AB69" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AC69" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AD69" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE69" s="6" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AF69" s="6" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AG69" s="6" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="70">
@@ -6043,6 +7295,14 @@
       <c r="W70" s="6" t="inlineStr"/>
       <c r="X70" s="6" t="inlineStr"/>
       <c r="Y70" s="6" t="inlineStr"/>
+      <c r="Z70" s="2" t="inlineStr"/>
+      <c r="AA70" s="2" t="inlineStr"/>
+      <c r="AB70" s="6" t="inlineStr"/>
+      <c r="AC70" s="6" t="inlineStr"/>
+      <c r="AD70" s="6" t="inlineStr"/>
+      <c r="AE70" s="6" t="inlineStr"/>
+      <c r="AF70" s="6" t="inlineStr"/>
+      <c r="AG70" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6055,7 +7315,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V70"/>
+  <dimension ref="A1:AB70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6080,6 +7340,12 @@
     <col width="14" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
     <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="14" customWidth="1" min="23" max="23"/>
+    <col width="14" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6193,6 +7459,36 @@
           <t>ISP_OFFLOADING_AVG</t>
         </is>
       </c>
+      <c r="W1" s="7" t="inlineStr">
+        <is>
+          <t>ISPA3_TRANSMISSION_Y1</t>
+        </is>
+      </c>
+      <c r="X1" s="7" t="inlineStr">
+        <is>
+          <t>ISPA3_TRANSMISSION_Y2</t>
+        </is>
+      </c>
+      <c r="Y1" s="7" t="inlineStr">
+        <is>
+          <t>ISPA3_TRANSMISSION_Y3</t>
+        </is>
+      </c>
+      <c r="Z1" s="7" t="inlineStr">
+        <is>
+          <t>ISPA3_SPILL_Y1</t>
+        </is>
+      </c>
+      <c r="AA1" s="7" t="inlineStr">
+        <is>
+          <t>ISPA3_SPILL_Y2</t>
+        </is>
+      </c>
+      <c r="AB1" s="7" t="inlineStr">
+        <is>
+          <t>ISPA3_SPILL_Y3</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
@@ -6277,6 +7573,24 @@
       <c r="V2" s="5" t="n">
         <v>0.03333333333333333</v>
       </c>
+      <c r="W2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA2" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AB2" s="5" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
@@ -6361,6 +7675,24 @@
       <c r="V3" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA3" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB3" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
@@ -6445,6 +7777,24 @@
       <c r="V4" s="5" t="n">
         <v>0.03333333333333333</v>
       </c>
+      <c r="W4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z4" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA4" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AB4" s="5" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
@@ -6528,6 +7878,24 @@
       </c>
       <c r="V5" s="5" t="n">
         <v>0.06999999999999999</v>
+      </c>
+      <c r="W5" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="X5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AA5" s="5" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AB5" s="5" t="n">
+        <v>0.46</v>
       </c>
     </row>
     <row r="6">
@@ -6565,6 +7933,12 @@
       <c r="T6" s="5" t="inlineStr"/>
       <c r="U6" s="5" t="inlineStr"/>
       <c r="V6" s="5" t="inlineStr"/>
+      <c r="W6" s="5" t="inlineStr"/>
+      <c r="X6" s="5" t="inlineStr"/>
+      <c r="Y6" s="5" t="inlineStr"/>
+      <c r="Z6" s="5" t="inlineStr"/>
+      <c r="AA6" s="5" t="inlineStr"/>
+      <c r="AB6" s="5" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
@@ -6609,6 +7983,12 @@
       <c r="T7" s="5" t="inlineStr"/>
       <c r="U7" s="5" t="inlineStr"/>
       <c r="V7" s="5" t="inlineStr"/>
+      <c r="W7" s="5" t="inlineStr"/>
+      <c r="X7" s="5" t="inlineStr"/>
+      <c r="Y7" s="5" t="inlineStr"/>
+      <c r="Z7" s="5" t="inlineStr"/>
+      <c r="AA7" s="5" t="inlineStr"/>
+      <c r="AB7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
@@ -6692,6 +8072,24 @@
       </c>
       <c r="V8" s="5" t="n">
         <v>0.14</v>
+      </c>
+      <c r="W8" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="X8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AA8" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB8" s="5" t="n">
+        <v>0.08</v>
       </c>
     </row>
     <row r="9">
@@ -6731,6 +8129,12 @@
       <c r="T9" s="5" t="inlineStr"/>
       <c r="U9" s="5" t="inlineStr"/>
       <c r="V9" s="5" t="inlineStr"/>
+      <c r="W9" s="5" t="inlineStr"/>
+      <c r="X9" s="5" t="inlineStr"/>
+      <c r="Y9" s="5" t="inlineStr"/>
+      <c r="Z9" s="5" t="inlineStr"/>
+      <c r="AA9" s="5" t="inlineStr"/>
+      <c r="AB9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
@@ -6775,6 +8179,12 @@
       <c r="T10" s="5" t="inlineStr"/>
       <c r="U10" s="5" t="inlineStr"/>
       <c r="V10" s="5" t="inlineStr"/>
+      <c r="W10" s="5" t="inlineStr"/>
+      <c r="X10" s="5" t="inlineStr"/>
+      <c r="Y10" s="5" t="inlineStr"/>
+      <c r="Z10" s="5" t="inlineStr"/>
+      <c r="AA10" s="5" t="inlineStr"/>
+      <c r="AB10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
@@ -6817,6 +8227,12 @@
       <c r="T11" s="5" t="inlineStr"/>
       <c r="U11" s="5" t="inlineStr"/>
       <c r="V11" s="5" t="inlineStr"/>
+      <c r="W11" s="5" t="inlineStr"/>
+      <c r="X11" s="5" t="inlineStr"/>
+      <c r="Y11" s="5" t="inlineStr"/>
+      <c r="Z11" s="5" t="inlineStr"/>
+      <c r="AA11" s="5" t="inlineStr"/>
+      <c r="AB11" s="5" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
@@ -6853,6 +8269,12 @@
       <c r="T12" s="5" t="inlineStr"/>
       <c r="U12" s="5" t="inlineStr"/>
       <c r="V12" s="5" t="inlineStr"/>
+      <c r="W12" s="5" t="inlineStr"/>
+      <c r="X12" s="5" t="inlineStr"/>
+      <c r="Y12" s="5" t="inlineStr"/>
+      <c r="Z12" s="5" t="inlineStr"/>
+      <c r="AA12" s="5" t="inlineStr"/>
+      <c r="AB12" s="5" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
@@ -6936,6 +8358,24 @@
       </c>
       <c r="V13" s="5" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="W13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA13" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB13" s="5" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="14">
@@ -6977,6 +8417,12 @@
       <c r="T14" s="5" t="inlineStr"/>
       <c r="U14" s="5" t="inlineStr"/>
       <c r="V14" s="5" t="inlineStr"/>
+      <c r="W14" s="5" t="inlineStr"/>
+      <c r="X14" s="5" t="inlineStr"/>
+      <c r="Y14" s="5" t="inlineStr"/>
+      <c r="Z14" s="5" t="inlineStr"/>
+      <c r="AA14" s="5" t="inlineStr"/>
+      <c r="AB14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
@@ -7021,6 +8467,12 @@
       <c r="T15" s="5" t="inlineStr"/>
       <c r="U15" s="5" t="inlineStr"/>
       <c r="V15" s="5" t="inlineStr"/>
+      <c r="W15" s="5" t="inlineStr"/>
+      <c r="X15" s="5" t="inlineStr"/>
+      <c r="Y15" s="5" t="inlineStr"/>
+      <c r="Z15" s="5" t="inlineStr"/>
+      <c r="AA15" s="5" t="inlineStr"/>
+      <c r="AB15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
@@ -7104,6 +8556,24 @@
       </c>
       <c r="V16" s="5" t="n">
         <v>0.07666666666666667</v>
+      </c>
+      <c r="W16" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="X16" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Y16" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Z16" s="5" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AA16" s="5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="AB16" s="5" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="17">
@@ -7149,6 +8619,12 @@
       <c r="T17" s="5" t="inlineStr"/>
       <c r="U17" s="5" t="inlineStr"/>
       <c r="V17" s="5" t="inlineStr"/>
+      <c r="W17" s="5" t="inlineStr"/>
+      <c r="X17" s="5" t="inlineStr"/>
+      <c r="Y17" s="5" t="inlineStr"/>
+      <c r="Z17" s="5" t="inlineStr"/>
+      <c r="AA17" s="5" t="inlineStr"/>
+      <c r="AB17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
@@ -7193,6 +8669,12 @@
       <c r="T18" s="5" t="inlineStr"/>
       <c r="U18" s="5" t="inlineStr"/>
       <c r="V18" s="5" t="inlineStr"/>
+      <c r="W18" s="5" t="inlineStr"/>
+      <c r="X18" s="5" t="inlineStr"/>
+      <c r="Y18" s="5" t="inlineStr"/>
+      <c r="Z18" s="5" t="inlineStr"/>
+      <c r="AA18" s="5" t="inlineStr"/>
+      <c r="AB18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="inlineStr">
@@ -7277,6 +8759,24 @@
       <c r="V19" s="5" t="n">
         <v>0.03333333333333333</v>
       </c>
+      <c r="W19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA19" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AB19" s="5" t="n">
+        <v>0.05</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="8" t="inlineStr">
@@ -7361,6 +8861,24 @@
       <c r="V20" s="5" t="n">
         <v>0.14</v>
       </c>
+      <c r="W20" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="X20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AA20" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB20" s="5" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="8" t="inlineStr">
@@ -7445,6 +8963,24 @@
       <c r="V21" s="5" t="n">
         <v>0.14</v>
       </c>
+      <c r="W21" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="X21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z21" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AA21" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB21" s="5" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="8" t="inlineStr">
@@ -7529,6 +9065,24 @@
       <c r="V22" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA22" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB22" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
@@ -7613,6 +9167,24 @@
       <c r="V23" s="5" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="W23" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="X23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AA23" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AB23" s="5" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
@@ -7697,6 +9269,24 @@
       <c r="V24" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA24" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB24" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
@@ -7780,6 +9370,24 @@
       </c>
       <c r="V25" s="5" t="n">
         <v>0.07666666666666667</v>
+      </c>
+      <c r="W25" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="X25" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="Y25" s="5" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="Z25" s="5" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AA25" s="5" t="n">
+        <v>0.36</v>
+      </c>
+      <c r="AB25" s="5" t="n">
+        <v>0.52</v>
       </c>
     </row>
     <row r="26">
@@ -7817,6 +9425,12 @@
       <c r="T26" s="5" t="inlineStr"/>
       <c r="U26" s="5" t="inlineStr"/>
       <c r="V26" s="5" t="inlineStr"/>
+      <c r="W26" s="5" t="inlineStr"/>
+      <c r="X26" s="5" t="inlineStr"/>
+      <c r="Y26" s="5" t="inlineStr"/>
+      <c r="Z26" s="5" t="inlineStr"/>
+      <c r="AA26" s="5" t="inlineStr"/>
+      <c r="AB26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="inlineStr">
@@ -7853,6 +9467,12 @@
       <c r="T27" s="5" t="inlineStr"/>
       <c r="U27" s="5" t="inlineStr"/>
       <c r="V27" s="5" t="inlineStr"/>
+      <c r="W27" s="5" t="inlineStr"/>
+      <c r="X27" s="5" t="inlineStr"/>
+      <c r="Y27" s="5" t="inlineStr"/>
+      <c r="Z27" s="5" t="inlineStr"/>
+      <c r="AA27" s="5" t="inlineStr"/>
+      <c r="AB27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="inlineStr">
@@ -7893,6 +9513,12 @@
       <c r="T28" s="5" t="inlineStr"/>
       <c r="U28" s="5" t="inlineStr"/>
       <c r="V28" s="5" t="inlineStr"/>
+      <c r="W28" s="5" t="inlineStr"/>
+      <c r="X28" s="5" t="inlineStr"/>
+      <c r="Y28" s="5" t="inlineStr"/>
+      <c r="Z28" s="5" t="inlineStr"/>
+      <c r="AA28" s="5" t="inlineStr"/>
+      <c r="AB28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="inlineStr">
@@ -7977,6 +9603,24 @@
       <c r="V29" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA29" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB29" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="8" t="inlineStr">
@@ -8061,6 +9705,24 @@
       <c r="V30" s="5" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="W30" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="X30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AA30" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AB30" s="5" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
@@ -8145,6 +9807,24 @@
       <c r="V31" s="5" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="W31" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="X31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AA31" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AB31" s="5" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="8" t="inlineStr">
@@ -8228,6 +9908,24 @@
       </c>
       <c r="V32" s="5" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="W32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z32" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA32" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB32" s="5" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="33">
@@ -8273,6 +9971,12 @@
       <c r="T33" s="5" t="inlineStr"/>
       <c r="U33" s="5" t="inlineStr"/>
       <c r="V33" s="5" t="inlineStr"/>
+      <c r="W33" s="5" t="inlineStr"/>
+      <c r="X33" s="5" t="inlineStr"/>
+      <c r="Y33" s="5" t="inlineStr"/>
+      <c r="Z33" s="5" t="inlineStr"/>
+      <c r="AA33" s="5" t="inlineStr"/>
+      <c r="AB33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
@@ -8309,6 +10013,12 @@
       <c r="T34" s="5" t="inlineStr"/>
       <c r="U34" s="5" t="inlineStr"/>
       <c r="V34" s="5" t="inlineStr"/>
+      <c r="W34" s="5" t="inlineStr"/>
+      <c r="X34" s="5" t="inlineStr"/>
+      <c r="Y34" s="5" t="inlineStr"/>
+      <c r="Z34" s="5" t="inlineStr"/>
+      <c r="AA34" s="5" t="inlineStr"/>
+      <c r="AB34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
@@ -8345,6 +10055,12 @@
       <c r="T35" s="5" t="inlineStr"/>
       <c r="U35" s="5" t="inlineStr"/>
       <c r="V35" s="5" t="inlineStr"/>
+      <c r="W35" s="5" t="inlineStr"/>
+      <c r="X35" s="5" t="inlineStr"/>
+      <c r="Y35" s="5" t="inlineStr"/>
+      <c r="Z35" s="5" t="inlineStr"/>
+      <c r="AA35" s="5" t="inlineStr"/>
+      <c r="AB35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
@@ -8429,6 +10145,24 @@
       <c r="V36" s="5" t="n">
         <v>0.14</v>
       </c>
+      <c r="W36" s="5" t="n">
+        <v>0.17</v>
+      </c>
+      <c r="X36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AA36" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB36" s="5" t="n">
+        <v>0.08</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="8" t="inlineStr">
@@ -8512,6 +10246,24 @@
       </c>
       <c r="V37" s="5" t="n">
         <v>0.03333333333333333</v>
+      </c>
+      <c r="W37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA37" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AB37" s="5" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="38">
@@ -8553,6 +10305,12 @@
       <c r="T38" s="5" t="inlineStr"/>
       <c r="U38" s="5" t="inlineStr"/>
       <c r="V38" s="5" t="inlineStr"/>
+      <c r="W38" s="5" t="inlineStr"/>
+      <c r="X38" s="5" t="inlineStr"/>
+      <c r="Y38" s="5" t="inlineStr"/>
+      <c r="Z38" s="5" t="inlineStr"/>
+      <c r="AA38" s="5" t="inlineStr"/>
+      <c r="AB38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="inlineStr">
@@ -8635,6 +10393,24 @@
       <c r="V39" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y39" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z39" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA39" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB39" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
@@ -8717,6 +10493,24 @@
       <c r="V40" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y40" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA40" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB40" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
@@ -8801,6 +10595,24 @@
       <c r="V41" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y41" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z41" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA41" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB41" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="8" t="inlineStr">
@@ -8884,6 +10696,24 @@
       </c>
       <c r="V42" s="5" t="n">
         <v>0.03333333333333333</v>
+      </c>
+      <c r="W42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" s="5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AA42" s="5" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="AB42" s="5" t="n">
+        <v>0.05</v>
       </c>
     </row>
     <row r="43">
@@ -8927,6 +10757,12 @@
       <c r="T43" s="5" t="inlineStr"/>
       <c r="U43" s="5" t="inlineStr"/>
       <c r="V43" s="5" t="inlineStr"/>
+      <c r="W43" s="5" t="inlineStr"/>
+      <c r="X43" s="5" t="inlineStr"/>
+      <c r="Y43" s="5" t="inlineStr"/>
+      <c r="Z43" s="5" t="inlineStr"/>
+      <c r="AA43" s="5" t="inlineStr"/>
+      <c r="AB43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
@@ -8969,6 +10805,12 @@
       <c r="T44" s="5" t="inlineStr"/>
       <c r="U44" s="5" t="inlineStr"/>
       <c r="V44" s="5" t="inlineStr"/>
+      <c r="W44" s="5" t="inlineStr"/>
+      <c r="X44" s="5" t="inlineStr"/>
+      <c r="Y44" s="5" t="inlineStr"/>
+      <c r="Z44" s="5" t="inlineStr"/>
+      <c r="AA44" s="5" t="inlineStr"/>
+      <c r="AB44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
@@ -9053,6 +10895,24 @@
       <c r="V45" s="5" t="n">
         <v>0.2066666666666667</v>
       </c>
+      <c r="W45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA45" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB45" s="5" t="n">
+        <v>0.11</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
@@ -9136,6 +10996,24 @@
       </c>
       <c r="V46" s="5" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="W46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y46" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z46" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA46" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB46" s="5" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="47">
@@ -9181,6 +11059,12 @@
       <c r="T47" s="5" t="inlineStr"/>
       <c r="U47" s="5" t="inlineStr"/>
       <c r="V47" s="5" t="inlineStr"/>
+      <c r="W47" s="5" t="inlineStr"/>
+      <c r="X47" s="5" t="inlineStr"/>
+      <c r="Y47" s="5" t="inlineStr"/>
+      <c r="Z47" s="5" t="inlineStr"/>
+      <c r="AA47" s="5" t="inlineStr"/>
+      <c r="AB47" s="5" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
@@ -9264,6 +11148,24 @@
       </c>
       <c r="V48" s="5" t="n">
         <v>0.2533333333333334</v>
+      </c>
+      <c r="W48" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="X48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z48" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AA48" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AB48" s="5" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="49">
@@ -9307,6 +11209,12 @@
       <c r="T49" s="5" t="inlineStr"/>
       <c r="U49" s="5" t="inlineStr"/>
       <c r="V49" s="5" t="inlineStr"/>
+      <c r="W49" s="5" t="inlineStr"/>
+      <c r="X49" s="5" t="inlineStr"/>
+      <c r="Y49" s="5" t="inlineStr"/>
+      <c r="Z49" s="5" t="inlineStr"/>
+      <c r="AA49" s="5" t="inlineStr"/>
+      <c r="AB49" s="5" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
@@ -9351,6 +11259,12 @@
       <c r="T50" s="5" t="inlineStr"/>
       <c r="U50" s="5" t="inlineStr"/>
       <c r="V50" s="5" t="inlineStr"/>
+      <c r="W50" s="5" t="inlineStr"/>
+      <c r="X50" s="5" t="inlineStr"/>
+      <c r="Y50" s="5" t="inlineStr"/>
+      <c r="Z50" s="5" t="inlineStr"/>
+      <c r="AA50" s="5" t="inlineStr"/>
+      <c r="AB50" s="5" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
@@ -9391,6 +11305,12 @@
       <c r="T51" s="5" t="inlineStr"/>
       <c r="U51" s="5" t="inlineStr"/>
       <c r="V51" s="5" t="inlineStr"/>
+      <c r="W51" s="5" t="inlineStr"/>
+      <c r="X51" s="5" t="inlineStr"/>
+      <c r="Y51" s="5" t="inlineStr"/>
+      <c r="Z51" s="5" t="inlineStr"/>
+      <c r="AA51" s="5" t="inlineStr"/>
+      <c r="AB51" s="5" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="inlineStr">
@@ -9431,6 +11351,12 @@
       <c r="T52" s="5" t="inlineStr"/>
       <c r="U52" s="5" t="inlineStr"/>
       <c r="V52" s="5" t="inlineStr"/>
+      <c r="W52" s="5" t="inlineStr"/>
+      <c r="X52" s="5" t="inlineStr"/>
+      <c r="Y52" s="5" t="inlineStr"/>
+      <c r="Z52" s="5" t="inlineStr"/>
+      <c r="AA52" s="5" t="inlineStr"/>
+      <c r="AB52" s="5" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
@@ -9510,6 +11436,24 @@
       </c>
       <c r="V53" s="5" t="n">
         <v>0.05666666666666667</v>
+      </c>
+      <c r="W53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y53" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z53" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AA53" s="5" t="n">
+        <v>0.22</v>
+      </c>
+      <c r="AB53" s="5" t="n">
+        <v>0.2</v>
       </c>
     </row>
     <row r="54">
@@ -9590,6 +11534,24 @@
       </c>
       <c r="V54" s="5" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="W54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y54" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z54" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA54" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB54" s="5" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="55">
@@ -9627,6 +11589,12 @@
       <c r="T55" s="5" t="inlineStr"/>
       <c r="U55" s="5" t="inlineStr"/>
       <c r="V55" s="5" t="inlineStr"/>
+      <c r="W55" s="5" t="inlineStr"/>
+      <c r="X55" s="5" t="inlineStr"/>
+      <c r="Y55" s="5" t="inlineStr"/>
+      <c r="Z55" s="5" t="inlineStr"/>
+      <c r="AA55" s="5" t="inlineStr"/>
+      <c r="AB55" s="5" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
@@ -9667,6 +11635,12 @@
       <c r="T56" s="5" t="inlineStr"/>
       <c r="U56" s="5" t="inlineStr"/>
       <c r="V56" s="5" t="inlineStr"/>
+      <c r="W56" s="5" t="inlineStr"/>
+      <c r="X56" s="5" t="inlineStr"/>
+      <c r="Y56" s="5" t="inlineStr"/>
+      <c r="Z56" s="5" t="inlineStr"/>
+      <c r="AA56" s="5" t="inlineStr"/>
+      <c r="AB56" s="5" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="inlineStr">
@@ -9705,6 +11679,12 @@
       <c r="T57" s="5" t="inlineStr"/>
       <c r="U57" s="5" t="inlineStr"/>
       <c r="V57" s="5" t="inlineStr"/>
+      <c r="W57" s="5" t="inlineStr"/>
+      <c r="X57" s="5" t="inlineStr"/>
+      <c r="Y57" s="5" t="inlineStr"/>
+      <c r="Z57" s="5" t="inlineStr"/>
+      <c r="AA57" s="5" t="inlineStr"/>
+      <c r="AB57" s="5" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
@@ -9743,6 +11723,12 @@
       <c r="T58" s="5" t="inlineStr"/>
       <c r="U58" s="5" t="inlineStr"/>
       <c r="V58" s="5" t="inlineStr"/>
+      <c r="W58" s="5" t="inlineStr"/>
+      <c r="X58" s="5" t="inlineStr"/>
+      <c r="Y58" s="5" t="inlineStr"/>
+      <c r="Z58" s="5" t="inlineStr"/>
+      <c r="AA58" s="5" t="inlineStr"/>
+      <c r="AB58" s="5" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
@@ -9783,6 +11769,12 @@
       <c r="T59" s="5" t="inlineStr"/>
       <c r="U59" s="5" t="inlineStr"/>
       <c r="V59" s="5" t="inlineStr"/>
+      <c r="W59" s="5" t="inlineStr"/>
+      <c r="X59" s="5" t="inlineStr"/>
+      <c r="Y59" s="5" t="inlineStr"/>
+      <c r="Z59" s="5" t="inlineStr"/>
+      <c r="AA59" s="5" t="inlineStr"/>
+      <c r="AB59" s="5" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
@@ -9819,6 +11811,12 @@
       <c r="T60" s="5" t="inlineStr"/>
       <c r="U60" s="5" t="inlineStr"/>
       <c r="V60" s="5" t="inlineStr"/>
+      <c r="W60" s="5" t="inlineStr"/>
+      <c r="X60" s="5" t="inlineStr"/>
+      <c r="Y60" s="5" t="inlineStr"/>
+      <c r="Z60" s="5" t="inlineStr"/>
+      <c r="AA60" s="5" t="inlineStr"/>
+      <c r="AB60" s="5" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
@@ -9898,6 +11896,24 @@
       </c>
       <c r="V61" s="5" t="n">
         <v>0.2066666666666667</v>
+      </c>
+      <c r="W61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="X61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y61" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z61" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="AA61" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AB61" s="5" t="n">
+        <v>0.11</v>
       </c>
     </row>
     <row r="62">
@@ -9939,6 +11955,12 @@
       <c r="T62" s="5" t="inlineStr"/>
       <c r="U62" s="5" t="inlineStr"/>
       <c r="V62" s="5" t="inlineStr"/>
+      <c r="W62" s="5" t="inlineStr"/>
+      <c r="X62" s="5" t="inlineStr"/>
+      <c r="Y62" s="5" t="inlineStr"/>
+      <c r="Z62" s="5" t="inlineStr"/>
+      <c r="AA62" s="5" t="inlineStr"/>
+      <c r="AB62" s="5" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
@@ -9979,6 +12001,12 @@
       <c r="T63" s="5" t="inlineStr"/>
       <c r="U63" s="5" t="inlineStr"/>
       <c r="V63" s="5" t="inlineStr"/>
+      <c r="W63" s="5" t="inlineStr"/>
+      <c r="X63" s="5" t="inlineStr"/>
+      <c r="Y63" s="5" t="inlineStr"/>
+      <c r="Z63" s="5" t="inlineStr"/>
+      <c r="AA63" s="5" t="inlineStr"/>
+      <c r="AB63" s="5" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
@@ -10019,6 +12047,12 @@
       <c r="T64" s="5" t="inlineStr"/>
       <c r="U64" s="5" t="inlineStr"/>
       <c r="V64" s="5" t="inlineStr"/>
+      <c r="W64" s="5" t="inlineStr"/>
+      <c r="X64" s="5" t="inlineStr"/>
+      <c r="Y64" s="5" t="inlineStr"/>
+      <c r="Z64" s="5" t="inlineStr"/>
+      <c r="AA64" s="5" t="inlineStr"/>
+      <c r="AB64" s="5" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="8" t="inlineStr">
@@ -10059,6 +12093,12 @@
       <c r="T65" s="5" t="inlineStr"/>
       <c r="U65" s="5" t="inlineStr"/>
       <c r="V65" s="5" t="inlineStr"/>
+      <c r="W65" s="5" t="inlineStr"/>
+      <c r="X65" s="5" t="inlineStr"/>
+      <c r="Y65" s="5" t="inlineStr"/>
+      <c r="Z65" s="5" t="inlineStr"/>
+      <c r="AA65" s="5" t="inlineStr"/>
+      <c r="AB65" s="5" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
@@ -10139,6 +12179,24 @@
       <c r="V66" s="5" t="n">
         <v>0.2533333333333334</v>
       </c>
+      <c r="W66" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="X66" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y66" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z66" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AA66" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AB66" s="5" t="n">
+        <v>0.06</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="8" t="inlineStr">
@@ -10218,6 +12276,24 @@
       </c>
       <c r="V67" s="5" t="n">
         <v>0.06999999999999999</v>
+      </c>
+      <c r="W67" s="5" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="X67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y67" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z67" s="5" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="AA67" s="5" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="AB67" s="5" t="n">
+        <v>0.46</v>
       </c>
     </row>
     <row r="68">
@@ -10259,6 +12335,12 @@
       <c r="T68" s="5" t="inlineStr"/>
       <c r="U68" s="5" t="inlineStr"/>
       <c r="V68" s="5" t="inlineStr"/>
+      <c r="W68" s="5" t="inlineStr"/>
+      <c r="X68" s="5" t="inlineStr"/>
+      <c r="Y68" s="5" t="inlineStr"/>
+      <c r="Z68" s="5" t="inlineStr"/>
+      <c r="AA68" s="5" t="inlineStr"/>
+      <c r="AB68" s="5" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="8" t="inlineStr">
@@ -10338,6 +12420,24 @@
       </c>
       <c r="V69" s="5" t="n">
         <v>0.2533333333333334</v>
+      </c>
+      <c r="W69" s="5" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="X69" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y69" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z69" s="5" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AA69" s="5" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="AB69" s="5" t="n">
+        <v>0.06</v>
       </c>
     </row>
     <row r="70">
@@ -10379,6 +12479,12 @@
       <c r="T70" s="5" t="inlineStr"/>
       <c r="U70" s="5" t="inlineStr"/>
       <c r="V70" s="5" t="inlineStr"/>
+      <c r="W70" s="5" t="inlineStr"/>
+      <c r="X70" s="5" t="inlineStr"/>
+      <c r="Y70" s="5" t="inlineStr"/>
+      <c r="Z70" s="5" t="inlineStr"/>
+      <c r="AA70" s="5" t="inlineStr"/>
+      <c r="AB70" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C70">
@@ -10621,6 +12727,78 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="W2:W70">
+    <cfRule type="colorScale" priority="21">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="X2:X70">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Y2:Y70">
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Z2:Z70">
+    <cfRule type="colorScale" priority="24">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AA2:AA70">
+    <cfRule type="colorScale" priority="25">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB2:AB70">
+    <cfRule type="colorScale" priority="26">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="percentile" val="50"/>
+        <cfvo type="max"/>
+        <color rgb="0063BE7B"/>
+        <color rgb="00FFEB84"/>
+        <color rgb="00F8696B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>